<commit_message>
Author Tab Tested and Two TC added for Req Tab
</commit_message>
<xml_diff>
--- a/testData/requirementTabTestData/requirementTab_testData.xlsx
+++ b/testData/requirementTabTestData/requirementTab_testData.xlsx
@@ -1,11 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29816"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29912"/>
   <workbookPr/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{BE75F180-1D9A-461B-AF11-C27102412427}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{72AAFBD2-10B3-4F05-B512-576B35A07306}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" firstSheet="50" activeTab="61" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" firstSheet="78" activeTab="80" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="tc001" sheetId="1" r:id="rId1"/>
@@ -33,43 +33,62 @@
     <sheet name="tc028" sheetId="23" r:id="rId23"/>
     <sheet name="tc029" sheetId="27" r:id="rId24"/>
     <sheet name="tc030" sheetId="19" r:id="rId25"/>
-    <sheet name="tc032" sheetId="21" r:id="rId26"/>
-    <sheet name="tc033" sheetId="22" r:id="rId27"/>
-    <sheet name="tc035" sheetId="24" r:id="rId28"/>
-    <sheet name="tc036" sheetId="30" r:id="rId29"/>
-    <sheet name="tc037" sheetId="25" r:id="rId30"/>
-    <sheet name="tc038" sheetId="31" r:id="rId31"/>
-    <sheet name="tc039" sheetId="32" r:id="rId32"/>
-    <sheet name="tc040" sheetId="33" r:id="rId33"/>
-    <sheet name="tc041" sheetId="34" r:id="rId34"/>
-    <sheet name="tc042" sheetId="35" r:id="rId35"/>
-    <sheet name="tc043" sheetId="36" r:id="rId36"/>
-    <sheet name="tc044" sheetId="39" r:id="rId37"/>
-    <sheet name="tc045" sheetId="52" r:id="rId38"/>
-    <sheet name="tc046" sheetId="38" r:id="rId39"/>
-    <sheet name="tc047" sheetId="37" r:id="rId40"/>
-    <sheet name="tc048" sheetId="40" r:id="rId41"/>
-    <sheet name="tc049" sheetId="41" r:id="rId42"/>
-    <sheet name="tc050" sheetId="42" r:id="rId43"/>
-    <sheet name="tc051" sheetId="43" r:id="rId44"/>
-    <sheet name="tc052" sheetId="44" r:id="rId45"/>
-    <sheet name="tc053" sheetId="45" r:id="rId46"/>
-    <sheet name="tc054" sheetId="46" r:id="rId47"/>
-    <sheet name="tc055" sheetId="47" r:id="rId48"/>
-    <sheet name="tc063" sheetId="53" r:id="rId49"/>
-    <sheet name="tc064" sheetId="54" r:id="rId50"/>
-    <sheet name="tc065" sheetId="48" r:id="rId51"/>
-    <sheet name="tc066" sheetId="49" r:id="rId52"/>
-    <sheet name="tc073" sheetId="50" r:id="rId53"/>
-    <sheet name="tc074" sheetId="55" r:id="rId54"/>
-    <sheet name="tc077" sheetId="51" r:id="rId55"/>
-    <sheet name="tc086" sheetId="56" r:id="rId56"/>
-    <sheet name="tc087" sheetId="57" r:id="rId57"/>
-    <sheet name="tc088" sheetId="58" r:id="rId58"/>
-    <sheet name="tc096" sheetId="60" r:id="rId59"/>
-    <sheet name="tc097" sheetId="61" r:id="rId60"/>
-    <sheet name="tc098" sheetId="62" r:id="rId61"/>
-    <sheet name="tc099" sheetId="63" r:id="rId62"/>
+    <sheet name="tc031" sheetId="73" r:id="rId26"/>
+    <sheet name="tc032" sheetId="21" r:id="rId27"/>
+    <sheet name="tc033" sheetId="22" r:id="rId28"/>
+    <sheet name="tc035" sheetId="24" r:id="rId29"/>
+    <sheet name="tc036" sheetId="30" r:id="rId30"/>
+    <sheet name="tc037" sheetId="25" r:id="rId31"/>
+    <sheet name="tc038" sheetId="31" r:id="rId32"/>
+    <sheet name="tc039" sheetId="32" r:id="rId33"/>
+    <sheet name="tc040" sheetId="33" r:id="rId34"/>
+    <sheet name="tc041" sheetId="34" r:id="rId35"/>
+    <sheet name="tc042" sheetId="35" r:id="rId36"/>
+    <sheet name="tc043" sheetId="36" r:id="rId37"/>
+    <sheet name="tc044" sheetId="39" r:id="rId38"/>
+    <sheet name="tc045" sheetId="52" r:id="rId39"/>
+    <sheet name="tc046" sheetId="38" r:id="rId40"/>
+    <sheet name="tc047" sheetId="37" r:id="rId41"/>
+    <sheet name="tc048" sheetId="40" r:id="rId42"/>
+    <sheet name="tc049" sheetId="41" r:id="rId43"/>
+    <sheet name="tc050" sheetId="42" r:id="rId44"/>
+    <sheet name="tc051" sheetId="43" r:id="rId45"/>
+    <sheet name="tc052" sheetId="44" r:id="rId46"/>
+    <sheet name="tc053" sheetId="45" r:id="rId47"/>
+    <sheet name="tc054" sheetId="46" r:id="rId48"/>
+    <sheet name="tc055" sheetId="47" r:id="rId49"/>
+    <sheet name="tc061" sheetId="74" r:id="rId50"/>
+    <sheet name="tc062" sheetId="75" r:id="rId51"/>
+    <sheet name="tc063" sheetId="53" r:id="rId52"/>
+    <sheet name="tc064" sheetId="54" r:id="rId53"/>
+    <sheet name="tc065" sheetId="48" r:id="rId54"/>
+    <sheet name="tc066" sheetId="49" r:id="rId55"/>
+    <sheet name="tc073" sheetId="50" r:id="rId56"/>
+    <sheet name="tc074" sheetId="55" r:id="rId57"/>
+    <sheet name="tc077" sheetId="51" r:id="rId58"/>
+    <sheet name="tc086" sheetId="56" r:id="rId59"/>
+    <sheet name="tc087" sheetId="57" r:id="rId60"/>
+    <sheet name="tc088" sheetId="58" r:id="rId61"/>
+    <sheet name="tc093" sheetId="64" r:id="rId62"/>
+    <sheet name="tc094" sheetId="66" r:id="rId63"/>
+    <sheet name="tc096" sheetId="60" r:id="rId64"/>
+    <sheet name="tc097" sheetId="61" r:id="rId65"/>
+    <sheet name="tc098" sheetId="62" r:id="rId66"/>
+    <sheet name="tc099" sheetId="63" r:id="rId67"/>
+    <sheet name="tc100" sheetId="67" r:id="rId68"/>
+    <sheet name="tc102" sheetId="68" r:id="rId69"/>
+    <sheet name="tc103" sheetId="69" r:id="rId70"/>
+    <sheet name="tc104" sheetId="70" r:id="rId71"/>
+    <sheet name="tc105" sheetId="76" r:id="rId72"/>
+    <sheet name="tc106" sheetId="77" r:id="rId73"/>
+    <sheet name="tc107" sheetId="78" r:id="rId74"/>
+    <sheet name="tc110" sheetId="71" r:id="rId75"/>
+    <sheet name="tc111" sheetId="72" r:id="rId76"/>
+    <sheet name="tc129" sheetId="79" r:id="rId77"/>
+    <sheet name="tc130" sheetId="80" r:id="rId78"/>
+    <sheet name="tc131" sheetId="81" r:id="rId79"/>
+    <sheet name="tc132" sheetId="82" r:id="rId80"/>
+    <sheet name="tc133" sheetId="83" r:id="rId81"/>
   </sheets>
   <calcPr calcId="191028"/>
   <extLst>
@@ -92,7 +111,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="503" uniqueCount="117">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="613" uniqueCount="129">
   <si>
     <t>Project Name</t>
   </si>
@@ -181,9 +200,6 @@
     <t>Functional</t>
   </si>
   <si>
-    <t>Projectname</t>
-  </si>
-  <si>
     <t>epic</t>
   </si>
   <si>
@@ -443,6 +459,45 @@
   </si>
   <si>
     <t>Module for testing</t>
+  </si>
+  <si>
+    <t xml:space="preserve">module name </t>
+  </si>
+  <si>
+    <t>rq title</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Epic requirement </t>
+  </si>
+  <si>
+    <t>RQ testing</t>
+  </si>
+  <si>
+    <t>Module testing</t>
+  </si>
+  <si>
+    <t>SelectEpic</t>
+  </si>
+  <si>
+    <t>SET- DRIV</t>
+  </si>
+  <si>
+    <t>mdName</t>
+  </si>
+  <si>
+    <t>SetMdName</t>
+  </si>
+  <si>
+    <t>Module20</t>
+  </si>
+  <si>
+    <t>RqNAme</t>
+  </si>
+  <si>
+    <t>Requirement_testing</t>
+  </si>
+  <si>
+    <t>jTesting</t>
   </si>
 </sst>
 </file>
@@ -940,19 +995,19 @@
   <sheetData>
     <row r="1" spans="1:5">
       <c r="A1" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="C1" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="D1" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>41</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>42</v>
       </c>
     </row>
     <row r="2" spans="1:5">
@@ -963,13 +1018,13 @@
         <v>19</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D2" s="1" t="s">
         <v>26</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
     </row>
   </sheetData>
@@ -989,14 +1044,14 @@
   <sheetData>
     <row r="1" spans="1:3">
       <c r="A1" t="s">
+        <v>37</v>
+      </c>
+      <c r="B1" t="s">
         <v>38</v>
       </c>
-      <c r="B1" t="s">
+      <c r="C1" t="s">
         <v>39</v>
       </c>
-      <c r="C1" t="s">
-        <v>40</v>
-      </c>
     </row>
     <row r="2" spans="1:3">
       <c r="A2" t="s">
@@ -1006,7 +1061,7 @@
         <v>6</v>
       </c>
       <c r="C2" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
   </sheetData>
@@ -1051,10 +1106,10 @@
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="B1" s="3" t="s">
         <v>30</v>
-      </c>
-      <c r="B1" s="3" t="s">
-        <v>31</v>
       </c>
     </row>
     <row r="2" spans="1:2">
@@ -1062,7 +1117,7 @@
         <v>19</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
   </sheetData>
@@ -1077,19 +1132,19 @@
   <sheetData>
     <row r="1" spans="1:5">
       <c r="A1" s="3" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B1" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="C1" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="C1" s="3" t="s">
-        <v>31</v>
-      </c>
       <c r="D1" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="E1" s="3" t="s">
         <v>47</v>
-      </c>
-      <c r="E1" s="3" t="s">
-        <v>48</v>
       </c>
     </row>
     <row r="2" spans="1:5">
@@ -1100,10 +1155,10 @@
         <v>19</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="E2" s="3" t="s">
         <v>11</v>
@@ -1127,7 +1182,7 @@
         <v>15</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="D1" s="6" t="s">
         <v>1</v>
@@ -1135,16 +1190,16 @@
     </row>
     <row r="2" spans="1:4">
       <c r="A2" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="B2" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="C2" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="C2" s="1" t="s">
-        <v>52</v>
-      </c>
       <c r="D2" s="6" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
   </sheetData>
@@ -1162,10 +1217,10 @@
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" t="s">
+        <v>37</v>
+      </c>
+      <c r="B1" t="s">
         <v>38</v>
-      </c>
-      <c r="B1" t="s">
-        <v>39</v>
       </c>
     </row>
     <row r="2" spans="1:2">
@@ -1183,49 +1238,43 @@
 
 <file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E3C081D6-A9C0-44C4-B61F-ECF5E1994215}">
-  <dimension ref="A1:F2"/>
+  <dimension ref="A1:E2"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="26.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6">
-      <c r="A1" t="s">
-        <v>29</v>
-      </c>
-      <c r="B1" t="s">
+    <row r="1" spans="1:5">
+      <c r="A1" t="s">
         <v>20</v>
       </c>
+      <c r="B1" t="s">
+        <v>15</v>
+      </c>
       <c r="C1" t="s">
-        <v>15</v>
+        <v>21</v>
       </c>
       <c r="D1" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="E1" t="s">
-        <v>22</v>
-      </c>
-      <c r="F1" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="2" spans="1:6">
-      <c r="A2" t="s">
-        <v>5</v>
-      </c>
-      <c r="B2" t="s">
+    <row r="2" spans="1:5">
+      <c r="A2" t="s">
         <v>24</v>
       </c>
+      <c r="B2" t="s">
+        <v>25</v>
+      </c>
       <c r="C2" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="D2" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="E2" t="s">
-        <v>27</v>
-      </c>
-      <c r="F2" t="s">
         <v>28</v>
       </c>
     </row>
@@ -1246,24 +1295,24 @@
   <sheetData>
     <row r="1" spans="1:3">
       <c r="A1" t="s">
+        <v>52</v>
+      </c>
+      <c r="B1" t="s">
         <v>53</v>
       </c>
-      <c r="B1" t="s">
+      <c r="C1" t="s">
         <v>54</v>
       </c>
-      <c r="C1" t="s">
+    </row>
+    <row r="2" spans="1:3">
+      <c r="A2" t="s">
+        <v>5</v>
+      </c>
+      <c r="B2" t="s">
         <v>55</v>
       </c>
-    </row>
-    <row r="2" spans="1:3">
-      <c r="A2" t="s">
-        <v>5</v>
-      </c>
-      <c r="B2" t="s">
+      <c r="C2" t="s">
         <v>56</v>
-      </c>
-      <c r="C2" t="s">
-        <v>57</v>
       </c>
     </row>
   </sheetData>
@@ -1281,19 +1330,19 @@
   <sheetData>
     <row r="1" spans="1:7">
       <c r="A1" t="s">
+        <v>37</v>
+      </c>
+      <c r="B1" t="s">
         <v>38</v>
       </c>
-      <c r="B1" t="s">
-        <v>39</v>
-      </c>
       <c r="C1" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="D1" t="s">
         <v>15</v>
       </c>
       <c r="E1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="F1" t="s">
         <v>22</v>
@@ -1307,10 +1356,10 @@
         <v>5</v>
       </c>
       <c r="B2" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C2" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="D2" t="s">
         <v>25</v>
@@ -1423,13 +1472,13 @@
   <sheetData>
     <row r="1" spans="1:3">
       <c r="A1" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="B1" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="B1" s="3" t="s">
-        <v>31</v>
-      </c>
       <c r="C1" s="3" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="2" spans="1:3">
@@ -1437,7 +1486,7 @@
         <v>19</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C2" s="3" t="s">
         <v>11</v>
@@ -1455,16 +1504,16 @@
   <sheetData>
     <row r="1" spans="1:6">
       <c r="A1" t="s">
+        <v>37</v>
+      </c>
+      <c r="B1" t="s">
         <v>38</v>
-      </c>
-      <c r="B1" t="s">
-        <v>39</v>
       </c>
       <c r="C1" t="s">
         <v>15</v>
       </c>
       <c r="D1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="E1" t="s">
         <v>22</v>
@@ -1478,7 +1527,7 @@
         <v>5</v>
       </c>
       <c r="B2" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C2" t="s">
         <v>25</v>
@@ -1508,22 +1557,22 @@
   <sheetData>
     <row r="1" spans="1:6">
       <c r="A1" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="B1" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="C1" s="3" t="s">
         <v>39</v>
       </c>
-      <c r="C1" s="3" t="s">
-        <v>40</v>
-      </c>
       <c r="D1" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="E1" s="3" t="s">
         <v>61</v>
       </c>
-      <c r="E1" s="3" t="s">
+      <c r="F1" s="3" t="s">
         <v>62</v>
-      </c>
-      <c r="F1" s="3" t="s">
-        <v>63</v>
       </c>
     </row>
     <row r="2" spans="1:6">
@@ -1534,16 +1583,16 @@
         <v>6</v>
       </c>
       <c r="C2" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="D2" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="E2" s="3" t="s">
         <v>64</v>
       </c>
-      <c r="D2" s="3" t="s">
-        <v>64</v>
-      </c>
-      <c r="E2" s="3" t="s">
-        <v>65</v>
-      </c>
       <c r="F2" s="3" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
   </sheetData>
@@ -1563,16 +1612,16 @@
   <sheetData>
     <row r="1" spans="1:4">
       <c r="A1" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="B1" s="4" t="s">
         <v>38</v>
-      </c>
-      <c r="B1" s="4" t="s">
-        <v>39</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>11</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
     </row>
     <row r="2" spans="1:4">
@@ -1583,10 +1632,10 @@
         <v>6</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
   </sheetData>
@@ -1601,10 +1650,10 @@
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" s="3" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="2" spans="1:2">
@@ -1612,7 +1661,7 @@
         <v>19</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
   </sheetData>
@@ -1621,6 +1670,32 @@
 </file>
 
 <file path=xl/worksheets/sheet26.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{62439209-6131-4BE4-BE2D-E6BCB6386DC8}">
+  <dimension ref="A1:B2"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" spans="1:2">
+      <c r="A1" t="s">
+        <v>52</v>
+      </c>
+      <c r="B1" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2">
+      <c r="A2" t="s">
+        <v>5</v>
+      </c>
+      <c r="B2" t="s">
+        <v>55</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet27.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E3AFD247-EFEB-43D1-A5E4-94260D9F042E}">
   <dimension ref="A1:B2"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -1642,15 +1717,15 @@
         <v>5</v>
       </c>
       <c r="B2" t="s">
-        <v>70</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet27.xml><?xml version="1.0" encoding="utf-8"?>
+        <v>69</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet28.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{49C7D945-A188-4743-BACF-F57BC8D8AB86}">
   <dimension ref="A1:B2"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -1672,15 +1747,15 @@
         <v>5</v>
       </c>
       <c r="B2" t="s">
-        <v>70</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet28.xml><?xml version="1.0" encoding="utf-8"?>
+        <v>69</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet29.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0E83F4D4-5FFA-485C-BDFA-643C5CC60A7E}">
   <dimension ref="A1:B2"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -1691,26 +1766,52 @@
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" t="s">
+        <v>52</v>
+      </c>
+      <c r="B1" t="s">
         <v>53</v>
       </c>
-      <c r="B1" t="s">
-        <v>54</v>
-      </c>
     </row>
     <row r="2" spans="1:2">
       <c r="A2" t="s">
         <v>5</v>
       </c>
       <c r="B2" t="s">
-        <v>56</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet29.xml><?xml version="1.0" encoding="utf-8"?>
+        <v>55</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6191B1E8-3F90-4D43-967E-7EE476AB5B81}">
+  <dimension ref="A1:B2"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" spans="1:2">
+      <c r="A1" t="s">
+        <v>13</v>
+      </c>
+      <c r="B1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2">
+      <c r="A2" t="s">
+        <v>14</v>
+      </c>
+      <c r="B2" t="s">
+        <v>15</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet30.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8B4C698C-6A33-4329-A05F-252C36050919}">
   <dimension ref="A1:B2"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -1739,33 +1840,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6191B1E8-3F90-4D43-967E-7EE476AB5B81}">
-  <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1" spans="1:2">
-      <c r="A1" t="s">
-        <v>13</v>
-      </c>
-      <c r="B1" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="2" spans="1:2">
-      <c r="A2" t="s">
-        <v>14</v>
-      </c>
-      <c r="B2" t="s">
-        <v>15</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet30.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet31.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B5FC98DF-CF4C-4978-974B-D4FADFCADB14}">
   <dimension ref="A1:B2"/>
   <sheetFormatPr defaultColWidth="16.85546875" defaultRowHeight="15"/>
@@ -1775,26 +1850,26 @@
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" t="s">
-        <v>53</v>
-      </c>
-      <c r="B1" t="s">
-        <v>54</v>
+        <v>52</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>18</v>
       </c>
     </row>
     <row r="2" spans="1:2">
       <c r="A2" t="s">
         <v>5</v>
       </c>
-      <c r="B2" t="s">
-        <v>56</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet31.xml><?xml version="1.0" encoding="utf-8"?>
+      <c r="B2" s="1" t="s">
+        <v>19</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet32.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A839ABB3-9810-4866-9009-03B8EC041C5D}">
   <dimension ref="A1:C2"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -1807,7 +1882,7 @@
         <v>18</v>
       </c>
       <c r="C1" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="2" spans="1:3">
@@ -1818,15 +1893,15 @@
         <v>19</v>
       </c>
       <c r="C2" t="s">
-        <v>43</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet32.xml><?xml version="1.0" encoding="utf-8"?>
+        <v>42</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet33.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E3263998-2B97-4B1C-A029-FD6DD8C1EF37}">
   <dimension ref="A1:C2"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -1839,7 +1914,7 @@
         <v>18</v>
       </c>
       <c r="C1" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="2" spans="1:3">
@@ -1850,15 +1925,15 @@
         <v>19</v>
       </c>
       <c r="C2" t="s">
-        <v>43</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet33.xml><?xml version="1.0" encoding="utf-8"?>
+        <v>42</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet34.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E29F0755-87F3-476B-9C2A-E1FFC8CED030}">
   <dimension ref="A1:C2"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -1871,7 +1946,7 @@
         <v>18</v>
       </c>
       <c r="C1" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="2" spans="1:3">
@@ -1882,15 +1957,15 @@
         <v>19</v>
       </c>
       <c r="C2" t="s">
-        <v>43</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet34.xml><?xml version="1.0" encoding="utf-8"?>
+        <v>42</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet35.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{329E8FAE-2129-4C94-87E6-C180C21CB613}">
   <dimension ref="A1:D2"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -1903,10 +1978,48 @@
         <v>18</v>
       </c>
       <c r="C1" t="s">
+        <v>70</v>
+      </c>
+      <c r="D1" t="s">
         <v>71</v>
       </c>
+    </row>
+    <row r="2" spans="1:4">
+      <c r="A2" t="s">
+        <v>5</v>
+      </c>
+      <c r="B2" t="s">
+        <v>19</v>
+      </c>
+      <c r="C2" t="s">
+        <v>42</v>
+      </c>
+      <c r="D2" t="s">
+        <v>72</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet36.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A5CE032F-302C-42A6-BC66-0FA2D092FC8A}">
+  <dimension ref="A1:D2"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" spans="1:4">
+      <c r="A1" t="s">
+        <v>17</v>
+      </c>
+      <c r="B1" t="s">
+        <v>18</v>
+      </c>
+      <c r="C1" t="s">
+        <v>70</v>
+      </c>
       <c r="D1" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
     <row r="2" spans="1:4">
@@ -1917,7 +2030,7 @@
         <v>19</v>
       </c>
       <c r="C2" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D2" t="s">
         <v>73</v>
@@ -1928,45 +2041,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet35.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A5CE032F-302C-42A6-BC66-0FA2D092FC8A}">
-  <dimension ref="A1:D2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1" spans="1:4">
-      <c r="A1" t="s">
-        <v>17</v>
-      </c>
-      <c r="B1" t="s">
-        <v>18</v>
-      </c>
-      <c r="C1" t="s">
-        <v>71</v>
-      </c>
-      <c r="D1" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4">
-      <c r="A2" t="s">
-        <v>5</v>
-      </c>
-      <c r="B2" t="s">
-        <v>19</v>
-      </c>
-      <c r="C2" t="s">
-        <v>43</v>
-      </c>
-      <c r="D2" t="s">
-        <v>74</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet36.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet37.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{74185B4F-4AE7-4DA3-9215-6ECBA7280E7B}">
   <dimension ref="A1:C2"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -1979,7 +2054,7 @@
         <v>18</v>
       </c>
       <c r="C1" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="2" spans="1:3">
@@ -1990,15 +2065,15 @@
         <v>19</v>
       </c>
       <c r="C2" t="s">
-        <v>43</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet37.xml><?xml version="1.0" encoding="utf-8"?>
+        <v>42</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet38.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7D8774BA-3EC4-46E1-BB9D-1078ACED313F}">
   <dimension ref="A1:I2"/>
   <sheetFormatPr defaultColWidth="14" defaultRowHeight="15"/>
@@ -2011,13 +2086,13 @@
         <v>18</v>
       </c>
       <c r="C1" t="s">
+        <v>70</v>
+      </c>
+      <c r="D1" t="s">
         <v>71</v>
       </c>
-      <c r="D1" t="s">
-        <v>72</v>
-      </c>
       <c r="E1" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="F1" t="s">
         <v>21</v>
@@ -2026,47 +2101,47 @@
         <v>23</v>
       </c>
       <c r="H1" t="s">
+        <v>75</v>
+      </c>
+      <c r="I1" t="s">
         <v>76</v>
       </c>
-      <c r="I1" t="s">
+    </row>
+    <row r="2" spans="1:9">
+      <c r="A2" t="s">
+        <v>5</v>
+      </c>
+      <c r="B2" t="s">
+        <v>19</v>
+      </c>
+      <c r="C2" t="s">
+        <v>42</v>
+      </c>
+      <c r="D2" t="s">
         <v>77</v>
       </c>
-    </row>
-    <row r="2" spans="1:9">
-      <c r="A2" t="s">
-        <v>5</v>
-      </c>
-      <c r="B2" t="s">
-        <v>19</v>
-      </c>
-      <c r="C2" t="s">
-        <v>43</v>
-      </c>
-      <c r="D2" t="s">
+      <c r="E2" t="s">
         <v>78</v>
       </c>
-      <c r="E2" t="s">
+      <c r="F2" t="s">
         <v>79</v>
       </c>
-      <c r="F2" t="s">
+      <c r="G2" t="s">
         <v>80</v>
       </c>
-      <c r="G2" t="s">
+      <c r="H2" t="s">
         <v>81</v>
       </c>
-      <c r="H2" t="s">
+      <c r="I2" t="s">
         <v>82</v>
       </c>
-      <c r="I2" t="s">
-        <v>83</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet38.xml><?xml version="1.0" encoding="utf-8"?>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet39.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A5C4203B-5A01-4381-A3CE-38EA6C51F801}">
   <dimension ref="A1:D2"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -2079,56 +2154,24 @@
         <v>18</v>
       </c>
       <c r="C1" t="s">
+        <v>70</v>
+      </c>
+      <c r="D1" t="s">
         <v>71</v>
       </c>
-      <c r="D1" t="s">
+    </row>
+    <row r="2" spans="1:4">
+      <c r="A2" t="s">
+        <v>5</v>
+      </c>
+      <c r="B2" t="s">
+        <v>19</v>
+      </c>
+      <c r="C2" t="s">
+        <v>42</v>
+      </c>
+      <c r="D2" t="s">
         <v>72</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4">
-      <c r="A2" t="s">
-        <v>5</v>
-      </c>
-      <c r="B2" t="s">
-        <v>19</v>
-      </c>
-      <c r="C2" t="s">
-        <v>43</v>
-      </c>
-      <c r="D2" t="s">
-        <v>73</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet39.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{35D5D97A-4287-4435-9AB2-0BB45EA4FBC3}">
-  <dimension ref="A1:C2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1" spans="1:3">
-      <c r="A1" t="s">
-        <v>17</v>
-      </c>
-      <c r="B1" t="s">
-        <v>18</v>
-      </c>
-      <c r="C1" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3">
-      <c r="A2" t="s">
-        <v>5</v>
-      </c>
-      <c r="B2" t="s">
-        <v>19</v>
-      </c>
-      <c r="C2" t="s">
-        <v>43</v>
       </c>
     </row>
   </sheetData>
@@ -2160,6 +2203,38 @@
 </file>
 
 <file path=xl/worksheets/sheet40.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{35D5D97A-4287-4435-9AB2-0BB45EA4FBC3}">
+  <dimension ref="A1:C2"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" spans="1:3">
+      <c r="A1" t="s">
+        <v>17</v>
+      </c>
+      <c r="B1" t="s">
+        <v>18</v>
+      </c>
+      <c r="C1" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3">
+      <c r="A2" t="s">
+        <v>5</v>
+      </c>
+      <c r="B2" t="s">
+        <v>19</v>
+      </c>
+      <c r="C2" t="s">
+        <v>42</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet41.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{294C6248-6B39-4869-9A5F-1A9888AB4466}">
   <dimension ref="A1:D2"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -2172,10 +2247,10 @@
         <v>18</v>
       </c>
       <c r="C1" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="D1" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
     </row>
     <row r="2" spans="1:4">
@@ -2186,18 +2261,18 @@
         <v>19</v>
       </c>
       <c r="C2" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D2" t="s">
-        <v>84</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet41.xml><?xml version="1.0" encoding="utf-8"?>
+        <v>83</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet42.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{56AA5574-913A-4A1D-9D18-82898727775C}">
   <dimension ref="A1:C2"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -2207,13 +2282,45 @@
   <sheetData>
     <row r="1" spans="1:3">
       <c r="A1" t="s">
+        <v>84</v>
+      </c>
+      <c r="B1" t="s">
         <v>85</v>
       </c>
-      <c r="B1" t="s">
+      <c r="C1" t="s">
         <v>86</v>
       </c>
+    </row>
+    <row r="2" spans="1:3">
+      <c r="A2" t="s">
+        <v>6</v>
+      </c>
+      <c r="B2" t="s">
+        <v>44</v>
+      </c>
+      <c r="C2" t="s">
+        <v>87</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet43.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D1996804-B5A0-41DE-8EAB-89A8717FC7C7}">
+  <dimension ref="A1:C2"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" spans="1:3">
+      <c r="A1" t="s">
+        <v>84</v>
+      </c>
+      <c r="B1" t="s">
+        <v>85</v>
+      </c>
       <c r="C1" t="s">
-        <v>87</v>
+        <v>23</v>
       </c>
     </row>
     <row r="2" spans="1:3">
@@ -2221,114 +2328,82 @@
         <v>6</v>
       </c>
       <c r="B2" t="s">
-        <v>45</v>
+        <v>44</v>
+      </c>
+      <c r="C2" t="s">
+        <v>80</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet44.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CEEC45CA-B3F0-4D96-A6FC-9B253BF98967}">
+  <dimension ref="A1:D2"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" spans="1:4">
+      <c r="A1" t="s">
+        <v>84</v>
+      </c>
+      <c r="B1" t="s">
+        <v>85</v>
+      </c>
+      <c r="C1" t="s">
+        <v>71</v>
+      </c>
+      <c r="D1" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4">
+      <c r="A2" t="s">
+        <v>6</v>
+      </c>
+      <c r="B2" t="s">
+        <v>44</v>
       </c>
       <c r="C2" t="s">
         <v>88</v>
       </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet42.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D1996804-B5A0-41DE-8EAB-89A8717FC7C7}">
-  <dimension ref="A1:C2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1" spans="1:3">
-      <c r="A1" t="s">
-        <v>85</v>
-      </c>
-      <c r="B1" t="s">
-        <v>86</v>
-      </c>
-      <c r="C1" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3">
-      <c r="A2" t="s">
-        <v>6</v>
-      </c>
-      <c r="B2" t="s">
-        <v>45</v>
-      </c>
-      <c r="C2" t="s">
-        <v>81</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet43.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CEEC45CA-B3F0-4D96-A6FC-9B253BF98967}">
-  <dimension ref="A1:D2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1" spans="1:4">
-      <c r="A1" t="s">
-        <v>85</v>
-      </c>
-      <c r="B1" t="s">
-        <v>86</v>
-      </c>
-      <c r="C1" t="s">
-        <v>72</v>
-      </c>
-      <c r="D1" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4">
-      <c r="A2" t="s">
-        <v>6</v>
-      </c>
-      <c r="B2" t="s">
-        <v>45</v>
-      </c>
-      <c r="C2" t="s">
-        <v>89</v>
-      </c>
       <c r="D2" t="s">
-        <v>81</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet44.xml><?xml version="1.0" encoding="utf-8"?>
+        <v>80</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet45.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9CEA2948-6B4B-43CF-AB32-61387B2A8875}">
   <dimension ref="A1:B2"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" t="s">
+        <v>84</v>
+      </c>
+      <c r="B1" t="s">
         <v>85</v>
       </c>
-      <c r="B1" t="s">
-        <v>86</v>
-      </c>
     </row>
     <row r="2" spans="1:2">
       <c r="A2" t="s">
         <v>6</v>
       </c>
       <c r="B2" t="s">
-        <v>45</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet45.xml><?xml version="1.0" encoding="utf-8"?>
+        <v>44</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet46.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{14C972A6-008E-41DF-A05C-AF5318F8FD4B}">
   <dimension ref="A1:I2"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -2341,13 +2416,13 @@
         <v>18</v>
       </c>
       <c r="C1" t="s">
+        <v>70</v>
+      </c>
+      <c r="D1" t="s">
         <v>71</v>
       </c>
-      <c r="D1" t="s">
-        <v>72</v>
-      </c>
       <c r="E1" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="F1" t="s">
         <v>21</v>
@@ -2356,13 +2431,78 @@
         <v>23</v>
       </c>
       <c r="H1" t="s">
+        <v>75</v>
+      </c>
+      <c r="I1" t="s">
         <v>76</v>
       </c>
-      <c r="I1" t="s">
+    </row>
+    <row r="2" spans="1:9">
+      <c r="A2" t="s">
+        <v>5</v>
+      </c>
+      <c r="B2" t="s">
+        <v>19</v>
+      </c>
+      <c r="C2" t="s">
+        <v>42</v>
+      </c>
+      <c r="D2" t="s">
         <v>77</v>
       </c>
-    </row>
-    <row r="2" spans="1:9">
+      <c r="E2" t="s">
+        <v>78</v>
+      </c>
+      <c r="F2" t="s">
+        <v>79</v>
+      </c>
+      <c r="G2" t="s">
+        <v>80</v>
+      </c>
+      <c r="H2" t="s">
+        <v>81</v>
+      </c>
+      <c r="I2" t="s">
+        <v>82</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet47.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8DC0861F-7791-458B-B1CF-76DF8B36CFCB}">
+  <dimension ref="A1:H2"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" spans="1:8">
+      <c r="A1" t="s">
+        <v>17</v>
+      </c>
+      <c r="B1" t="s">
+        <v>18</v>
+      </c>
+      <c r="C1" t="s">
+        <v>70</v>
+      </c>
+      <c r="D1" t="s">
+        <v>74</v>
+      </c>
+      <c r="E1" t="s">
+        <v>21</v>
+      </c>
+      <c r="F1" t="s">
+        <v>23</v>
+      </c>
+      <c r="G1" t="s">
+        <v>75</v>
+      </c>
+      <c r="H1" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8">
       <c r="A2" t="s">
         <v>5</v>
       </c>
@@ -2370,7 +2510,7 @@
         <v>19</v>
       </c>
       <c r="C2" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D2" t="s">
         <v>78</v>
@@ -2387,78 +2527,13 @@
       <c r="H2" t="s">
         <v>82</v>
       </c>
-      <c r="I2" t="s">
-        <v>83</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet46.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8DC0861F-7791-458B-B1CF-76DF8B36CFCB}">
-  <dimension ref="A1:H2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1" spans="1:8">
-      <c r="A1" t="s">
-        <v>17</v>
-      </c>
-      <c r="B1" t="s">
-        <v>18</v>
-      </c>
-      <c r="C1" t="s">
-        <v>71</v>
-      </c>
-      <c r="D1" t="s">
-        <v>75</v>
-      </c>
-      <c r="E1" t="s">
-        <v>21</v>
-      </c>
-      <c r="F1" t="s">
-        <v>23</v>
-      </c>
-      <c r="G1" t="s">
-        <v>76</v>
-      </c>
-      <c r="H1" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="2" spans="1:8">
-      <c r="A2" t="s">
-        <v>5</v>
-      </c>
-      <c r="B2" t="s">
-        <v>19</v>
-      </c>
-      <c r="C2" t="s">
-        <v>43</v>
-      </c>
-      <c r="D2" t="s">
-        <v>79</v>
-      </c>
-      <c r="E2" t="s">
-        <v>80</v>
-      </c>
-      <c r="F2" t="s">
-        <v>81</v>
-      </c>
-      <c r="G2" t="s">
-        <v>82</v>
-      </c>
-      <c r="H2" t="s">
-        <v>83</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet47.xml><?xml version="1.0" encoding="utf-8"?>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet48.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{702F240E-6DDC-40E1-A471-6D34CE8EC8A9}">
   <dimension ref="A1:C2"/>
   <sheetFormatPr defaultColWidth="14.5703125" defaultRowHeight="15"/>
@@ -2471,7 +2546,7 @@
         <v>18</v>
       </c>
       <c r="C1" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="2" spans="1:3">
@@ -2482,15 +2557,15 @@
         <v>19</v>
       </c>
       <c r="C2" t="s">
-        <v>43</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet48.xml><?xml version="1.0" encoding="utf-8"?>
+        <v>42</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet49.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1B6F8DC7-5D71-4D0F-BD39-85D8C4667F97}">
   <dimension ref="A1:D2"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -2503,74 +2578,24 @@
         <v>18</v>
       </c>
       <c r="C1" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="D1" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4">
+      <c r="A2" t="s">
+        <v>5</v>
+      </c>
+      <c r="B2" t="s">
+        <v>19</v>
+      </c>
+      <c r="C2" t="s">
+        <v>42</v>
+      </c>
+      <c r="D2" t="s">
         <v>90</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4">
-      <c r="A2" t="s">
-        <v>5</v>
-      </c>
-      <c r="B2" t="s">
-        <v>19</v>
-      </c>
-      <c r="C2" t="s">
-        <v>43</v>
-      </c>
-      <c r="D2" t="s">
-        <v>91</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet49.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7696B79F-033D-404F-9E1D-E22617A3BDAC}">
-  <dimension ref="A1:F2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1" spans="1:6">
-      <c r="A1" s="7" t="s">
-        <v>92</v>
-      </c>
-      <c r="B1" t="s">
-        <v>93</v>
-      </c>
-      <c r="C1" t="s">
-        <v>94</v>
-      </c>
-      <c r="D1" t="s">
-        <v>21</v>
-      </c>
-      <c r="E1" t="s">
-        <v>22</v>
-      </c>
-      <c r="F1" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="2" spans="1:6">
-      <c r="A2" s="7" t="s">
-        <v>95</v>
-      </c>
-      <c r="B2" t="s">
-        <v>96</v>
-      </c>
-      <c r="C2" t="s">
-        <v>97</v>
-      </c>
-      <c r="D2" t="s">
-        <v>26</v>
-      </c>
-      <c r="E2" t="s">
-        <v>27</v>
-      </c>
-      <c r="F2" t="s">
-        <v>28</v>
       </c>
     </row>
   </sheetData>
@@ -2609,19 +2634,157 @@
 </file>
 
 <file path=xl/worksheets/sheet50.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B54BFBCC-7C3F-461E-8867-D0FC9227F8D2}">
+  <dimension ref="A1:E2"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" spans="1:5">
+      <c r="A1" t="s">
+        <v>20</v>
+      </c>
+      <c r="B1" t="s">
+        <v>15</v>
+      </c>
+      <c r="C1" t="s">
+        <v>21</v>
+      </c>
+      <c r="D1" t="s">
+        <v>22</v>
+      </c>
+      <c r="E1" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5">
+      <c r="A2" t="s">
+        <v>24</v>
+      </c>
+      <c r="B2" t="s">
+        <v>25</v>
+      </c>
+      <c r="C2" t="s">
+        <v>26</v>
+      </c>
+      <c r="D2" t="s">
+        <v>27</v>
+      </c>
+      <c r="E2" t="s">
+        <v>28</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet51.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1B6C8D86-E59C-4B0D-9190-1A812D82FFD2}">
+  <dimension ref="A1:E2"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" spans="1:5">
+      <c r="A1" t="s">
+        <v>20</v>
+      </c>
+      <c r="B1" t="s">
+        <v>15</v>
+      </c>
+      <c r="C1" t="s">
+        <v>21</v>
+      </c>
+      <c r="D1" t="s">
+        <v>22</v>
+      </c>
+      <c r="E1" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5">
+      <c r="A2" t="s">
+        <v>24</v>
+      </c>
+      <c r="B2" t="s">
+        <v>25</v>
+      </c>
+      <c r="C2" t="s">
+        <v>26</v>
+      </c>
+      <c r="D2" t="s">
+        <v>27</v>
+      </c>
+      <c r="E2" t="s">
+        <v>28</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet52.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7696B79F-033D-404F-9E1D-E22617A3BDAC}">
+  <dimension ref="A1:F2"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" spans="1:6">
+      <c r="A1" s="7" t="s">
+        <v>91</v>
+      </c>
+      <c r="B1" t="s">
+        <v>92</v>
+      </c>
+      <c r="C1" t="s">
+        <v>93</v>
+      </c>
+      <c r="D1" t="s">
+        <v>21</v>
+      </c>
+      <c r="E1" t="s">
+        <v>22</v>
+      </c>
+      <c r="F1" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6">
+      <c r="A2" s="7" t="s">
+        <v>94</v>
+      </c>
+      <c r="B2" t="s">
+        <v>95</v>
+      </c>
+      <c r="C2" t="s">
+        <v>96</v>
+      </c>
+      <c r="D2" t="s">
+        <v>26</v>
+      </c>
+      <c r="E2" t="s">
+        <v>27</v>
+      </c>
+      <c r="F2" t="s">
+        <v>28</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet53.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4A192C83-0F47-4844-AB01-D5A2E984F7DB}">
   <dimension ref="A1:G2"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:7">
       <c r="A1" s="6" t="s">
+        <v>91</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>92</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="C1" s="1" t="s">
         <v>93</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>94</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>21</v>
@@ -2633,18 +2796,18 @@
         <v>23</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
     </row>
     <row r="2" spans="1:7">
       <c r="A2" s="6" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="D2" s="1" t="s">
         <v>26</v>
@@ -2656,51 +2819,51 @@
         <v>28</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>100</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet51.xml><?xml version="1.0" encoding="utf-8"?>
+        <v>99</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet54.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3011021D-4819-4690-B3D7-76A026828EC9}">
   <dimension ref="A1:G2"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:7">
       <c r="A1" s="1" t="s">
+        <v>100</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>101</v>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>93</v>
-      </c>
-      <c r="C1" s="1" t="s">
+      <c r="D1" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="E1" s="1" t="s">
         <v>102</v>
       </c>
-      <c r="D1" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="E1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>103</v>
       </c>
-      <c r="F1" s="1" t="s">
-        <v>104</v>
-      </c>
       <c r="G1" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="2" spans="1:7">
       <c r="A2" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="B2" s="1" t="s">
         <v>105</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="C2" s="1" t="s">
         <v>106</v>
-      </c>
-      <c r="C2" s="1" t="s">
-        <v>107</v>
       </c>
       <c r="D2" s="1" t="s">
         <v>26</v>
@@ -2712,57 +2875,57 @@
         <v>28</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>108</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet52.xml><?xml version="1.0" encoding="utf-8"?>
+        <v>107</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet55.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{02E7FD6A-85B6-48DD-983C-2558ACC9E840}">
   <dimension ref="A1:C2"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:3">
       <c r="A1" s="1" t="s">
+        <v>100</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>101</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>93</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>102</v>
       </c>
     </row>
     <row r="2" spans="1:3">
       <c r="A2" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="B2" s="1" t="s">
         <v>105</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="C2" s="1" t="s">
         <v>106</v>
       </c>
-      <c r="C2" s="1" t="s">
-        <v>107</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet53.xml><?xml version="1.0" encoding="utf-8"?>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet56.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{47958D0E-DE08-4FC8-AE6D-9F22489AEEFF}">
   <dimension ref="A1:F2"/>
   <sheetFormatPr defaultColWidth="18.85546875" defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:6">
       <c r="A1" t="s">
-        <v>85</v>
-      </c>
-      <c r="B1" t="s">
-        <v>109</v>
+        <v>84</v>
+      </c>
+      <c r="B1" t="s">
+        <v>108</v>
       </c>
       <c r="C1" t="s">
         <v>15</v>
@@ -2782,10 +2945,10 @@
         <v>6</v>
       </c>
       <c r="B2" t="s">
+        <v>109</v>
+      </c>
+      <c r="C2" t="s">
         <v>110</v>
-      </c>
-      <c r="C2" t="s">
-        <v>111</v>
       </c>
       <c r="D2" t="s">
         <v>26</v>
@@ -2802,27 +2965,30 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet54.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet57.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{42B9D63B-BC76-46EA-ADB4-8766AF6817A7}">
   <dimension ref="A1:A2"/>
   <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="19.28515625" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:1">
       <c r="A1" s="1" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
     </row>
     <row r="2" spans="1:1">
       <c r="A2" s="1" t="s">
-        <v>113</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet55.xml><?xml version="1.0" encoding="utf-8"?>
+        <v>112</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet58.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{006ED08C-28C3-460C-941C-159F30186152}">
   <dimension ref="A1:B2"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -2833,36 +2999,36 @@
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" t="s">
-        <v>85</v>
-      </c>
-      <c r="B1" t="s">
+        <v>84</v>
+      </c>
+      <c r="B1" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2">
+      <c r="A2" t="s">
         <v>114</v>
       </c>
-    </row>
-    <row r="2" spans="1:2">
-      <c r="A2" t="s">
+      <c r="B2" t="s">
         <v>115</v>
       </c>
-      <c r="B2" t="s">
-        <v>116</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet56.xml><?xml version="1.0" encoding="utf-8"?>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet59.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DDA25AE5-6655-45CB-9149-A8A61B5E732F}">
   <dimension ref="A1:F2"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:6">
       <c r="A1" t="s">
-        <v>85</v>
-      </c>
-      <c r="B1" t="s">
-        <v>109</v>
+        <v>84</v>
+      </c>
+      <c r="B1" t="s">
+        <v>108</v>
       </c>
       <c r="C1" t="s">
         <v>15</v>
@@ -2882,10 +3048,10 @@
         <v>6</v>
       </c>
       <c r="B2" t="s">
+        <v>109</v>
+      </c>
+      <c r="C2" t="s">
         <v>110</v>
-      </c>
-      <c r="C2" t="s">
-        <v>111</v>
       </c>
       <c r="D2" t="s">
         <v>26</v>
@@ -2894,150 +3060,6 @@
         <v>27</v>
       </c>
       <c r="F2" t="s">
-        <v>28</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet57.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C2F0C090-2891-474A-9164-D1CFD32D2A23}">
-  <dimension ref="A1:F2"/>
-  <sheetFormatPr defaultColWidth="14.7109375" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1" spans="1:6">
-      <c r="A1" t="s">
-        <v>85</v>
-      </c>
-      <c r="B1" t="s">
-        <v>109</v>
-      </c>
-      <c r="C1" t="s">
-        <v>15</v>
-      </c>
-      <c r="D1" t="s">
-        <v>21</v>
-      </c>
-      <c r="E1" t="s">
-        <v>22</v>
-      </c>
-      <c r="F1" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="2" spans="1:6">
-      <c r="A2" t="s">
-        <v>6</v>
-      </c>
-      <c r="B2" t="s">
-        <v>110</v>
-      </c>
-      <c r="C2" t="s">
-        <v>111</v>
-      </c>
-      <c r="D2" t="s">
-        <v>26</v>
-      </c>
-      <c r="E2" t="s">
-        <v>27</v>
-      </c>
-      <c r="F2" t="s">
-        <v>28</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet58.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{22B1F532-E3A9-4507-B737-44BD308773F5}">
-  <dimension ref="A1:F2"/>
-  <sheetFormatPr defaultColWidth="13.85546875" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1" spans="1:6">
-      <c r="A1" t="s">
-        <v>85</v>
-      </c>
-      <c r="B1" t="s">
-        <v>109</v>
-      </c>
-      <c r="C1" t="s">
-        <v>15</v>
-      </c>
-      <c r="D1" t="s">
-        <v>21</v>
-      </c>
-      <c r="E1" t="s">
-        <v>22</v>
-      </c>
-      <c r="F1" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="2" spans="1:6">
-      <c r="A2" t="s">
-        <v>6</v>
-      </c>
-      <c r="B2" t="s">
-        <v>110</v>
-      </c>
-      <c r="C2" t="s">
-        <v>111</v>
-      </c>
-      <c r="D2" t="s">
-        <v>26</v>
-      </c>
-      <c r="E2" t="s">
-        <v>27</v>
-      </c>
-      <c r="F2" t="s">
-        <v>28</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet59.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4F180104-CB7F-4225-88B2-B743F65A2E71}">
-  <dimension ref="A1:E2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1" spans="1:5">
-      <c r="A1" t="s">
-        <v>20</v>
-      </c>
-      <c r="B1" t="s">
-        <v>15</v>
-      </c>
-      <c r="C1" t="s">
-        <v>21</v>
-      </c>
-      <c r="D1" t="s">
-        <v>22</v>
-      </c>
-      <c r="E1" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5">
-      <c r="A2" t="s">
-        <v>24</v>
-      </c>
-      <c r="B2" t="s">
-        <v>25</v>
-      </c>
-      <c r="C2" t="s">
-        <v>26</v>
-      </c>
-      <c r="D2" t="s">
-        <v>27</v>
-      </c>
-      <c r="E2" t="s">
         <v>28</v>
       </c>
     </row>
@@ -3097,42 +3119,232 @@
 </file>
 
 <file path=xl/worksheets/sheet60.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C2F0C090-2891-474A-9164-D1CFD32D2A23}">
+  <dimension ref="A1:F2"/>
+  <sheetFormatPr defaultColWidth="14.7109375" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" spans="1:6">
+      <c r="A1" t="s">
+        <v>84</v>
+      </c>
+      <c r="B1" t="s">
+        <v>108</v>
+      </c>
+      <c r="C1" t="s">
+        <v>15</v>
+      </c>
+      <c r="D1" t="s">
+        <v>21</v>
+      </c>
+      <c r="E1" t="s">
+        <v>22</v>
+      </c>
+      <c r="F1" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6">
+      <c r="A2" t="s">
+        <v>6</v>
+      </c>
+      <c r="B2" t="s">
+        <v>109</v>
+      </c>
+      <c r="C2" t="s">
+        <v>110</v>
+      </c>
+      <c r="D2" t="s">
+        <v>26</v>
+      </c>
+      <c r="E2" t="s">
+        <v>27</v>
+      </c>
+      <c r="F2" t="s">
+        <v>28</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet61.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{22B1F532-E3A9-4507-B737-44BD308773F5}">
+  <dimension ref="A1:F2"/>
+  <sheetFormatPr defaultColWidth="13.85546875" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" spans="1:6">
+      <c r="A1" t="s">
+        <v>84</v>
+      </c>
+      <c r="B1" t="s">
+        <v>108</v>
+      </c>
+      <c r="C1" t="s">
+        <v>15</v>
+      </c>
+      <c r="D1" t="s">
+        <v>21</v>
+      </c>
+      <c r="E1" t="s">
+        <v>22</v>
+      </c>
+      <c r="F1" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6">
+      <c r="A2" t="s">
+        <v>6</v>
+      </c>
+      <c r="B2" t="s">
+        <v>109</v>
+      </c>
+      <c r="C2" t="s">
+        <v>110</v>
+      </c>
+      <c r="D2" t="s">
+        <v>26</v>
+      </c>
+      <c r="E2" t="s">
+        <v>27</v>
+      </c>
+      <c r="F2" t="s">
+        <v>28</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet62.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{545270BF-46D2-413A-9419-76683720126A}">
+  <dimension ref="A1:B2"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" spans="1:2">
+      <c r="A1" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2">
+      <c r="A2" s="1" t="s">
+        <v>118</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>119</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet63.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7A8A7719-5FC7-406C-A809-EBB81C7D304F}">
+  <dimension ref="A1:A2"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" spans="1:1">
+      <c r="A1" s="1" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1">
+      <c r="A2" s="1" t="s">
+        <v>120</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet64.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4F180104-CB7F-4225-88B2-B743F65A2E71}">
+  <dimension ref="A1:E2"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" spans="1:5">
+      <c r="A1" t="s">
+        <v>20</v>
+      </c>
+      <c r="B1" t="s">
+        <v>15</v>
+      </c>
+      <c r="C1" t="s">
+        <v>21</v>
+      </c>
+      <c r="D1" t="s">
+        <v>22</v>
+      </c>
+      <c r="E1" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5">
+      <c r="A2" t="s">
+        <v>24</v>
+      </c>
+      <c r="B2" t="s">
+        <v>25</v>
+      </c>
+      <c r="C2" t="s">
+        <v>26</v>
+      </c>
+      <c r="D2" t="s">
+        <v>27</v>
+      </c>
+      <c r="E2" t="s">
+        <v>28</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet65.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F12CCDE5-920D-49D0-950B-159A5A491EE7}">
   <dimension ref="A1:G2"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:7">
       <c r="A1" s="1" t="s">
+        <v>100</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>101</v>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>93</v>
-      </c>
-      <c r="C1" s="1" t="s">
+      <c r="D1" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="E1" s="1" t="s">
         <v>102</v>
       </c>
-      <c r="D1" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="E1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>103</v>
       </c>
-      <c r="F1" s="1" t="s">
-        <v>104</v>
-      </c>
       <c r="G1" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="2" spans="1:7">
       <c r="A2" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="B2" s="1" t="s">
         <v>105</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="C2" s="1" t="s">
         <v>106</v>
-      </c>
-      <c r="C2" s="1" t="s">
-        <v>107</v>
       </c>
       <c r="D2" s="1" t="s">
         <v>26</v>
@@ -3144,20 +3356,20 @@
         <v>28</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>108</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet61.xml><?xml version="1.0" encoding="utf-8"?>
+        <v>107</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet66.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{57C2C09D-3106-4A2C-A972-09AF8ED3E7CC}">
   <dimension ref="A1:B2"/>
   <sheetFormatPr defaultColWidth="13.85546875" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="16384" width="13.85546875" customWidth="1"/>
+    <col min="1" max="1" width="13.85546875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2">
@@ -3181,7 +3393,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet62.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet67.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{28C5798F-1A42-4810-A643-274C39BB5B89}">
   <dimension ref="A1:D2"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -3194,7 +3406,7 @@
         <v>15</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="D1" s="6" t="s">
         <v>1</v>
@@ -3202,16 +3414,78 @@
     </row>
     <row r="2" spans="1:4">
       <c r="A2" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="B2" s="1" t="s">
         <v>50</v>
       </c>
+      <c r="C2" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="D2" s="6" t="s">
+        <v>49</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet68.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DD547580-CDD4-4CA1-99D1-F4DBEB4DC61C}">
+  <dimension ref="A1:B2"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="16" customWidth="1"/>
+    <col min="2" max="2" width="14.5703125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2">
+      <c r="A1" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="B1" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2">
+      <c r="A2" s="1" t="s">
+        <v>112</v>
+      </c>
+      <c r="B2" t="s">
+        <v>122</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet69.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5C851C18-BB40-4C4C-9358-B9D27BF745A2}">
+  <dimension ref="A1:C2"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" spans="1:3">
+      <c r="A1" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>124</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3">
+      <c r="A2" s="1" t="s">
+        <v>122</v>
+      </c>
       <c r="B2" s="1" t="s">
-        <v>51</v>
+        <v>125</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>52</v>
-      </c>
-      <c r="D2" s="6" t="s">
-        <v>50</v>
+        <v>101</v>
       </c>
     </row>
   </sheetData>
@@ -3221,18 +3495,220 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{29DDC4E0-08CB-46D1-AE6D-9F161D97ECBA}">
-  <dimension ref="A1:F2"/>
+  <dimension ref="A1:E2"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="39.5703125" customWidth="1"/>
   </cols>
   <sheetData>
+    <row r="1" spans="1:5">
+      <c r="A1" t="s">
+        <v>20</v>
+      </c>
+      <c r="B1" t="s">
+        <v>15</v>
+      </c>
+      <c r="C1" t="s">
+        <v>21</v>
+      </c>
+      <c r="D1" t="s">
+        <v>22</v>
+      </c>
+      <c r="E1" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5">
+      <c r="A2" t="s">
+        <v>24</v>
+      </c>
+      <c r="B2" t="s">
+        <v>25</v>
+      </c>
+      <c r="C2" t="s">
+        <v>26</v>
+      </c>
+      <c r="D2" t="s">
+        <v>27</v>
+      </c>
+      <c r="E2" t="s">
+        <v>28</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet70.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{30CA7E00-9554-459F-BF47-6B8E0B27B5B9}">
+  <dimension ref="A1:C2"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" spans="1:3">
+      <c r="A1" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>124</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3">
+      <c r="A2" s="1" t="s">
+        <v>122</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>125</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>101</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet71.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{93B51C47-FA71-48A7-A2FD-49CB882674F9}">
+  <dimension ref="A1:C2"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" spans="1:3">
+      <c r="A1" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>124</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3">
+      <c r="A2" s="1" t="s">
+        <v>122</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>125</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>101</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet72.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{485C4B2E-FC36-4946-BA8B-78C7FADE4211}">
+  <dimension ref="A1:G2"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" spans="1:7">
+      <c r="A1" s="1" t="s">
+        <v>100</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>101</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>102</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>103</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7">
+      <c r="A2" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>105</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="F2" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="G2" s="1" t="s">
+        <v>107</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet73.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EBC66432-A9A4-4E48-A474-1F35C5F1C633}">
+  <dimension ref="A1:D2"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" spans="1:4">
+      <c r="A1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="D1" s="6" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4">
+      <c r="A2" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="D2" s="6" t="s">
+        <v>49</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet74.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{849D9C7E-7FB2-4797-90F9-A5CEADA89D9C}">
+  <dimension ref="A1:F2"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
     <row r="1" spans="1:6">
       <c r="A1" t="s">
-        <v>29</v>
-      </c>
-      <c r="B1" t="s">
-        <v>20</v>
+        <v>84</v>
+      </c>
+      <c r="B1" t="s">
+        <v>108</v>
       </c>
       <c r="C1" t="s">
         <v>15</v>
@@ -3249,13 +3725,13 @@
     </row>
     <row r="2" spans="1:6">
       <c r="A2" t="s">
-        <v>5</v>
-      </c>
-      <c r="B2" t="s">
-        <v>24</v>
+        <v>6</v>
+      </c>
+      <c r="B2" t="s">
+        <v>109</v>
       </c>
       <c r="C2" t="s">
-        <v>25</v>
+        <v>110</v>
       </c>
       <c r="D2" t="s">
         <v>26</v>
@@ -3265,6 +3741,136 @@
       </c>
       <c r="F2" t="s">
         <v>28</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet75.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C4A8AAC5-4185-4C1C-93D4-1D0A64F4E1B7}">
+  <dimension ref="A1:B2"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" spans="1:2">
+      <c r="A1" s="1" t="s">
+        <v>84</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2">
+      <c r="A2" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>127</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet76.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9539B7F2-18EC-49F7-91A3-B0ABA5965519}">
+  <dimension ref="A1:B2"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" spans="1:2">
+      <c r="A1" s="1" t="s">
+        <v>84</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2">
+      <c r="A2" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>127</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet77.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{223C53EB-97BE-4EFF-B890-3A3BD91E9E72}">
+  <dimension ref="A1:B2"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" spans="1:2">
+      <c r="A1" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2">
+      <c r="A2" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>128</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet78.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7E2B8556-771D-4DAD-8C21-33E755A02656}">
+  <dimension ref="A1:B2"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" spans="1:2">
+      <c r="A1" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2">
+      <c r="A2" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>128</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet79.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A7FA2BA4-A228-45F5-B096-B0B6F3C5FCD9}">
+  <dimension ref="A1:B2"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" spans="1:2">
+      <c r="A1" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2">
+      <c r="A2" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>128</v>
       </c>
     </row>
   </sheetData>
@@ -3282,13 +3888,13 @@
   <sheetData>
     <row r="1" spans="1:4">
       <c r="A1" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="B1" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="C1" s="3" t="s">
         <v>31</v>
-      </c>
-      <c r="C1" s="3" t="s">
-        <v>32</v>
       </c>
       <c r="D1" s="3" t="s">
         <v>13</v>
@@ -3299,13 +3905,65 @@
         <v>19</v>
       </c>
       <c r="B2" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="C2" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="C2" s="3" t="s">
+      <c r="D2" s="3" t="s">
+        <v>33</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet80.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{763B8C95-495E-4740-BDD6-D904F75864FB}">
+  <dimension ref="A1:B2"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" spans="1:2">
+      <c r="A1" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="D2" s="3" t="s">
+      <c r="B1" s="1" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2">
+      <c r="A2" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>128</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet81.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0D8151D4-D1A1-47AD-8B8F-43868BB4348D}">
+  <dimension ref="A1:B2"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" spans="1:2">
+      <c r="A1" s="1" t="s">
         <v>34</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2">
+      <c r="A2" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>128</v>
       </c>
     </row>
   </sheetData>
@@ -3320,16 +3978,16 @@
   <sheetData>
     <row r="1" spans="1:4">
       <c r="A1" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="D1" s="3" t="s">
         <v>35</v>
-      </c>
-      <c r="B1" s="3" t="s">
-        <v>30</v>
-      </c>
-      <c r="C1" s="3" t="s">
-        <v>31</v>
-      </c>
-      <c r="D1" s="3" t="s">
-        <v>36</v>
       </c>
     </row>
     <row r="2" spans="1:4">
@@ -3340,10 +3998,10 @@
         <v>19</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Added new tc-126 to tc-128
</commit_message>
<xml_diff>
--- a/testData/requirementTabTestData/requirementTab_testData.xlsx
+++ b/testData/requirementTabTestData/requirementTab_testData.xlsx
@@ -1,11 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29816"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29912"/>
   <workbookPr/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{BE75F180-1D9A-461B-AF11-C27102412427}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{207880DB-32DE-4A25-BF9B-492FE793168F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" firstSheet="50" activeTab="61" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" firstSheet="77" activeTab="77" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="tc001" sheetId="1" r:id="rId1"/>
@@ -33,43 +33,65 @@
     <sheet name="tc028" sheetId="23" r:id="rId23"/>
     <sheet name="tc029" sheetId="27" r:id="rId24"/>
     <sheet name="tc030" sheetId="19" r:id="rId25"/>
-    <sheet name="tc032" sheetId="21" r:id="rId26"/>
-    <sheet name="tc033" sheetId="22" r:id="rId27"/>
-    <sheet name="tc035" sheetId="24" r:id="rId28"/>
-    <sheet name="tc036" sheetId="30" r:id="rId29"/>
-    <sheet name="tc037" sheetId="25" r:id="rId30"/>
-    <sheet name="tc038" sheetId="31" r:id="rId31"/>
-    <sheet name="tc039" sheetId="32" r:id="rId32"/>
-    <sheet name="tc040" sheetId="33" r:id="rId33"/>
-    <sheet name="tc041" sheetId="34" r:id="rId34"/>
-    <sheet name="tc042" sheetId="35" r:id="rId35"/>
-    <sheet name="tc043" sheetId="36" r:id="rId36"/>
-    <sheet name="tc044" sheetId="39" r:id="rId37"/>
-    <sheet name="tc045" sheetId="52" r:id="rId38"/>
-    <sheet name="tc046" sheetId="38" r:id="rId39"/>
-    <sheet name="tc047" sheetId="37" r:id="rId40"/>
-    <sheet name="tc048" sheetId="40" r:id="rId41"/>
-    <sheet name="tc049" sheetId="41" r:id="rId42"/>
-    <sheet name="tc050" sheetId="42" r:id="rId43"/>
-    <sheet name="tc051" sheetId="43" r:id="rId44"/>
-    <sheet name="tc052" sheetId="44" r:id="rId45"/>
-    <sheet name="tc053" sheetId="45" r:id="rId46"/>
-    <sheet name="tc054" sheetId="46" r:id="rId47"/>
-    <sheet name="tc055" sheetId="47" r:id="rId48"/>
-    <sheet name="tc063" sheetId="53" r:id="rId49"/>
-    <sheet name="tc064" sheetId="54" r:id="rId50"/>
-    <sheet name="tc065" sheetId="48" r:id="rId51"/>
-    <sheet name="tc066" sheetId="49" r:id="rId52"/>
-    <sheet name="tc073" sheetId="50" r:id="rId53"/>
-    <sheet name="tc074" sheetId="55" r:id="rId54"/>
-    <sheet name="tc077" sheetId="51" r:id="rId55"/>
-    <sheet name="tc086" sheetId="56" r:id="rId56"/>
-    <sheet name="tc087" sheetId="57" r:id="rId57"/>
-    <sheet name="tc088" sheetId="58" r:id="rId58"/>
-    <sheet name="tc096" sheetId="60" r:id="rId59"/>
-    <sheet name="tc097" sheetId="61" r:id="rId60"/>
-    <sheet name="tc098" sheetId="62" r:id="rId61"/>
-    <sheet name="tc099" sheetId="63" r:id="rId62"/>
+    <sheet name="tc031" sheetId="73" r:id="rId26"/>
+    <sheet name="tc032" sheetId="21" r:id="rId27"/>
+    <sheet name="tc033" sheetId="22" r:id="rId28"/>
+    <sheet name="tc035" sheetId="24" r:id="rId29"/>
+    <sheet name="tc036" sheetId="30" r:id="rId30"/>
+    <sheet name="tc037" sheetId="25" r:id="rId31"/>
+    <sheet name="tc038" sheetId="31" r:id="rId32"/>
+    <sheet name="tc039" sheetId="32" r:id="rId33"/>
+    <sheet name="tc040" sheetId="33" r:id="rId34"/>
+    <sheet name="tc041" sheetId="34" r:id="rId35"/>
+    <sheet name="tc042" sheetId="35" r:id="rId36"/>
+    <sheet name="tc043" sheetId="36" r:id="rId37"/>
+    <sheet name="tc044" sheetId="39" r:id="rId38"/>
+    <sheet name="tc045" sheetId="52" r:id="rId39"/>
+    <sheet name="tc046" sheetId="38" r:id="rId40"/>
+    <sheet name="tc047" sheetId="37" r:id="rId41"/>
+    <sheet name="tc048" sheetId="40" r:id="rId42"/>
+    <sheet name="tc049" sheetId="41" r:id="rId43"/>
+    <sheet name="tc050" sheetId="42" r:id="rId44"/>
+    <sheet name="tc051" sheetId="43" r:id="rId45"/>
+    <sheet name="tc052" sheetId="44" r:id="rId46"/>
+    <sheet name="tc053" sheetId="45" r:id="rId47"/>
+    <sheet name="tc054" sheetId="46" r:id="rId48"/>
+    <sheet name="tc055" sheetId="47" r:id="rId49"/>
+    <sheet name="tc061" sheetId="74" r:id="rId50"/>
+    <sheet name="tc062" sheetId="75" r:id="rId51"/>
+    <sheet name="tc063" sheetId="53" r:id="rId52"/>
+    <sheet name="tc064" sheetId="54" r:id="rId53"/>
+    <sheet name="tc065" sheetId="48" r:id="rId54"/>
+    <sheet name="tc066" sheetId="49" r:id="rId55"/>
+    <sheet name="tc073" sheetId="50" r:id="rId56"/>
+    <sheet name="tc074" sheetId="55" r:id="rId57"/>
+    <sheet name="tc077" sheetId="51" r:id="rId58"/>
+    <sheet name="tc086" sheetId="56" r:id="rId59"/>
+    <sheet name="tc087" sheetId="57" r:id="rId60"/>
+    <sheet name="tc088" sheetId="58" r:id="rId61"/>
+    <sheet name="tc093" sheetId="64" r:id="rId62"/>
+    <sheet name="tc094" sheetId="66" r:id="rId63"/>
+    <sheet name="tc096" sheetId="60" r:id="rId64"/>
+    <sheet name="tc097" sheetId="61" r:id="rId65"/>
+    <sheet name="tc098" sheetId="62" r:id="rId66"/>
+    <sheet name="tc099" sheetId="63" r:id="rId67"/>
+    <sheet name="tc100" sheetId="67" r:id="rId68"/>
+    <sheet name="tc102" sheetId="68" r:id="rId69"/>
+    <sheet name="tc103" sheetId="69" r:id="rId70"/>
+    <sheet name="tc104" sheetId="70" r:id="rId71"/>
+    <sheet name="tc105" sheetId="76" r:id="rId72"/>
+    <sheet name="tc106" sheetId="77" r:id="rId73"/>
+    <sheet name="tc107" sheetId="78" r:id="rId74"/>
+    <sheet name="tc110" sheetId="71" r:id="rId75"/>
+    <sheet name="tc111" sheetId="72" r:id="rId76"/>
+    <sheet name="tc117" sheetId="85" r:id="rId77"/>
+    <sheet name="tc118" sheetId="86" r:id="rId78"/>
+    <sheet name="tc119" sheetId="84" r:id="rId79"/>
+    <sheet name="tc129" sheetId="79" r:id="rId80"/>
+    <sheet name="tc130" sheetId="80" r:id="rId81"/>
+    <sheet name="tc131" sheetId="81" r:id="rId82"/>
+    <sheet name="tc132" sheetId="82" r:id="rId83"/>
+    <sheet name="tc133" sheetId="83" r:id="rId84"/>
   </sheets>
   <calcPr calcId="191028"/>
   <extLst>
@@ -92,7 +114,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="503" uniqueCount="117">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="629" uniqueCount="131">
   <si>
     <t>Project Name</t>
   </si>
@@ -181,9 +203,6 @@
     <t>Functional</t>
   </si>
   <si>
-    <t>Projectname</t>
-  </si>
-  <si>
     <t>epic</t>
   </si>
   <si>
@@ -443,6 +462,51 @@
   </si>
   <si>
     <t>Module for testing</t>
+  </si>
+  <si>
+    <t xml:space="preserve">module name </t>
+  </si>
+  <si>
+    <t>rq title</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Epic requirement </t>
+  </si>
+  <si>
+    <t>RQ testing</t>
+  </si>
+  <si>
+    <t>Module testing</t>
+  </si>
+  <si>
+    <t>SelectEpic</t>
+  </si>
+  <si>
+    <t>SET- DRIV</t>
+  </si>
+  <si>
+    <t>mdName</t>
+  </si>
+  <si>
+    <t>SetMdName</t>
+  </si>
+  <si>
+    <t>Module20</t>
+  </si>
+  <si>
+    <t>RqNAme</t>
+  </si>
+  <si>
+    <t>Requirement_testing</t>
+  </si>
+  <si>
+    <t>req</t>
+  </si>
+  <si>
+    <t>jTesting</t>
+  </si>
+  <si>
+    <t>RQ-2167</t>
   </si>
 </sst>
 </file>
@@ -940,19 +1004,19 @@
   <sheetData>
     <row r="1" spans="1:5">
       <c r="A1" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="C1" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="D1" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>41</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>42</v>
       </c>
     </row>
     <row r="2" spans="1:5">
@@ -963,13 +1027,13 @@
         <v>19</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D2" s="1" t="s">
         <v>26</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
     </row>
   </sheetData>
@@ -989,14 +1053,14 @@
   <sheetData>
     <row r="1" spans="1:3">
       <c r="A1" t="s">
+        <v>37</v>
+      </c>
+      <c r="B1" t="s">
         <v>38</v>
       </c>
-      <c r="B1" t="s">
+      <c r="C1" t="s">
         <v>39</v>
       </c>
-      <c r="C1" t="s">
-        <v>40</v>
-      </c>
     </row>
     <row r="2" spans="1:3">
       <c r="A2" t="s">
@@ -1006,7 +1070,7 @@
         <v>6</v>
       </c>
       <c r="C2" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
   </sheetData>
@@ -1051,10 +1115,10 @@
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="B1" s="3" t="s">
         <v>30</v>
-      </c>
-      <c r="B1" s="3" t="s">
-        <v>31</v>
       </c>
     </row>
     <row r="2" spans="1:2">
@@ -1062,7 +1126,7 @@
         <v>19</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
   </sheetData>
@@ -1077,19 +1141,19 @@
   <sheetData>
     <row r="1" spans="1:5">
       <c r="A1" s="3" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B1" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="C1" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="C1" s="3" t="s">
-        <v>31</v>
-      </c>
       <c r="D1" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="E1" s="3" t="s">
         <v>47</v>
-      </c>
-      <c r="E1" s="3" t="s">
-        <v>48</v>
       </c>
     </row>
     <row r="2" spans="1:5">
@@ -1100,10 +1164,10 @@
         <v>19</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="E2" s="3" t="s">
         <v>11</v>
@@ -1127,7 +1191,7 @@
         <v>15</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="D1" s="6" t="s">
         <v>1</v>
@@ -1135,16 +1199,16 @@
     </row>
     <row r="2" spans="1:4">
       <c r="A2" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="B2" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="C2" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="C2" s="1" t="s">
-        <v>52</v>
-      </c>
       <c r="D2" s="6" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
   </sheetData>
@@ -1162,10 +1226,10 @@
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" t="s">
+        <v>37</v>
+      </c>
+      <c r="B1" t="s">
         <v>38</v>
-      </c>
-      <c r="B1" t="s">
-        <v>39</v>
       </c>
     </row>
     <row r="2" spans="1:2">
@@ -1183,49 +1247,43 @@
 
 <file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E3C081D6-A9C0-44C4-B61F-ECF5E1994215}">
-  <dimension ref="A1:F2"/>
+  <dimension ref="A1:E2"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="26.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6">
-      <c r="A1" t="s">
-        <v>29</v>
-      </c>
-      <c r="B1" t="s">
+    <row r="1" spans="1:5">
+      <c r="A1" t="s">
         <v>20</v>
       </c>
+      <c r="B1" t="s">
+        <v>15</v>
+      </c>
       <c r="C1" t="s">
-        <v>15</v>
+        <v>21</v>
       </c>
       <c r="D1" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="E1" t="s">
-        <v>22</v>
-      </c>
-      <c r="F1" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="2" spans="1:6">
-      <c r="A2" t="s">
-        <v>5</v>
-      </c>
-      <c r="B2" t="s">
+    <row r="2" spans="1:5">
+      <c r="A2" t="s">
         <v>24</v>
       </c>
+      <c r="B2" t="s">
+        <v>25</v>
+      </c>
       <c r="C2" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="D2" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="E2" t="s">
-        <v>27</v>
-      </c>
-      <c r="F2" t="s">
         <v>28</v>
       </c>
     </row>
@@ -1246,24 +1304,24 @@
   <sheetData>
     <row r="1" spans="1:3">
       <c r="A1" t="s">
+        <v>52</v>
+      </c>
+      <c r="B1" t="s">
         <v>53</v>
       </c>
-      <c r="B1" t="s">
+      <c r="C1" t="s">
         <v>54</v>
       </c>
-      <c r="C1" t="s">
+    </row>
+    <row r="2" spans="1:3">
+      <c r="A2" t="s">
+        <v>5</v>
+      </c>
+      <c r="B2" t="s">
         <v>55</v>
       </c>
-    </row>
-    <row r="2" spans="1:3">
-      <c r="A2" t="s">
-        <v>5</v>
-      </c>
-      <c r="B2" t="s">
+      <c r="C2" t="s">
         <v>56</v>
-      </c>
-      <c r="C2" t="s">
-        <v>57</v>
       </c>
     </row>
   </sheetData>
@@ -1281,19 +1339,19 @@
   <sheetData>
     <row r="1" spans="1:7">
       <c r="A1" t="s">
+        <v>37</v>
+      </c>
+      <c r="B1" t="s">
         <v>38</v>
       </c>
-      <c r="B1" t="s">
-        <v>39</v>
-      </c>
       <c r="C1" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="D1" t="s">
         <v>15</v>
       </c>
       <c r="E1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="F1" t="s">
         <v>22</v>
@@ -1307,10 +1365,10 @@
         <v>5</v>
       </c>
       <c r="B2" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C2" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="D2" t="s">
         <v>25</v>
@@ -1423,13 +1481,13 @@
   <sheetData>
     <row r="1" spans="1:3">
       <c r="A1" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="B1" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="B1" s="3" t="s">
-        <v>31</v>
-      </c>
       <c r="C1" s="3" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="2" spans="1:3">
@@ -1437,7 +1495,7 @@
         <v>19</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C2" s="3" t="s">
         <v>11</v>
@@ -1455,16 +1513,16 @@
   <sheetData>
     <row r="1" spans="1:6">
       <c r="A1" t="s">
+        <v>37</v>
+      </c>
+      <c r="B1" t="s">
         <v>38</v>
-      </c>
-      <c r="B1" t="s">
-        <v>39</v>
       </c>
       <c r="C1" t="s">
         <v>15</v>
       </c>
       <c r="D1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="E1" t="s">
         <v>22</v>
@@ -1478,7 +1536,7 @@
         <v>5</v>
       </c>
       <c r="B2" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C2" t="s">
         <v>25</v>
@@ -1508,22 +1566,22 @@
   <sheetData>
     <row r="1" spans="1:6">
       <c r="A1" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="B1" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="C1" s="3" t="s">
         <v>39</v>
       </c>
-      <c r="C1" s="3" t="s">
-        <v>40</v>
-      </c>
       <c r="D1" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="E1" s="3" t="s">
         <v>61</v>
       </c>
-      <c r="E1" s="3" t="s">
+      <c r="F1" s="3" t="s">
         <v>62</v>
-      </c>
-      <c r="F1" s="3" t="s">
-        <v>63</v>
       </c>
     </row>
     <row r="2" spans="1:6">
@@ -1534,16 +1592,16 @@
         <v>6</v>
       </c>
       <c r="C2" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="D2" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="E2" s="3" t="s">
         <v>64</v>
       </c>
-      <c r="D2" s="3" t="s">
-        <v>64</v>
-      </c>
-      <c r="E2" s="3" t="s">
-        <v>65</v>
-      </c>
       <c r="F2" s="3" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
   </sheetData>
@@ -1563,16 +1621,16 @@
   <sheetData>
     <row r="1" spans="1:4">
       <c r="A1" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="B1" s="4" t="s">
         <v>38</v>
-      </c>
-      <c r="B1" s="4" t="s">
-        <v>39</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>11</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
     </row>
     <row r="2" spans="1:4">
@@ -1583,10 +1641,10 @@
         <v>6</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
   </sheetData>
@@ -1601,10 +1659,10 @@
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" s="3" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="2" spans="1:2">
@@ -1612,7 +1670,7 @@
         <v>19</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
   </sheetData>
@@ -1621,6 +1679,32 @@
 </file>
 
 <file path=xl/worksheets/sheet26.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{62439209-6131-4BE4-BE2D-E6BCB6386DC8}">
+  <dimension ref="A1:B2"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" spans="1:2">
+      <c r="A1" t="s">
+        <v>52</v>
+      </c>
+      <c r="B1" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2">
+      <c r="A2" t="s">
+        <v>5</v>
+      </c>
+      <c r="B2" t="s">
+        <v>55</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet27.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E3AFD247-EFEB-43D1-A5E4-94260D9F042E}">
   <dimension ref="A1:B2"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -1642,15 +1726,15 @@
         <v>5</v>
       </c>
       <c r="B2" t="s">
-        <v>70</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet27.xml><?xml version="1.0" encoding="utf-8"?>
+        <v>69</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet28.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{49C7D945-A188-4743-BACF-F57BC8D8AB86}">
   <dimension ref="A1:B2"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -1672,15 +1756,15 @@
         <v>5</v>
       </c>
       <c r="B2" t="s">
-        <v>70</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet28.xml><?xml version="1.0" encoding="utf-8"?>
+        <v>69</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet29.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0E83F4D4-5FFA-485C-BDFA-643C5CC60A7E}">
   <dimension ref="A1:B2"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -1691,26 +1775,52 @@
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" t="s">
+        <v>52</v>
+      </c>
+      <c r="B1" t="s">
         <v>53</v>
       </c>
-      <c r="B1" t="s">
-        <v>54</v>
-      </c>
     </row>
     <row r="2" spans="1:2">
       <c r="A2" t="s">
         <v>5</v>
       </c>
       <c r="B2" t="s">
-        <v>56</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet29.xml><?xml version="1.0" encoding="utf-8"?>
+        <v>55</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6191B1E8-3F90-4D43-967E-7EE476AB5B81}">
+  <dimension ref="A1:B2"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" spans="1:2">
+      <c r="A1" t="s">
+        <v>13</v>
+      </c>
+      <c r="B1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2">
+      <c r="A2" t="s">
+        <v>14</v>
+      </c>
+      <c r="B2" t="s">
+        <v>15</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet30.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8B4C698C-6A33-4329-A05F-252C36050919}">
   <dimension ref="A1:B2"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -1739,33 +1849,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6191B1E8-3F90-4D43-967E-7EE476AB5B81}">
-  <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1" spans="1:2">
-      <c r="A1" t="s">
-        <v>13</v>
-      </c>
-      <c r="B1" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="2" spans="1:2">
-      <c r="A2" t="s">
-        <v>14</v>
-      </c>
-      <c r="B2" t="s">
-        <v>15</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet30.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet31.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B5FC98DF-CF4C-4978-974B-D4FADFCADB14}">
   <dimension ref="A1:B2"/>
   <sheetFormatPr defaultColWidth="16.85546875" defaultRowHeight="15"/>
@@ -1775,26 +1859,26 @@
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" t="s">
-        <v>53</v>
-      </c>
-      <c r="B1" t="s">
-        <v>54</v>
+        <v>52</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>18</v>
       </c>
     </row>
     <row r="2" spans="1:2">
       <c r="A2" t="s">
         <v>5</v>
       </c>
-      <c r="B2" t="s">
-        <v>56</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet31.xml><?xml version="1.0" encoding="utf-8"?>
+      <c r="B2" s="1" t="s">
+        <v>19</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet32.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A839ABB3-9810-4866-9009-03B8EC041C5D}">
   <dimension ref="A1:C2"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -1807,7 +1891,7 @@
         <v>18</v>
       </c>
       <c r="C1" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="2" spans="1:3">
@@ -1818,15 +1902,15 @@
         <v>19</v>
       </c>
       <c r="C2" t="s">
-        <v>43</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet32.xml><?xml version="1.0" encoding="utf-8"?>
+        <v>42</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet33.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E3263998-2B97-4B1C-A029-FD6DD8C1EF37}">
   <dimension ref="A1:C2"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -1839,7 +1923,7 @@
         <v>18</v>
       </c>
       <c r="C1" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="2" spans="1:3">
@@ -1850,15 +1934,15 @@
         <v>19</v>
       </c>
       <c r="C2" t="s">
-        <v>43</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet33.xml><?xml version="1.0" encoding="utf-8"?>
+        <v>42</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet34.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E29F0755-87F3-476B-9C2A-E1FFC8CED030}">
   <dimension ref="A1:C2"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -1871,7 +1955,7 @@
         <v>18</v>
       </c>
       <c r="C1" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="2" spans="1:3">
@@ -1882,15 +1966,15 @@
         <v>19</v>
       </c>
       <c r="C2" t="s">
-        <v>43</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet34.xml><?xml version="1.0" encoding="utf-8"?>
+        <v>42</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet35.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{329E8FAE-2129-4C94-87E6-C180C21CB613}">
   <dimension ref="A1:D2"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -1903,10 +1987,48 @@
         <v>18</v>
       </c>
       <c r="C1" t="s">
+        <v>70</v>
+      </c>
+      <c r="D1" t="s">
         <v>71</v>
       </c>
+    </row>
+    <row r="2" spans="1:4">
+      <c r="A2" t="s">
+        <v>5</v>
+      </c>
+      <c r="B2" t="s">
+        <v>19</v>
+      </c>
+      <c r="C2" t="s">
+        <v>42</v>
+      </c>
+      <c r="D2" t="s">
+        <v>72</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet36.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A5CE032F-302C-42A6-BC66-0FA2D092FC8A}">
+  <dimension ref="A1:D2"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" spans="1:4">
+      <c r="A1" t="s">
+        <v>17</v>
+      </c>
+      <c r="B1" t="s">
+        <v>18</v>
+      </c>
+      <c r="C1" t="s">
+        <v>70</v>
+      </c>
       <c r="D1" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
     <row r="2" spans="1:4">
@@ -1917,7 +2039,7 @@
         <v>19</v>
       </c>
       <c r="C2" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D2" t="s">
         <v>73</v>
@@ -1928,45 +2050,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet35.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A5CE032F-302C-42A6-BC66-0FA2D092FC8A}">
-  <dimension ref="A1:D2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1" spans="1:4">
-      <c r="A1" t="s">
-        <v>17</v>
-      </c>
-      <c r="B1" t="s">
-        <v>18</v>
-      </c>
-      <c r="C1" t="s">
-        <v>71</v>
-      </c>
-      <c r="D1" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4">
-      <c r="A2" t="s">
-        <v>5</v>
-      </c>
-      <c r="B2" t="s">
-        <v>19</v>
-      </c>
-      <c r="C2" t="s">
-        <v>43</v>
-      </c>
-      <c r="D2" t="s">
-        <v>74</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet36.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet37.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{74185B4F-4AE7-4DA3-9215-6ECBA7280E7B}">
   <dimension ref="A1:C2"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -1979,7 +2063,7 @@
         <v>18</v>
       </c>
       <c r="C1" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="2" spans="1:3">
@@ -1990,15 +2074,15 @@
         <v>19</v>
       </c>
       <c r="C2" t="s">
-        <v>43</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet37.xml><?xml version="1.0" encoding="utf-8"?>
+        <v>42</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet38.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7D8774BA-3EC4-46E1-BB9D-1078ACED313F}">
   <dimension ref="A1:I2"/>
   <sheetFormatPr defaultColWidth="14" defaultRowHeight="15"/>
@@ -2011,13 +2095,13 @@
         <v>18</v>
       </c>
       <c r="C1" t="s">
+        <v>70</v>
+      </c>
+      <c r="D1" t="s">
         <v>71</v>
       </c>
-      <c r="D1" t="s">
-        <v>72</v>
-      </c>
       <c r="E1" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="F1" t="s">
         <v>21</v>
@@ -2026,47 +2110,47 @@
         <v>23</v>
       </c>
       <c r="H1" t="s">
+        <v>75</v>
+      </c>
+      <c r="I1" t="s">
         <v>76</v>
       </c>
-      <c r="I1" t="s">
+    </row>
+    <row r="2" spans="1:9">
+      <c r="A2" t="s">
+        <v>5</v>
+      </c>
+      <c r="B2" t="s">
+        <v>19</v>
+      </c>
+      <c r="C2" t="s">
+        <v>42</v>
+      </c>
+      <c r="D2" t="s">
         <v>77</v>
       </c>
-    </row>
-    <row r="2" spans="1:9">
-      <c r="A2" t="s">
-        <v>5</v>
-      </c>
-      <c r="B2" t="s">
-        <v>19</v>
-      </c>
-      <c r="C2" t="s">
-        <v>43</v>
-      </c>
-      <c r="D2" t="s">
+      <c r="E2" t="s">
         <v>78</v>
       </c>
-      <c r="E2" t="s">
+      <c r="F2" t="s">
         <v>79</v>
       </c>
-      <c r="F2" t="s">
+      <c r="G2" t="s">
         <v>80</v>
       </c>
-      <c r="G2" t="s">
+      <c r="H2" t="s">
         <v>81</v>
       </c>
-      <c r="H2" t="s">
+      <c r="I2" t="s">
         <v>82</v>
       </c>
-      <c r="I2" t="s">
-        <v>83</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet38.xml><?xml version="1.0" encoding="utf-8"?>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet39.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A5C4203B-5A01-4381-A3CE-38EA6C51F801}">
   <dimension ref="A1:D2"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -2079,56 +2163,24 @@
         <v>18</v>
       </c>
       <c r="C1" t="s">
+        <v>70</v>
+      </c>
+      <c r="D1" t="s">
         <v>71</v>
       </c>
-      <c r="D1" t="s">
+    </row>
+    <row r="2" spans="1:4">
+      <c r="A2" t="s">
+        <v>5</v>
+      </c>
+      <c r="B2" t="s">
+        <v>19</v>
+      </c>
+      <c r="C2" t="s">
+        <v>42</v>
+      </c>
+      <c r="D2" t="s">
         <v>72</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4">
-      <c r="A2" t="s">
-        <v>5</v>
-      </c>
-      <c r="B2" t="s">
-        <v>19</v>
-      </c>
-      <c r="C2" t="s">
-        <v>43</v>
-      </c>
-      <c r="D2" t="s">
-        <v>73</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet39.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{35D5D97A-4287-4435-9AB2-0BB45EA4FBC3}">
-  <dimension ref="A1:C2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1" spans="1:3">
-      <c r="A1" t="s">
-        <v>17</v>
-      </c>
-      <c r="B1" t="s">
-        <v>18</v>
-      </c>
-      <c r="C1" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3">
-      <c r="A2" t="s">
-        <v>5</v>
-      </c>
-      <c r="B2" t="s">
-        <v>19</v>
-      </c>
-      <c r="C2" t="s">
-        <v>43</v>
       </c>
     </row>
   </sheetData>
@@ -2160,6 +2212,38 @@
 </file>
 
 <file path=xl/worksheets/sheet40.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{35D5D97A-4287-4435-9AB2-0BB45EA4FBC3}">
+  <dimension ref="A1:C2"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" spans="1:3">
+      <c r="A1" t="s">
+        <v>17</v>
+      </c>
+      <c r="B1" t="s">
+        <v>18</v>
+      </c>
+      <c r="C1" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3">
+      <c r="A2" t="s">
+        <v>5</v>
+      </c>
+      <c r="B2" t="s">
+        <v>19</v>
+      </c>
+      <c r="C2" t="s">
+        <v>42</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet41.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{294C6248-6B39-4869-9A5F-1A9888AB4466}">
   <dimension ref="A1:D2"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -2172,10 +2256,10 @@
         <v>18</v>
       </c>
       <c r="C1" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="D1" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
     </row>
     <row r="2" spans="1:4">
@@ -2186,18 +2270,18 @@
         <v>19</v>
       </c>
       <c r="C2" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D2" t="s">
-        <v>84</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet41.xml><?xml version="1.0" encoding="utf-8"?>
+        <v>83</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet42.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{56AA5574-913A-4A1D-9D18-82898727775C}">
   <dimension ref="A1:C2"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -2207,13 +2291,45 @@
   <sheetData>
     <row r="1" spans="1:3">
       <c r="A1" t="s">
+        <v>84</v>
+      </c>
+      <c r="B1" t="s">
         <v>85</v>
       </c>
-      <c r="B1" t="s">
+      <c r="C1" t="s">
         <v>86</v>
       </c>
+    </row>
+    <row r="2" spans="1:3">
+      <c r="A2" t="s">
+        <v>6</v>
+      </c>
+      <c r="B2" t="s">
+        <v>44</v>
+      </c>
+      <c r="C2" t="s">
+        <v>87</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet43.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D1996804-B5A0-41DE-8EAB-89A8717FC7C7}">
+  <dimension ref="A1:C2"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" spans="1:3">
+      <c r="A1" t="s">
+        <v>84</v>
+      </c>
+      <c r="B1" t="s">
+        <v>85</v>
+      </c>
       <c r="C1" t="s">
-        <v>87</v>
+        <v>23</v>
       </c>
     </row>
     <row r="2" spans="1:3">
@@ -2221,114 +2337,82 @@
         <v>6</v>
       </c>
       <c r="B2" t="s">
-        <v>45</v>
+        <v>44</v>
+      </c>
+      <c r="C2" t="s">
+        <v>80</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet44.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CEEC45CA-B3F0-4D96-A6FC-9B253BF98967}">
+  <dimension ref="A1:D2"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" spans="1:4">
+      <c r="A1" t="s">
+        <v>84</v>
+      </c>
+      <c r="B1" t="s">
+        <v>85</v>
+      </c>
+      <c r="C1" t="s">
+        <v>71</v>
+      </c>
+      <c r="D1" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4">
+      <c r="A2" t="s">
+        <v>6</v>
+      </c>
+      <c r="B2" t="s">
+        <v>44</v>
       </c>
       <c r="C2" t="s">
         <v>88</v>
       </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet42.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D1996804-B5A0-41DE-8EAB-89A8717FC7C7}">
-  <dimension ref="A1:C2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1" spans="1:3">
-      <c r="A1" t="s">
-        <v>85</v>
-      </c>
-      <c r="B1" t="s">
-        <v>86</v>
-      </c>
-      <c r="C1" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3">
-      <c r="A2" t="s">
-        <v>6</v>
-      </c>
-      <c r="B2" t="s">
-        <v>45</v>
-      </c>
-      <c r="C2" t="s">
-        <v>81</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet43.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CEEC45CA-B3F0-4D96-A6FC-9B253BF98967}">
-  <dimension ref="A1:D2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1" spans="1:4">
-      <c r="A1" t="s">
-        <v>85</v>
-      </c>
-      <c r="B1" t="s">
-        <v>86</v>
-      </c>
-      <c r="C1" t="s">
-        <v>72</v>
-      </c>
-      <c r="D1" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4">
-      <c r="A2" t="s">
-        <v>6</v>
-      </c>
-      <c r="B2" t="s">
-        <v>45</v>
-      </c>
-      <c r="C2" t="s">
-        <v>89</v>
-      </c>
       <c r="D2" t="s">
-        <v>81</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet44.xml><?xml version="1.0" encoding="utf-8"?>
+        <v>80</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet45.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9CEA2948-6B4B-43CF-AB32-61387B2A8875}">
   <dimension ref="A1:B2"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" t="s">
+        <v>84</v>
+      </c>
+      <c r="B1" t="s">
         <v>85</v>
       </c>
-      <c r="B1" t="s">
-        <v>86</v>
-      </c>
     </row>
     <row r="2" spans="1:2">
       <c r="A2" t="s">
         <v>6</v>
       </c>
       <c r="B2" t="s">
-        <v>45</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet45.xml><?xml version="1.0" encoding="utf-8"?>
+        <v>44</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet46.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{14C972A6-008E-41DF-A05C-AF5318F8FD4B}">
   <dimension ref="A1:I2"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -2341,13 +2425,13 @@
         <v>18</v>
       </c>
       <c r="C1" t="s">
+        <v>70</v>
+      </c>
+      <c r="D1" t="s">
         <v>71</v>
       </c>
-      <c r="D1" t="s">
-        <v>72</v>
-      </c>
       <c r="E1" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="F1" t="s">
         <v>21</v>
@@ -2356,13 +2440,78 @@
         <v>23</v>
       </c>
       <c r="H1" t="s">
+        <v>75</v>
+      </c>
+      <c r="I1" t="s">
         <v>76</v>
       </c>
-      <c r="I1" t="s">
+    </row>
+    <row r="2" spans="1:9">
+      <c r="A2" t="s">
+        <v>5</v>
+      </c>
+      <c r="B2" t="s">
+        <v>19</v>
+      </c>
+      <c r="C2" t="s">
+        <v>42</v>
+      </c>
+      <c r="D2" t="s">
         <v>77</v>
       </c>
-    </row>
-    <row r="2" spans="1:9">
+      <c r="E2" t="s">
+        <v>78</v>
+      </c>
+      <c r="F2" t="s">
+        <v>79</v>
+      </c>
+      <c r="G2" t="s">
+        <v>80</v>
+      </c>
+      <c r="H2" t="s">
+        <v>81</v>
+      </c>
+      <c r="I2" t="s">
+        <v>82</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet47.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8DC0861F-7791-458B-B1CF-76DF8B36CFCB}">
+  <dimension ref="A1:H2"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" spans="1:8">
+      <c r="A1" t="s">
+        <v>17</v>
+      </c>
+      <c r="B1" t="s">
+        <v>18</v>
+      </c>
+      <c r="C1" t="s">
+        <v>70</v>
+      </c>
+      <c r="D1" t="s">
+        <v>74</v>
+      </c>
+      <c r="E1" t="s">
+        <v>21</v>
+      </c>
+      <c r="F1" t="s">
+        <v>23</v>
+      </c>
+      <c r="G1" t="s">
+        <v>75</v>
+      </c>
+      <c r="H1" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8">
       <c r="A2" t="s">
         <v>5</v>
       </c>
@@ -2370,7 +2519,7 @@
         <v>19</v>
       </c>
       <c r="C2" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D2" t="s">
         <v>78</v>
@@ -2387,78 +2536,13 @@
       <c r="H2" t="s">
         <v>82</v>
       </c>
-      <c r="I2" t="s">
-        <v>83</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet46.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8DC0861F-7791-458B-B1CF-76DF8B36CFCB}">
-  <dimension ref="A1:H2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1" spans="1:8">
-      <c r="A1" t="s">
-        <v>17</v>
-      </c>
-      <c r="B1" t="s">
-        <v>18</v>
-      </c>
-      <c r="C1" t="s">
-        <v>71</v>
-      </c>
-      <c r="D1" t="s">
-        <v>75</v>
-      </c>
-      <c r="E1" t="s">
-        <v>21</v>
-      </c>
-      <c r="F1" t="s">
-        <v>23</v>
-      </c>
-      <c r="G1" t="s">
-        <v>76</v>
-      </c>
-      <c r="H1" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="2" spans="1:8">
-      <c r="A2" t="s">
-        <v>5</v>
-      </c>
-      <c r="B2" t="s">
-        <v>19</v>
-      </c>
-      <c r="C2" t="s">
-        <v>43</v>
-      </c>
-      <c r="D2" t="s">
-        <v>79</v>
-      </c>
-      <c r="E2" t="s">
-        <v>80</v>
-      </c>
-      <c r="F2" t="s">
-        <v>81</v>
-      </c>
-      <c r="G2" t="s">
-        <v>82</v>
-      </c>
-      <c r="H2" t="s">
-        <v>83</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet47.xml><?xml version="1.0" encoding="utf-8"?>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet48.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{702F240E-6DDC-40E1-A471-6D34CE8EC8A9}">
   <dimension ref="A1:C2"/>
   <sheetFormatPr defaultColWidth="14.5703125" defaultRowHeight="15"/>
@@ -2471,7 +2555,7 @@
         <v>18</v>
       </c>
       <c r="C1" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="2" spans="1:3">
@@ -2482,15 +2566,15 @@
         <v>19</v>
       </c>
       <c r="C2" t="s">
-        <v>43</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet48.xml><?xml version="1.0" encoding="utf-8"?>
+        <v>42</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet49.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1B6F8DC7-5D71-4D0F-BD39-85D8C4667F97}">
   <dimension ref="A1:D2"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -2503,74 +2587,24 @@
         <v>18</v>
       </c>
       <c r="C1" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="D1" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4">
+      <c r="A2" t="s">
+        <v>5</v>
+      </c>
+      <c r="B2" t="s">
+        <v>19</v>
+      </c>
+      <c r="C2" t="s">
+        <v>42</v>
+      </c>
+      <c r="D2" t="s">
         <v>90</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4">
-      <c r="A2" t="s">
-        <v>5</v>
-      </c>
-      <c r="B2" t="s">
-        <v>19</v>
-      </c>
-      <c r="C2" t="s">
-        <v>43</v>
-      </c>
-      <c r="D2" t="s">
-        <v>91</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet49.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7696B79F-033D-404F-9E1D-E22617A3BDAC}">
-  <dimension ref="A1:F2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1" spans="1:6">
-      <c r="A1" s="7" t="s">
-        <v>92</v>
-      </c>
-      <c r="B1" t="s">
-        <v>93</v>
-      </c>
-      <c r="C1" t="s">
-        <v>94</v>
-      </c>
-      <c r="D1" t="s">
-        <v>21</v>
-      </c>
-      <c r="E1" t="s">
-        <v>22</v>
-      </c>
-      <c r="F1" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="2" spans="1:6">
-      <c r="A2" s="7" t="s">
-        <v>95</v>
-      </c>
-      <c r="B2" t="s">
-        <v>96</v>
-      </c>
-      <c r="C2" t="s">
-        <v>97</v>
-      </c>
-      <c r="D2" t="s">
-        <v>26</v>
-      </c>
-      <c r="E2" t="s">
-        <v>27</v>
-      </c>
-      <c r="F2" t="s">
-        <v>28</v>
       </c>
     </row>
   </sheetData>
@@ -2609,19 +2643,157 @@
 </file>
 
 <file path=xl/worksheets/sheet50.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B54BFBCC-7C3F-461E-8867-D0FC9227F8D2}">
+  <dimension ref="A1:E2"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" spans="1:5">
+      <c r="A1" t="s">
+        <v>20</v>
+      </c>
+      <c r="B1" t="s">
+        <v>15</v>
+      </c>
+      <c r="C1" t="s">
+        <v>21</v>
+      </c>
+      <c r="D1" t="s">
+        <v>22</v>
+      </c>
+      <c r="E1" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5">
+      <c r="A2" t="s">
+        <v>24</v>
+      </c>
+      <c r="B2" t="s">
+        <v>25</v>
+      </c>
+      <c r="C2" t="s">
+        <v>26</v>
+      </c>
+      <c r="D2" t="s">
+        <v>27</v>
+      </c>
+      <c r="E2" t="s">
+        <v>28</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet51.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1B6C8D86-E59C-4B0D-9190-1A812D82FFD2}">
+  <dimension ref="A1:E2"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" spans="1:5">
+      <c r="A1" t="s">
+        <v>20</v>
+      </c>
+      <c r="B1" t="s">
+        <v>15</v>
+      </c>
+      <c r="C1" t="s">
+        <v>21</v>
+      </c>
+      <c r="D1" t="s">
+        <v>22</v>
+      </c>
+      <c r="E1" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5">
+      <c r="A2" t="s">
+        <v>24</v>
+      </c>
+      <c r="B2" t="s">
+        <v>25</v>
+      </c>
+      <c r="C2" t="s">
+        <v>26</v>
+      </c>
+      <c r="D2" t="s">
+        <v>27</v>
+      </c>
+      <c r="E2" t="s">
+        <v>28</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet52.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7696B79F-033D-404F-9E1D-E22617A3BDAC}">
+  <dimension ref="A1:F2"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" spans="1:6">
+      <c r="A1" s="7" t="s">
+        <v>91</v>
+      </c>
+      <c r="B1" t="s">
+        <v>92</v>
+      </c>
+      <c r="C1" t="s">
+        <v>93</v>
+      </c>
+      <c r="D1" t="s">
+        <v>21</v>
+      </c>
+      <c r="E1" t="s">
+        <v>22</v>
+      </c>
+      <c r="F1" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6">
+      <c r="A2" s="7" t="s">
+        <v>94</v>
+      </c>
+      <c r="B2" t="s">
+        <v>95</v>
+      </c>
+      <c r="C2" t="s">
+        <v>96</v>
+      </c>
+      <c r="D2" t="s">
+        <v>26</v>
+      </c>
+      <c r="E2" t="s">
+        <v>27</v>
+      </c>
+      <c r="F2" t="s">
+        <v>28</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet53.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4A192C83-0F47-4844-AB01-D5A2E984F7DB}">
   <dimension ref="A1:G2"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:7">
       <c r="A1" s="6" t="s">
+        <v>91</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>92</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="C1" s="1" t="s">
         <v>93</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>94</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>21</v>
@@ -2633,18 +2805,18 @@
         <v>23</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
     </row>
     <row r="2" spans="1:7">
       <c r="A2" s="6" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="D2" s="1" t="s">
         <v>26</v>
@@ -2656,51 +2828,51 @@
         <v>28</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>100</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet51.xml><?xml version="1.0" encoding="utf-8"?>
+        <v>99</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet54.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3011021D-4819-4690-B3D7-76A026828EC9}">
   <dimension ref="A1:G2"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:7">
       <c r="A1" s="1" t="s">
+        <v>100</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>101</v>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>93</v>
-      </c>
-      <c r="C1" s="1" t="s">
+      <c r="D1" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="E1" s="1" t="s">
         <v>102</v>
       </c>
-      <c r="D1" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="E1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>103</v>
       </c>
-      <c r="F1" s="1" t="s">
-        <v>104</v>
-      </c>
       <c r="G1" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="2" spans="1:7">
       <c r="A2" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="B2" s="1" t="s">
         <v>105</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="C2" s="1" t="s">
         <v>106</v>
-      </c>
-      <c r="C2" s="1" t="s">
-        <v>107</v>
       </c>
       <c r="D2" s="1" t="s">
         <v>26</v>
@@ -2712,57 +2884,57 @@
         <v>28</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>108</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet52.xml><?xml version="1.0" encoding="utf-8"?>
+        <v>107</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet55.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{02E7FD6A-85B6-48DD-983C-2558ACC9E840}">
   <dimension ref="A1:C2"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:3">
       <c r="A1" s="1" t="s">
+        <v>100</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>101</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>93</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>102</v>
       </c>
     </row>
     <row r="2" spans="1:3">
       <c r="A2" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="B2" s="1" t="s">
         <v>105</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="C2" s="1" t="s">
         <v>106</v>
       </c>
-      <c r="C2" s="1" t="s">
-        <v>107</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet53.xml><?xml version="1.0" encoding="utf-8"?>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet56.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{47958D0E-DE08-4FC8-AE6D-9F22489AEEFF}">
   <dimension ref="A1:F2"/>
   <sheetFormatPr defaultColWidth="18.85546875" defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:6">
       <c r="A1" t="s">
-        <v>85</v>
-      </c>
-      <c r="B1" t="s">
-        <v>109</v>
+        <v>84</v>
+      </c>
+      <c r="B1" t="s">
+        <v>108</v>
       </c>
       <c r="C1" t="s">
         <v>15</v>
@@ -2782,10 +2954,10 @@
         <v>6</v>
       </c>
       <c r="B2" t="s">
+        <v>109</v>
+      </c>
+      <c r="C2" t="s">
         <v>110</v>
-      </c>
-      <c r="C2" t="s">
-        <v>111</v>
       </c>
       <c r="D2" t="s">
         <v>26</v>
@@ -2802,27 +2974,30 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet54.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet57.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{42B9D63B-BC76-46EA-ADB4-8766AF6817A7}">
   <dimension ref="A1:A2"/>
   <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="19.28515625" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:1">
       <c r="A1" s="1" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
     </row>
     <row r="2" spans="1:1">
       <c r="A2" s="1" t="s">
-        <v>113</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet55.xml><?xml version="1.0" encoding="utf-8"?>
+        <v>112</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet58.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{006ED08C-28C3-460C-941C-159F30186152}">
   <dimension ref="A1:B2"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -2833,36 +3008,36 @@
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" t="s">
-        <v>85</v>
-      </c>
-      <c r="B1" t="s">
+        <v>84</v>
+      </c>
+      <c r="B1" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2">
+      <c r="A2" t="s">
         <v>114</v>
       </c>
-    </row>
-    <row r="2" spans="1:2">
-      <c r="A2" t="s">
+      <c r="B2" t="s">
         <v>115</v>
       </c>
-      <c r="B2" t="s">
-        <v>116</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet56.xml><?xml version="1.0" encoding="utf-8"?>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet59.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DDA25AE5-6655-45CB-9149-A8A61B5E732F}">
   <dimension ref="A1:F2"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:6">
       <c r="A1" t="s">
-        <v>85</v>
-      </c>
-      <c r="B1" t="s">
-        <v>109</v>
+        <v>84</v>
+      </c>
+      <c r="B1" t="s">
+        <v>108</v>
       </c>
       <c r="C1" t="s">
         <v>15</v>
@@ -2882,10 +3057,10 @@
         <v>6</v>
       </c>
       <c r="B2" t="s">
+        <v>109</v>
+      </c>
+      <c r="C2" t="s">
         <v>110</v>
-      </c>
-      <c r="C2" t="s">
-        <v>111</v>
       </c>
       <c r="D2" t="s">
         <v>26</v>
@@ -2894,150 +3069,6 @@
         <v>27</v>
       </c>
       <c r="F2" t="s">
-        <v>28</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet57.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C2F0C090-2891-474A-9164-D1CFD32D2A23}">
-  <dimension ref="A1:F2"/>
-  <sheetFormatPr defaultColWidth="14.7109375" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1" spans="1:6">
-      <c r="A1" t="s">
-        <v>85</v>
-      </c>
-      <c r="B1" t="s">
-        <v>109</v>
-      </c>
-      <c r="C1" t="s">
-        <v>15</v>
-      </c>
-      <c r="D1" t="s">
-        <v>21</v>
-      </c>
-      <c r="E1" t="s">
-        <v>22</v>
-      </c>
-      <c r="F1" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="2" spans="1:6">
-      <c r="A2" t="s">
-        <v>6</v>
-      </c>
-      <c r="B2" t="s">
-        <v>110</v>
-      </c>
-      <c r="C2" t="s">
-        <v>111</v>
-      </c>
-      <c r="D2" t="s">
-        <v>26</v>
-      </c>
-      <c r="E2" t="s">
-        <v>27</v>
-      </c>
-      <c r="F2" t="s">
-        <v>28</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet58.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{22B1F532-E3A9-4507-B737-44BD308773F5}">
-  <dimension ref="A1:F2"/>
-  <sheetFormatPr defaultColWidth="13.85546875" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1" spans="1:6">
-      <c r="A1" t="s">
-        <v>85</v>
-      </c>
-      <c r="B1" t="s">
-        <v>109</v>
-      </c>
-      <c r="C1" t="s">
-        <v>15</v>
-      </c>
-      <c r="D1" t="s">
-        <v>21</v>
-      </c>
-      <c r="E1" t="s">
-        <v>22</v>
-      </c>
-      <c r="F1" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="2" spans="1:6">
-      <c r="A2" t="s">
-        <v>6</v>
-      </c>
-      <c r="B2" t="s">
-        <v>110</v>
-      </c>
-      <c r="C2" t="s">
-        <v>111</v>
-      </c>
-      <c r="D2" t="s">
-        <v>26</v>
-      </c>
-      <c r="E2" t="s">
-        <v>27</v>
-      </c>
-      <c r="F2" t="s">
-        <v>28</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet59.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4F180104-CB7F-4225-88B2-B743F65A2E71}">
-  <dimension ref="A1:E2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1" spans="1:5">
-      <c r="A1" t="s">
-        <v>20</v>
-      </c>
-      <c r="B1" t="s">
-        <v>15</v>
-      </c>
-      <c r="C1" t="s">
-        <v>21</v>
-      </c>
-      <c r="D1" t="s">
-        <v>22</v>
-      </c>
-      <c r="E1" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5">
-      <c r="A2" t="s">
-        <v>24</v>
-      </c>
-      <c r="B2" t="s">
-        <v>25</v>
-      </c>
-      <c r="C2" t="s">
-        <v>26</v>
-      </c>
-      <c r="D2" t="s">
-        <v>27</v>
-      </c>
-      <c r="E2" t="s">
         <v>28</v>
       </c>
     </row>
@@ -3097,42 +3128,232 @@
 </file>
 
 <file path=xl/worksheets/sheet60.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C2F0C090-2891-474A-9164-D1CFD32D2A23}">
+  <dimension ref="A1:F2"/>
+  <sheetFormatPr defaultColWidth="14.7109375" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" spans="1:6">
+      <c r="A1" t="s">
+        <v>84</v>
+      </c>
+      <c r="B1" t="s">
+        <v>108</v>
+      </c>
+      <c r="C1" t="s">
+        <v>15</v>
+      </c>
+      <c r="D1" t="s">
+        <v>21</v>
+      </c>
+      <c r="E1" t="s">
+        <v>22</v>
+      </c>
+      <c r="F1" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6">
+      <c r="A2" t="s">
+        <v>6</v>
+      </c>
+      <c r="B2" t="s">
+        <v>109</v>
+      </c>
+      <c r="C2" t="s">
+        <v>110</v>
+      </c>
+      <c r="D2" t="s">
+        <v>26</v>
+      </c>
+      <c r="E2" t="s">
+        <v>27</v>
+      </c>
+      <c r="F2" t="s">
+        <v>28</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet61.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{22B1F532-E3A9-4507-B737-44BD308773F5}">
+  <dimension ref="A1:F2"/>
+  <sheetFormatPr defaultColWidth="13.85546875" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" spans="1:6">
+      <c r="A1" t="s">
+        <v>84</v>
+      </c>
+      <c r="B1" t="s">
+        <v>108</v>
+      </c>
+      <c r="C1" t="s">
+        <v>15</v>
+      </c>
+      <c r="D1" t="s">
+        <v>21</v>
+      </c>
+      <c r="E1" t="s">
+        <v>22</v>
+      </c>
+      <c r="F1" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6">
+      <c r="A2" t="s">
+        <v>6</v>
+      </c>
+      <c r="B2" t="s">
+        <v>109</v>
+      </c>
+      <c r="C2" t="s">
+        <v>110</v>
+      </c>
+      <c r="D2" t="s">
+        <v>26</v>
+      </c>
+      <c r="E2" t="s">
+        <v>27</v>
+      </c>
+      <c r="F2" t="s">
+        <v>28</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet62.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{545270BF-46D2-413A-9419-76683720126A}">
+  <dimension ref="A1:B2"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" spans="1:2">
+      <c r="A1" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2">
+      <c r="A2" s="1" t="s">
+        <v>118</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>119</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet63.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7A8A7719-5FC7-406C-A809-EBB81C7D304F}">
+  <dimension ref="A1:A2"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" spans="1:1">
+      <c r="A1" s="1" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1">
+      <c r="A2" s="1" t="s">
+        <v>120</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet64.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4F180104-CB7F-4225-88B2-B743F65A2E71}">
+  <dimension ref="A1:E2"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" spans="1:5">
+      <c r="A1" t="s">
+        <v>20</v>
+      </c>
+      <c r="B1" t="s">
+        <v>15</v>
+      </c>
+      <c r="C1" t="s">
+        <v>21</v>
+      </c>
+      <c r="D1" t="s">
+        <v>22</v>
+      </c>
+      <c r="E1" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5">
+      <c r="A2" t="s">
+        <v>24</v>
+      </c>
+      <c r="B2" t="s">
+        <v>25</v>
+      </c>
+      <c r="C2" t="s">
+        <v>26</v>
+      </c>
+      <c r="D2" t="s">
+        <v>27</v>
+      </c>
+      <c r="E2" t="s">
+        <v>28</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet65.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F12CCDE5-920D-49D0-950B-159A5A491EE7}">
   <dimension ref="A1:G2"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:7">
       <c r="A1" s="1" t="s">
+        <v>100</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>101</v>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>93</v>
-      </c>
-      <c r="C1" s="1" t="s">
+      <c r="D1" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="E1" s="1" t="s">
         <v>102</v>
       </c>
-      <c r="D1" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="E1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>103</v>
       </c>
-      <c r="F1" s="1" t="s">
-        <v>104</v>
-      </c>
       <c r="G1" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="2" spans="1:7">
       <c r="A2" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="B2" s="1" t="s">
         <v>105</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="C2" s="1" t="s">
         <v>106</v>
-      </c>
-      <c r="C2" s="1" t="s">
-        <v>107</v>
       </c>
       <c r="D2" s="1" t="s">
         <v>26</v>
@@ -3144,20 +3365,20 @@
         <v>28</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>108</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet61.xml><?xml version="1.0" encoding="utf-8"?>
+        <v>107</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet66.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{57C2C09D-3106-4A2C-A972-09AF8ED3E7CC}">
   <dimension ref="A1:B2"/>
   <sheetFormatPr defaultColWidth="13.85546875" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="16384" width="13.85546875" customWidth="1"/>
+    <col min="1" max="1" width="13.85546875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2">
@@ -3181,7 +3402,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet62.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet67.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{28C5798F-1A42-4810-A643-274C39BB5B89}">
   <dimension ref="A1:D2"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -3194,7 +3415,7 @@
         <v>15</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="D1" s="6" t="s">
         <v>1</v>
@@ -3202,16 +3423,78 @@
     </row>
     <row r="2" spans="1:4">
       <c r="A2" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="B2" s="1" t="s">
         <v>50</v>
       </c>
+      <c r="C2" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="D2" s="6" t="s">
+        <v>49</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet68.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DD547580-CDD4-4CA1-99D1-F4DBEB4DC61C}">
+  <dimension ref="A1:B2"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="16" customWidth="1"/>
+    <col min="2" max="2" width="14.5703125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2">
+      <c r="A1" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="B1" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2">
+      <c r="A2" s="1" t="s">
+        <v>112</v>
+      </c>
+      <c r="B2" t="s">
+        <v>122</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet69.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5C851C18-BB40-4C4C-9358-B9D27BF745A2}">
+  <dimension ref="A1:C2"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" spans="1:3">
+      <c r="A1" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>124</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3">
+      <c r="A2" s="1" t="s">
+        <v>122</v>
+      </c>
       <c r="B2" s="1" t="s">
-        <v>51</v>
+        <v>125</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>52</v>
-      </c>
-      <c r="D2" s="6" t="s">
-        <v>50</v>
+        <v>101</v>
       </c>
     </row>
   </sheetData>
@@ -3221,18 +3504,220 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{29DDC4E0-08CB-46D1-AE6D-9F161D97ECBA}">
-  <dimension ref="A1:F2"/>
+  <dimension ref="A1:E2"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="39.5703125" customWidth="1"/>
   </cols>
   <sheetData>
+    <row r="1" spans="1:5">
+      <c r="A1" t="s">
+        <v>20</v>
+      </c>
+      <c r="B1" t="s">
+        <v>15</v>
+      </c>
+      <c r="C1" t="s">
+        <v>21</v>
+      </c>
+      <c r="D1" t="s">
+        <v>22</v>
+      </c>
+      <c r="E1" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5">
+      <c r="A2" t="s">
+        <v>24</v>
+      </c>
+      <c r="B2" t="s">
+        <v>25</v>
+      </c>
+      <c r="C2" t="s">
+        <v>26</v>
+      </c>
+      <c r="D2" t="s">
+        <v>27</v>
+      </c>
+      <c r="E2" t="s">
+        <v>28</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet70.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{30CA7E00-9554-459F-BF47-6B8E0B27B5B9}">
+  <dimension ref="A1:C2"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" spans="1:3">
+      <c r="A1" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>124</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3">
+      <c r="A2" s="1" t="s">
+        <v>122</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>125</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>101</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet71.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{93B51C47-FA71-48A7-A2FD-49CB882674F9}">
+  <dimension ref="A1:C2"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" spans="1:3">
+      <c r="A1" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>124</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3">
+      <c r="A2" s="1" t="s">
+        <v>122</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>125</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>101</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet72.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{485C4B2E-FC36-4946-BA8B-78C7FADE4211}">
+  <dimension ref="A1:G2"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" spans="1:7">
+      <c r="A1" s="1" t="s">
+        <v>100</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>101</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>102</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>103</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7">
+      <c r="A2" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>105</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="F2" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="G2" s="1" t="s">
+        <v>107</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet73.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EBC66432-A9A4-4E48-A474-1F35C5F1C633}">
+  <dimension ref="A1:D2"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" spans="1:4">
+      <c r="A1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="D1" s="6" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4">
+      <c r="A2" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="D2" s="6" t="s">
+        <v>49</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet74.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{849D9C7E-7FB2-4797-90F9-A5CEADA89D9C}">
+  <dimension ref="A1:F2"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
     <row r="1" spans="1:6">
       <c r="A1" t="s">
-        <v>29</v>
-      </c>
-      <c r="B1" t="s">
-        <v>20</v>
+        <v>84</v>
+      </c>
+      <c r="B1" t="s">
+        <v>108</v>
       </c>
       <c r="C1" t="s">
         <v>15</v>
@@ -3249,13 +3734,13 @@
     </row>
     <row r="2" spans="1:6">
       <c r="A2" t="s">
-        <v>5</v>
-      </c>
-      <c r="B2" t="s">
-        <v>24</v>
+        <v>6</v>
+      </c>
+      <c r="B2" t="s">
+        <v>109</v>
       </c>
       <c r="C2" t="s">
-        <v>25</v>
+        <v>110</v>
       </c>
       <c r="D2" t="s">
         <v>26</v>
@@ -3265,6 +3750,148 @@
       </c>
       <c r="F2" t="s">
         <v>28</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet75.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C4A8AAC5-4185-4C1C-93D4-1D0A64F4E1B7}">
+  <dimension ref="A1:B2"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" spans="1:2">
+      <c r="A1" s="1" t="s">
+        <v>84</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2">
+      <c r="A2" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>127</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet76.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9539B7F2-18EC-49F7-91A3-B0ABA5965519}">
+  <dimension ref="A1:B2"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" spans="1:2">
+      <c r="A1" s="1" t="s">
+        <v>84</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2">
+      <c r="A2" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>127</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet77.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E1D6F0D0-409C-41C4-B05D-2C73D11E088E}">
+  <dimension ref="A1:C2"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" spans="1:3">
+      <c r="A1" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3">
+      <c r="A2" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>129</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>130</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet78.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B0B71A08-ABCC-473C-BDAE-49D46803B591}">
+  <dimension ref="A1:C2"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" spans="1:3">
+      <c r="A1" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3">
+      <c r="A2" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>129</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>130</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet79.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FFCE88DA-A526-4A91-B38E-F41DCEC7BD09}">
+  <dimension ref="A1:B2"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" spans="1:2">
+      <c r="A1" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2">
+      <c r="A2" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>129</v>
       </c>
     </row>
   </sheetData>
@@ -3282,13 +3909,13 @@
   <sheetData>
     <row r="1" spans="1:4">
       <c r="A1" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="B1" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="C1" s="3" t="s">
         <v>31</v>
-      </c>
-      <c r="C1" s="3" t="s">
-        <v>32</v>
       </c>
       <c r="D1" s="3" t="s">
         <v>13</v>
@@ -3299,13 +3926,143 @@
         <v>19</v>
       </c>
       <c r="B2" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="C2" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="C2" s="3" t="s">
+      <c r="D2" s="3" t="s">
+        <v>33</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet80.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{223C53EB-97BE-4EFF-B890-3A3BD91E9E72}">
+  <dimension ref="A1:B2"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" spans="1:2">
+      <c r="A1" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="D2" s="3" t="s">
+      <c r="B1" s="1" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2">
+      <c r="A2" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>129</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet81.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7E2B8556-771D-4DAD-8C21-33E755A02656}">
+  <dimension ref="A1:B2"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" spans="1:2">
+      <c r="A1" s="1" t="s">
         <v>34</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2">
+      <c r="A2" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>129</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet82.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A7FA2BA4-A228-45F5-B096-B0B6F3C5FCD9}">
+  <dimension ref="A1:B2"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" spans="1:2">
+      <c r="A1" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2">
+      <c r="A2" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>129</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet83.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{763B8C95-495E-4740-BDD6-D904F75864FB}">
+  <dimension ref="A1:B2"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" spans="1:2">
+      <c r="A1" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2">
+      <c r="A2" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>129</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet84.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0D8151D4-D1A1-47AD-8B8F-43868BB4348D}">
+  <dimension ref="A1:B2"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" spans="1:2">
+      <c r="A1" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2">
+      <c r="A2" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>129</v>
       </c>
     </row>
   </sheetData>
@@ -3320,16 +4077,16 @@
   <sheetData>
     <row r="1" spans="1:4">
       <c r="A1" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="D1" s="3" t="s">
         <v>35</v>
-      </c>
-      <c r="B1" s="3" t="s">
-        <v>30</v>
-      </c>
-      <c r="C1" s="3" t="s">
-        <v>31</v>
-      </c>
-      <c r="D1" s="3" t="s">
-        <v>36</v>
       </c>
     </row>
     <row r="2" spans="1:4">
@@ -3340,10 +4097,10 @@
         <v>19</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Added 6 automation tasks
</commit_message>
<xml_diff>
--- a/testData/requirementTabTestData/requirementTab_testData.xlsx
+++ b/testData/requirementTabTestData/requirementTab_testData.xlsx
@@ -1,11 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29912"/>
-  <workbookPr/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{72AAFBD2-10B3-4F05-B512-576B35A07306}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\SwarnadeepMondal\Desktop\Testing24-03\testData\requirementTabTestData\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" firstSheet="78" activeTab="80" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" activeTab="80"/>
   </bookViews>
   <sheets>
     <sheet name="tc001" sheetId="1" r:id="rId1"/>
@@ -88,30 +91,15 @@
     <sheet name="tc130" sheetId="80" r:id="rId78"/>
     <sheet name="tc131" sheetId="81" r:id="rId79"/>
     <sheet name="tc132" sheetId="82" r:id="rId80"/>
-    <sheet name="tc133" sheetId="83" r:id="rId81"/>
+    <sheet name="tc123" sheetId="84" r:id="rId81"/>
+    <sheet name="tc133" sheetId="83" r:id="rId82"/>
   </sheets>
-  <calcPr calcId="191028"/>
-  <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
-      <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
-  </extLst>
+  <calcPr/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="613" uniqueCount="129">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <si>
     <t>Project Name</t>
   </si>
@@ -499,11 +487,17 @@
   <si>
     <t>jTesting</t>
   </si>
+  <si>
+    <t>req</t>
+  </si>
+  <si>
+    <t>RQ-2123</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <fonts count="8">
     <font>
       <sz val="11"/>
@@ -519,10 +513,15 @@
       <charset val="134"/>
     </font>
     <font>
-      <sz val="8.1999999999999993"/>
+      <sz val="8.2"/>
       <color rgb="FF101828"/>
       <name val="Arial"/>
       <charset val="134"/>
+    </font>
+    <font>
+      <sz val="6.8"/>
+      <color rgb="FF6AAB73"/>
+      <name val="JetBrains Mono"/>
     </font>
     <font>
       <sz val="11"/>
@@ -533,18 +532,13 @@
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
-      <name val="Aptos Narrow"/>
-    </font>
-    <font>
-      <sz val="6.8"/>
-      <color rgb="FF6AAB73"/>
-      <name val="JetBrains Mono"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
     </font>
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
+      <name val="Aptos Narrow"/>
     </font>
     <font>
       <sz val="11"/>
@@ -561,13 +555,7 @@
     </fill>
   </fills>
   <borders count="1">
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
+    <border/>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
@@ -587,14 +575,6 @@
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleMedium9"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
 </styleSheet>
 </file>
 
@@ -603,10 +583,10 @@
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
-        <a:sysClr val="windowText" lastClr="000000"/>
+        <a:sysClr val="windowText"/>
       </a:dk1>
       <a:lt1>
-        <a:sysClr val="window" lastClr="FFFFFF"/>
+        <a:sysClr val="window"/>
       </a:lt1>
       <a:dk2>
         <a:srgbClr val="0E2841"/>
@@ -775,6 +755,7 @@
             </a:gs>
           </a:gsLst>
           <a:lin ang="5400000" scaled="0"/>
+          <a:tileRect/>
         </a:gradFill>
         <a:gradFill rotWithShape="1">
           <a:gsLst>
@@ -801,24 +782,25 @@
             </a:gs>
           </a:gsLst>
           <a:lin ang="5400000" scaled="0"/>
+          <a:tileRect/>
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
-        <a:ln w="12700" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln w="12700" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
           <a:miter lim="800000"/>
         </a:ln>
-        <a:ln w="19050" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln w="19050" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
           <a:miter lim="800000"/>
         </a:ln>
-        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln w="25400" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
@@ -879,53 +861,26 @@
             </a:gs>
           </a:gsLst>
           <a:lin ang="5400000" scaled="0"/>
+          <a:tileRect/>
         </a:gradFill>
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
-  <a:objectDefaults>
-    <a:lnDef>
-      <a:spPr/>
-      <a:bodyPr/>
-      <a:lstStyle/>
-      <a:style>
-        <a:lnRef idx="2">
-          <a:schemeClr val="accent1"/>
-        </a:lnRef>
-        <a:fillRef idx="0">
-          <a:schemeClr val="accent1"/>
-        </a:fillRef>
-        <a:effectRef idx="1">
-          <a:schemeClr val="accent1"/>
-        </a:effectRef>
-        <a:fontRef idx="minor">
-          <a:schemeClr val="tx1"/>
-        </a:fontRef>
-      </a:style>
-    </a:lnDef>
-  </a:objectDefaults>
-  <a:extraClrSchemeLst/>
-  <a:extLst>
-    <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
-    </a:ext>
-  </a:extLst>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E3"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+<worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="30.7109375" customWidth="1"/>
-    <col min="2" max="2" width="14.140625" customWidth="1"/>
-    <col min="3" max="3" width="18.28515625" customWidth="1"/>
+    <col min="1" max="1" width="30.75" customWidth="1"/>
+    <col min="2" max="2" width="14.125" customWidth="1"/>
+    <col min="3" max="3" width="18.25" customWidth="1"/>
     <col min="4" max="4" width="16" customWidth="1"/>
-    <col min="5" max="5" width="12.28515625" customWidth="1"/>
+    <col min="5" max="5" width="12.25" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5">
+    <row r="1" ht="15">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -942,7 +897,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:5">
+    <row r="2" ht="15">
       <c r="A2" t="s">
         <v>5</v>
       </c>
@@ -959,7 +914,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="3" spans="1:5">
+    <row r="3" ht="15">
       <c r="A3" t="s">
         <v>5</v>
       </c>
@@ -977,23 +932,21 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5B3E68E9-6114-4137-93A6-9E3D35854EF2}">
-  <dimension ref="A1:E2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+<worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="37.85546875" customWidth="1"/>
-    <col min="2" max="2" width="18.85546875" customWidth="1"/>
-    <col min="3" max="3" width="16.7109375" customWidth="1"/>
-    <col min="4" max="4" width="23.140625" customWidth="1"/>
-    <col min="5" max="5" width="23.7109375" customWidth="1"/>
+    <col min="1" max="1" width="37.875" customWidth="1"/>
+    <col min="2" max="2" width="18.875" customWidth="1"/>
+    <col min="3" max="3" width="16.75" customWidth="1"/>
+    <col min="4" max="4" width="23.125" customWidth="1"/>
+    <col min="5" max="5" width="23.75" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5">
+    <row r="1" ht="15">
       <c r="A1" s="1" t="s">
         <v>37</v>
       </c>
@@ -1010,7 +963,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="2" spans="1:5">
+    <row r="2" ht="15">
       <c r="A2" s="1" t="s">
         <v>5</v>
       </c>
@@ -1028,21 +981,19 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{29BEAA1A-A534-4468-B9EC-E9F8BB732A2D}">
-  <dimension ref="A1:C2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+<worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="39.5703125" customWidth="1"/>
+    <col min="1" max="1" width="39.625" customWidth="1"/>
     <col min="2" max="2" width="23" customWidth="1"/>
-    <col min="3" max="3" width="16.7109375" customWidth="1"/>
+    <col min="3" max="3" width="16.75" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3">
+    <row r="1" ht="15">
       <c r="A1" t="s">
         <v>37</v>
       </c>
@@ -1053,7 +1004,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="2" spans="1:3">
+    <row r="2" ht="15">
       <c r="A2" t="s">
         <v>5</v>
       </c>
@@ -1065,20 +1016,18 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6FE5E322-70B6-4F63-AE80-0840E4095282}">
-  <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+<worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="28.42578125" customWidth="1"/>
-    <col min="2" max="2" width="18.5703125" customWidth="1"/>
+    <col min="1" max="1" width="28.375" customWidth="1"/>
+    <col min="2" max="2" width="18.625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2">
+    <row r="1" ht="15">
       <c r="A1" t="s">
         <v>17</v>
       </c>
@@ -1086,7 +1035,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="2" spans="1:2">
+    <row r="2" ht="15">
       <c r="A2" t="s">
         <v>5</v>
       </c>
@@ -1095,86 +1044,80 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7C4F00CF-C1AA-4EBC-984F-C64E09298E67}">
-  <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1" spans="1:2">
-      <c r="A1" s="3" t="s">
+<worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetFormatPr defaultRowHeight="14.25"/>
+  <sheetData>
+    <row r="1" ht="15">
+      <c r="A1" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="B1" s="4" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="2" spans="1:2">
-      <c r="A2" s="3" t="s">
+    <row r="2" ht="15">
+      <c r="A2" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="B2" s="3" t="s">
+      <c r="B2" s="4" t="s">
         <v>45</v>
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0C944F0C-FA76-4DBA-99AE-F54BD5BF8527}">
-  <dimension ref="A1:E2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1" spans="1:5">
-      <c r="A1" s="3" t="s">
+<worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetFormatPr defaultRowHeight="14.25"/>
+  <sheetData>
+    <row r="1" ht="15">
+      <c r="A1" s="4" t="s">
         <v>34</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="B1" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="C1" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="D1" s="4" t="s">
         <v>46</v>
       </c>
-      <c r="E1" s="3" t="s">
+      <c r="E1" s="4" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="2" spans="1:5">
-      <c r="A2" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="B2" s="3" t="s">
+    <row r="2" ht="15">
+      <c r="A2" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="B2" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="C2" s="3" t="s">
+      <c r="C2" s="4" t="s">
         <v>48</v>
       </c>
-      <c r="D2" s="3" t="s">
+      <c r="D2" s="4" t="s">
         <v>46</v>
       </c>
-      <c r="E2" s="3" t="s">
+      <c r="E2" s="4" t="s">
         <v>11</v>
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0A546074-F4ED-46C4-9BFA-1A91CD65CFD3}">
-  <dimension ref="A1:D2"/>
-  <sheetFormatPr defaultColWidth="15.5703125" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1" spans="1:4">
+<worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetFormatPr defaultColWidth="15.625" defaultRowHeight="14.25"/>
+  <sheetData>
+    <row r="1" ht="15">
       <c r="A1" s="1" t="s">
         <v>1</v>
       </c>
@@ -1184,11 +1127,11 @@
       <c r="C1" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="D1" s="6" t="s">
+      <c r="D1" s="5" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:4">
+    <row r="2" ht="15">
       <c r="A2" s="1" t="s">
         <v>49</v>
       </c>
@@ -1198,24 +1141,22 @@
       <c r="C2" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="D2" s="6" t="s">
+      <c r="D2" s="5" t="s">
         <v>49</v>
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{710D6ACC-846B-479B-9D45-4664C5AACF8A}">
-  <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+<worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="44.140625" customWidth="1"/>
+    <col min="1" max="1" width="44.125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2">
+    <row r="1" ht="15">
       <c r="A1" t="s">
         <v>37</v>
       </c>
@@ -1223,7 +1164,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="2" spans="1:2">
+    <row r="2" ht="15">
       <c r="A2" t="s">
         <v>5</v>
       </c>
@@ -1232,19 +1173,17 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E3C081D6-A9C0-44C4-B61F-ECF5E1994215}">
-  <dimension ref="A1:E2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+<worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="26.7109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="26.75" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5">
+    <row r="1" ht="15">
       <c r="A1" t="s">
         <v>20</v>
       </c>
@@ -1261,7 +1200,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="2" spans="1:5">
+    <row r="2" ht="15">
       <c r="A2" t="s">
         <v>24</v>
       </c>
@@ -1279,21 +1218,19 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D1339B4C-E482-471A-B298-7F44E9BDAA0D}">
-  <dimension ref="A1:C2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+<worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="37.85546875" customWidth="1"/>
-    <col min="2" max="2" width="12.7109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="21.28515625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="37.875" customWidth="1"/>
+    <col min="2" max="2" width="12.75" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="21.25" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3">
+    <row r="1" ht="15">
       <c r="A1" t="s">
         <v>52</v>
       </c>
@@ -1304,7 +1241,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="2" spans="1:3">
+    <row r="2" ht="15">
       <c r="A2" t="s">
         <v>5</v>
       </c>
@@ -1316,19 +1253,17 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B902D842-DC6C-4B26-A4EA-6A91C104A4CF}">
-  <dimension ref="A1:G2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+<worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
-    <col min="4" max="4" width="10.7109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10.75" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7">
+    <row r="1" ht="15">
       <c r="A1" t="s">
         <v>37</v>
       </c>
@@ -1351,7 +1286,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="2" spans="1:7">
+    <row r="2" ht="15">
       <c r="A2" t="s">
         <v>5</v>
       </c>
@@ -1375,22 +1310,20 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8608B23C-4D98-43D6-A740-8ABC6DE5C5DD}">
-  <dimension ref="A1:D18"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+<worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="35.140625" customWidth="1"/>
+    <col min="1" max="1" width="35.125" customWidth="1"/>
     <col min="2" max="2" width="28" customWidth="1"/>
-    <col min="3" max="3" width="32.5703125" customWidth="1"/>
-    <col min="4" max="4" width="32.85546875" customWidth="1"/>
+    <col min="3" max="3" width="32.625" customWidth="1"/>
+    <col min="4" max="4" width="32.875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4">
+    <row r="1" ht="15">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1404,7 +1337,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="2" spans="1:4">
+    <row r="2" ht="15">
       <c r="A2" s="1" t="s">
         <v>5</v>
       </c>
@@ -1418,33 +1351,31 @@
         <v>12</v>
       </c>
     </row>
-    <row r="3" spans="1:4">
+    <row r="3" ht="15">
       <c r="A3" s="1"/>
       <c r="B3" s="1"/>
       <c r="C3" s="1"/>
       <c r="D3" s="1"/>
     </row>
-    <row r="16" spans="1:4">
-      <c r="C16" s="5"/>
-    </row>
-    <row r="18" spans="3:3">
-      <c r="C18" s="3"/>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+    <row r="16" ht="15">
+      <c r="C16" s="3"/>
+    </row>
+    <row r="18" ht="15">
+      <c r="C18" s="4"/>
+    </row>
+  </sheetData>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{28779ED8-A79D-4E0B-852B-088D1DC08811}">
-  <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+<worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="30.85546875" customWidth="1"/>
-    <col min="2" max="2" width="13.140625" customWidth="1"/>
+    <col min="1" max="1" width="30.875" customWidth="1"/>
+    <col min="2" max="2" width="13.125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2">
+    <row r="1" ht="15">
       <c r="A1" t="s">
         <v>17</v>
       </c>
@@ -1452,7 +1383,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="2" spans="1:2">
+    <row r="2" ht="15">
       <c r="A2" t="s">
         <v>5</v>
       </c>
@@ -1461,48 +1392,44 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C4AF5BF0-3AF2-4AD0-B35F-8942D3128B73}">
-  <dimension ref="A1:C2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1" spans="1:3">
-      <c r="A1" s="3" t="s">
+<worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetFormatPr defaultRowHeight="14.25"/>
+  <sheetData>
+    <row r="1" ht="15">
+      <c r="A1" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="B1" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="C1" s="4" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="2" spans="1:3">
-      <c r="A2" s="3" t="s">
+    <row r="2" ht="15">
+      <c r="A2" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="B2" s="3" t="s">
+      <c r="B2" s="4" t="s">
         <v>59</v>
       </c>
-      <c r="C2" s="3" t="s">
+      <c r="C2" s="4" t="s">
         <v>11</v>
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{816A20FB-0778-47B6-A652-A1B2BA52FD0E}">
-  <dimension ref="A1:F2"/>
-  <sheetFormatPr defaultColWidth="14" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1" spans="1:6">
+<worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetFormatPr defaultColWidth="14" defaultRowHeight="14.25"/>
+  <sheetData>
+    <row r="1" ht="15">
       <c r="A1" t="s">
         <v>37</v>
       </c>
@@ -1522,7 +1449,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="2" spans="1:6">
+    <row r="2" ht="15">
       <c r="A2" t="s">
         <v>5</v>
       </c>
@@ -1543,121 +1470,115 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DAEF2594-B7B7-40EF-9BFC-A865F0ACD5B2}">
-  <dimension ref="A1:F2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+<worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="1" width="39" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6">
-      <c r="A1" s="3" t="s">
+    <row r="1" ht="15">
+      <c r="A1" s="4" t="s">
         <v>37</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="B1" s="4" t="s">
         <v>38</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="C1" s="4" t="s">
         <v>39</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="D1" s="4" t="s">
         <v>60</v>
       </c>
-      <c r="E1" s="3" t="s">
+      <c r="E1" s="4" t="s">
         <v>61</v>
       </c>
-      <c r="F1" s="3" t="s">
+      <c r="F1" s="4" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="2" spans="1:6">
-      <c r="A2" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="B2" s="3" t="s">
+    <row r="2" ht="15">
+      <c r="A2" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="B2" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="C2" s="3" t="s">
+      <c r="C2" s="4" t="s">
         <v>63</v>
       </c>
-      <c r="D2" s="3" t="s">
+      <c r="D2" s="4" t="s">
         <v>63</v>
       </c>
-      <c r="E2" s="3" t="s">
+      <c r="E2" s="4" t="s">
         <v>64</v>
       </c>
-      <c r="F2" s="3" t="s">
+      <c r="F2" s="4" t="s">
         <v>63</v>
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F98E6EE4-5435-41BC-8AD6-B776B53E8FC7}">
-  <dimension ref="A1:D2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+<worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="1" width="21" customWidth="1"/>
-    <col min="2" max="2" width="17.28515625" customWidth="1"/>
-    <col min="3" max="3" width="29.42578125" customWidth="1"/>
+    <col min="2" max="2" width="17.25" customWidth="1"/>
+    <col min="3" max="3" width="29.375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4">
-      <c r="A1" s="4" t="s">
+    <row r="1" ht="15">
+      <c r="A1" s="6" t="s">
         <v>37</v>
       </c>
-      <c r="B1" s="4" t="s">
+      <c r="B1" s="6" t="s">
         <v>38</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="D1" s="4" t="s">
+      <c r="D1" s="6" t="s">
         <v>65</v>
       </c>
     </row>
-    <row r="2" spans="1:4">
-      <c r="A2" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="B2" s="4" t="s">
+    <row r="2" ht="15">
+      <c r="A2" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="B2" s="6" t="s">
         <v>6</v>
       </c>
       <c r="C2" s="1" t="s">
         <v>66</v>
       </c>
-      <c r="D2" s="4" t="s">
+      <c r="D2" s="6" t="s">
         <v>55</v>
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C29E5669-D6FB-40EE-905B-49DC274A1C27}">
-  <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1" spans="1:2">
-      <c r="A1" s="3" t="s">
+<worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetFormatPr defaultRowHeight="14.25"/>
+  <sheetData>
+    <row r="1" ht="15">
+      <c r="A1" s="4" t="s">
         <v>29</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>67</v>
       </c>
     </row>
-    <row r="2" spans="1:2">
-      <c r="A2" s="3" t="s">
+    <row r="2" ht="15">
+      <c r="A2" s="4" t="s">
         <v>19</v>
       </c>
       <c r="B2" s="1" t="s">
@@ -1665,16 +1586,14 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet26.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{62439209-6131-4BE4-BE2D-E6BCB6386DC8}">
-  <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1" spans="1:2">
+<worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetFormatPr defaultRowHeight="14.25"/>
+  <sheetData>
+    <row r="1" ht="15">
       <c r="A1" t="s">
         <v>52</v>
       </c>
@@ -1682,7 +1601,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="2" spans="1:2">
+    <row r="2" ht="15">
       <c r="A2" t="s">
         <v>5</v>
       </c>
@@ -1691,20 +1610,18 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet27.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E3AFD247-EFEB-43D1-A5E4-94260D9F042E}">
-  <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+<worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="37.140625" customWidth="1"/>
-    <col min="2" max="2" width="22.85546875" customWidth="1"/>
+    <col min="1" max="1" width="37.125" customWidth="1"/>
+    <col min="2" max="2" width="22.875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2">
+    <row r="1" ht="15">
       <c r="A1" t="s">
         <v>17</v>
       </c>
@@ -1712,7 +1629,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="2" spans="1:2">
+    <row r="2" ht="15">
       <c r="A2" t="s">
         <v>5</v>
       </c>
@@ -1721,20 +1638,18 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet28.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{49C7D945-A188-4743-BACF-F57BC8D8AB86}">
-  <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+<worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="30.28515625" customWidth="1"/>
-    <col min="2" max="2" width="18.42578125" customWidth="1"/>
+    <col min="1" max="1" width="30.25" customWidth="1"/>
+    <col min="2" max="2" width="18.375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2">
+    <row r="1" ht="15">
       <c r="A1" t="s">
         <v>17</v>
       </c>
@@ -1742,7 +1657,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="2" spans="1:2">
+    <row r="2" ht="15">
       <c r="A2" t="s">
         <v>5</v>
       </c>
@@ -1751,20 +1666,18 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet29.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0E83F4D4-5FFA-485C-BDFA-643C5CC60A7E}">
-  <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+<worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="20.140625" customWidth="1"/>
+    <col min="1" max="1" width="20.125" customWidth="1"/>
     <col min="2" max="2" width="17" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2">
+    <row r="1" ht="15">
       <c r="A1" t="s">
         <v>52</v>
       </c>
@@ -1772,7 +1685,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="2" spans="1:2">
+    <row r="2" ht="15">
       <c r="A2" t="s">
         <v>5</v>
       </c>
@@ -1781,16 +1694,14 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6191B1E8-3F90-4D43-967E-7EE476AB5B81}">
-  <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1" spans="1:2">
+<worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetFormatPr defaultRowHeight="14.25"/>
+  <sheetData>
+    <row r="1" ht="15">
       <c r="A1" t="s">
         <v>13</v>
       </c>
@@ -1798,7 +1709,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="2" spans="1:2">
+    <row r="2" ht="15">
       <c r="A2" t="s">
         <v>14</v>
       </c>
@@ -1807,19 +1718,17 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet30.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8B4C698C-6A33-4329-A05F-252C36050919}">
-  <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+<worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="28.140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="28.125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2">
+    <row r="1" ht="15">
       <c r="A1" s="1" t="s">
         <v>17</v>
       </c>
@@ -1827,7 +1736,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="2" spans="1:2">
+    <row r="2" ht="15">
       <c r="A2" s="1" t="s">
         <v>5</v>
       </c>
@@ -1836,19 +1745,17 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet31.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B5FC98DF-CF4C-4978-974B-D4FADFCADB14}">
-  <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultColWidth="16.85546875" defaultRowHeight="15"/>
+<worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetFormatPr defaultColWidth="16.875" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="28.140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="28.125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2">
+    <row r="1" ht="15">
       <c r="A1" t="s">
         <v>52</v>
       </c>
@@ -1856,7 +1763,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="2" spans="1:2">
+    <row r="2" ht="15">
       <c r="A2" t="s">
         <v>5</v>
       </c>
@@ -1865,16 +1772,14 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet32.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A839ABB3-9810-4866-9009-03B8EC041C5D}">
-  <dimension ref="A1:C2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1" spans="1:3">
+<worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetFormatPr defaultRowHeight="14.25"/>
+  <sheetData>
+    <row r="1" ht="15">
       <c r="A1" t="s">
         <v>17</v>
       </c>
@@ -1885,7 +1790,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="2" spans="1:3">
+    <row r="2" ht="15">
       <c r="A2" t="s">
         <v>5</v>
       </c>
@@ -1897,16 +1802,14 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet33.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E3263998-2B97-4B1C-A029-FD6DD8C1EF37}">
-  <dimension ref="A1:C2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1" spans="1:3">
+<worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetFormatPr defaultRowHeight="14.25"/>
+  <sheetData>
+    <row r="1" ht="15">
       <c r="A1" t="s">
         <v>17</v>
       </c>
@@ -1917,7 +1820,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="2" spans="1:3">
+    <row r="2" ht="15">
       <c r="A2" t="s">
         <v>5</v>
       </c>
@@ -1929,16 +1832,14 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet34.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E29F0755-87F3-476B-9C2A-E1FFC8CED030}">
-  <dimension ref="A1:C2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1" spans="1:3">
+<worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetFormatPr defaultRowHeight="14.25"/>
+  <sheetData>
+    <row r="1" ht="15">
       <c r="A1" t="s">
         <v>17</v>
       </c>
@@ -1949,7 +1850,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="2" spans="1:3">
+    <row r="2" ht="15">
       <c r="A2" t="s">
         <v>5</v>
       </c>
@@ -1961,16 +1862,14 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet35.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{329E8FAE-2129-4C94-87E6-C180C21CB613}">
-  <dimension ref="A1:D2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1" spans="1:4">
+<worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetFormatPr defaultRowHeight="14.25"/>
+  <sheetData>
+    <row r="1" ht="15">
       <c r="A1" t="s">
         <v>17</v>
       </c>
@@ -1984,7 +1883,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="2" spans="1:4">
+    <row r="2" ht="15">
       <c r="A2" t="s">
         <v>5</v>
       </c>
@@ -1999,16 +1898,14 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet36.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A5CE032F-302C-42A6-BC66-0FA2D092FC8A}">
-  <dimension ref="A1:D2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1" spans="1:4">
+<worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetFormatPr defaultRowHeight="14.25"/>
+  <sheetData>
+    <row r="1" ht="15">
       <c r="A1" t="s">
         <v>17</v>
       </c>
@@ -2022,7 +1919,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="2" spans="1:4">
+    <row r="2" ht="15">
       <c r="A2" t="s">
         <v>5</v>
       </c>
@@ -2037,16 +1934,14 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet37.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{74185B4F-4AE7-4DA3-9215-6ECBA7280E7B}">
-  <dimension ref="A1:C2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1" spans="1:3">
+<worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetFormatPr defaultRowHeight="14.25"/>
+  <sheetData>
+    <row r="1" ht="15">
       <c r="A1" t="s">
         <v>17</v>
       </c>
@@ -2057,7 +1952,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="2" spans="1:3">
+    <row r="2" ht="15">
       <c r="A2" t="s">
         <v>5</v>
       </c>
@@ -2069,16 +1964,14 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet38.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7D8774BA-3EC4-46E1-BB9D-1078ACED313F}">
-  <dimension ref="A1:I2"/>
-  <sheetFormatPr defaultColWidth="14" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1" spans="1:9">
+<worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetFormatPr defaultColWidth="14" defaultRowHeight="14.25"/>
+  <sheetData>
+    <row r="1" ht="15">
       <c r="A1" t="s">
         <v>17</v>
       </c>
@@ -2107,7 +2000,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="2" spans="1:9">
+    <row r="2" ht="15">
       <c r="A2" t="s">
         <v>5</v>
       </c>
@@ -2137,16 +2030,14 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet39.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A5C4203B-5A01-4381-A3CE-38EA6C51F801}">
-  <dimension ref="A1:D2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1" spans="1:4">
+<worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetFormatPr defaultRowHeight="14.25"/>
+  <sheetData>
+    <row r="1" ht="15">
       <c r="A1" t="s">
         <v>17</v>
       </c>
@@ -2160,7 +2051,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="2" spans="1:4">
+    <row r="2" ht="15">
       <c r="A2" t="s">
         <v>5</v>
       </c>
@@ -2175,39 +2066,35 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{326BFDAD-078A-4AAF-9BA5-44F9F397DA35}">
-  <dimension ref="A1:A2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+<worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="33.85546875" customWidth="1"/>
+    <col min="1" max="1" width="33.875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1">
+    <row r="1" ht="15">
       <c r="A1" s="1" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="2" spans="1:1">
-      <c r="A2" t="s">
-        <v>5</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+    <row r="2" ht="15">
+      <c r="A2" t="s">
+        <v>5</v>
+      </c>
+    </row>
+  </sheetData>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet40.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{35D5D97A-4287-4435-9AB2-0BB45EA4FBC3}">
-  <dimension ref="A1:C2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1" spans="1:3">
+<worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetFormatPr defaultRowHeight="14.25"/>
+  <sheetData>
+    <row r="1" ht="15">
       <c r="A1" t="s">
         <v>17</v>
       </c>
@@ -2218,7 +2105,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="2" spans="1:3">
+    <row r="2" ht="15">
       <c r="A2" t="s">
         <v>5</v>
       </c>
@@ -2230,16 +2117,14 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet41.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{294C6248-6B39-4869-9A5F-1A9888AB4466}">
-  <dimension ref="A1:D2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1" spans="1:4">
+<worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetFormatPr defaultRowHeight="14.25"/>
+  <sheetData>
+    <row r="1" ht="15">
       <c r="A1" t="s">
         <v>17</v>
       </c>
@@ -2253,7 +2138,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="2" spans="1:4">
+    <row r="2" ht="15">
       <c r="A2" t="s">
         <v>5</v>
       </c>
@@ -2268,19 +2153,17 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet42.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{56AA5574-913A-4A1D-9D18-82898727775C}">
-  <dimension ref="A1:C2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+<worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3">
+    <row r="1" ht="15">
       <c r="A1" t="s">
         <v>84</v>
       </c>
@@ -2291,7 +2174,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="2" spans="1:3">
+    <row r="2" ht="15">
       <c r="A2" t="s">
         <v>6</v>
       </c>
@@ -2303,16 +2186,14 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet43.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D1996804-B5A0-41DE-8EAB-89A8717FC7C7}">
-  <dimension ref="A1:C2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1" spans="1:3">
+<worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetFormatPr defaultRowHeight="14.25"/>
+  <sheetData>
+    <row r="1" ht="15">
       <c r="A1" t="s">
         <v>84</v>
       </c>
@@ -2323,7 +2204,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="2" spans="1:3">
+    <row r="2" ht="15">
       <c r="A2" t="s">
         <v>6</v>
       </c>
@@ -2335,16 +2216,14 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet44.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CEEC45CA-B3F0-4D96-A6FC-9B253BF98967}">
-  <dimension ref="A1:D2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1" spans="1:4">
+<worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetFormatPr defaultRowHeight="14.25"/>
+  <sheetData>
+    <row r="1" ht="15">
       <c r="A1" t="s">
         <v>84</v>
       </c>
@@ -2358,7 +2237,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="2" spans="1:4">
+    <row r="2" ht="15">
       <c r="A2" t="s">
         <v>6</v>
       </c>
@@ -2373,16 +2252,14 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet45.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9CEA2948-6B4B-43CF-AB32-61387B2A8875}">
-  <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1" spans="1:2">
+<worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetFormatPr defaultRowHeight="14.25"/>
+  <sheetData>
+    <row r="1" ht="15">
       <c r="A1" t="s">
         <v>84</v>
       </c>
@@ -2390,7 +2267,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="2" spans="1:2">
+    <row r="2" ht="15">
       <c r="A2" t="s">
         <v>6</v>
       </c>
@@ -2399,16 +2276,14 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet46.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{14C972A6-008E-41DF-A05C-AF5318F8FD4B}">
-  <dimension ref="A1:I2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1" spans="1:9">
+<worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetFormatPr defaultRowHeight="14.25"/>
+  <sheetData>
+    <row r="1" ht="15">
       <c r="A1" t="s">
         <v>17</v>
       </c>
@@ -2437,7 +2312,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="2" spans="1:9">
+    <row r="2" ht="15">
       <c r="A2" t="s">
         <v>5</v>
       </c>
@@ -2467,16 +2342,14 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet47.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8DC0861F-7791-458B-B1CF-76DF8B36CFCB}">
-  <dimension ref="A1:H2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1" spans="1:8">
+<worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetFormatPr defaultRowHeight="14.25"/>
+  <sheetData>
+    <row r="1" ht="15">
       <c r="A1" t="s">
         <v>17</v>
       </c>
@@ -2502,7 +2375,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="2" spans="1:8">
+    <row r="2" ht="15">
       <c r="A2" t="s">
         <v>5</v>
       </c>
@@ -2529,16 +2402,14 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet48.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{702F240E-6DDC-40E1-A471-6D34CE8EC8A9}">
-  <dimension ref="A1:C2"/>
-  <sheetFormatPr defaultColWidth="14.5703125" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1" spans="1:3">
+<worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetFormatPr defaultColWidth="14.625" defaultRowHeight="14.25"/>
+  <sheetData>
+    <row r="1" ht="15">
       <c r="A1" t="s">
         <v>17</v>
       </c>
@@ -2549,7 +2420,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="2" spans="1:3">
+    <row r="2" ht="15">
       <c r="A2" t="s">
         <v>5</v>
       </c>
@@ -2561,16 +2432,14 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet49.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1B6F8DC7-5D71-4D0F-BD39-85D8C4667F97}">
-  <dimension ref="A1:D2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1" spans="1:4">
+<worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetFormatPr defaultRowHeight="14.25"/>
+  <sheetData>
+    <row r="1" ht="15">
       <c r="A1" t="s">
         <v>17</v>
       </c>
@@ -2584,7 +2453,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="2" spans="1:4">
+    <row r="2" ht="15">
       <c r="A2" t="s">
         <v>5</v>
       </c>
@@ -2599,20 +2468,18 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3EE3B721-E210-46E8-9FE1-A1A0FFD663F0}">
-  <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+<worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="32.85546875" customWidth="1"/>
-    <col min="2" max="2" width="20.7109375" customWidth="1"/>
+    <col min="1" max="1" width="32.875" customWidth="1"/>
+    <col min="2" max="2" width="20.75" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2">
+    <row r="1" ht="15">
       <c r="A1" s="1" t="s">
         <v>17</v>
       </c>
@@ -2620,7 +2487,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="2" spans="1:2">
+    <row r="2" ht="15">
       <c r="A2" t="s">
         <v>5</v>
       </c>
@@ -2629,16 +2496,14 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet50.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B54BFBCC-7C3F-461E-8867-D0FC9227F8D2}">
-  <dimension ref="A1:E2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1" spans="1:5">
+<worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetFormatPr defaultRowHeight="14.25"/>
+  <sheetData>
+    <row r="1" ht="15">
       <c r="A1" t="s">
         <v>20</v>
       </c>
@@ -2655,7 +2520,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="2" spans="1:5">
+    <row r="2" ht="15">
       <c r="A2" t="s">
         <v>24</v>
       </c>
@@ -2673,16 +2538,14 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet51.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1B6C8D86-E59C-4B0D-9190-1A812D82FFD2}">
-  <dimension ref="A1:E2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1" spans="1:5">
+<worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetFormatPr defaultRowHeight="14.25"/>
+  <sheetData>
+    <row r="1" ht="15">
       <c r="A1" t="s">
         <v>20</v>
       </c>
@@ -2699,7 +2562,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="2" spans="1:5">
+    <row r="2" ht="15">
       <c r="A2" t="s">
         <v>24</v>
       </c>
@@ -2717,16 +2580,14 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet52.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7696B79F-033D-404F-9E1D-E22617A3BDAC}">
-  <dimension ref="A1:F2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1" spans="1:6">
+<worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetFormatPr defaultRowHeight="14.25"/>
+  <sheetData>
+    <row r="1" ht="15">
       <c r="A1" s="7" t="s">
         <v>91</v>
       </c>
@@ -2746,7 +2607,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="2" spans="1:6">
+    <row r="2" ht="15">
       <c r="A2" s="7" t="s">
         <v>94</v>
       </c>
@@ -2767,17 +2628,15 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet53.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4A192C83-0F47-4844-AB01-D5A2E984F7DB}">
-  <dimension ref="A1:G2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1" spans="1:7">
-      <c r="A1" s="6" t="s">
+<worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetFormatPr defaultRowHeight="14.25"/>
+  <sheetData>
+    <row r="1" ht="15">
+      <c r="A1" s="5" t="s">
         <v>91</v>
       </c>
       <c r="B1" s="1" t="s">
@@ -2799,8 +2658,8 @@
         <v>97</v>
       </c>
     </row>
-    <row r="2" spans="1:7">
-      <c r="A2" s="6" t="s">
+    <row r="2" ht="15">
+      <c r="A2" s="5" t="s">
         <v>94</v>
       </c>
       <c r="B2" s="1" t="s">
@@ -2823,16 +2682,14 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet54.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3011021D-4819-4690-B3D7-76A026828EC9}">
-  <dimension ref="A1:G2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1" spans="1:7">
+<worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetFormatPr defaultRowHeight="14.25"/>
+  <sheetData>
+    <row r="1" ht="15">
       <c r="A1" s="1" t="s">
         <v>100</v>
       </c>
@@ -2855,7 +2712,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="2" spans="1:7">
+    <row r="2" ht="15">
       <c r="A2" s="1" t="s">
         <v>104</v>
       </c>
@@ -2879,16 +2736,14 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet55.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{02E7FD6A-85B6-48DD-983C-2558ACC9E840}">
-  <dimension ref="A1:C2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1" spans="1:3">
+<worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetFormatPr defaultRowHeight="14.25"/>
+  <sheetData>
+    <row r="1" ht="15">
       <c r="A1" s="1" t="s">
         <v>100</v>
       </c>
@@ -2899,7 +2754,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="2" spans="1:3">
+    <row r="2" ht="15">
       <c r="A2" s="1" t="s">
         <v>104</v>
       </c>
@@ -2911,16 +2766,14 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet56.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{47958D0E-DE08-4FC8-AE6D-9F22489AEEFF}">
-  <dimension ref="A1:F2"/>
-  <sheetFormatPr defaultColWidth="18.85546875" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1" spans="1:6">
+<worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetFormatPr defaultColWidth="18.875" defaultRowHeight="14.25"/>
+  <sheetData>
+    <row r="1" ht="15">
       <c r="A1" t="s">
         <v>84</v>
       </c>
@@ -2940,7 +2793,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="2" spans="1:6">
+    <row r="2" ht="15">
       <c r="A2" t="s">
         <v>6</v>
       </c>
@@ -2961,43 +2814,39 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet57.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{42B9D63B-BC76-46EA-ADB4-8766AF6817A7}">
-  <dimension ref="A1:A2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+<worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="19.28515625" customWidth="1"/>
+    <col min="1" max="1" width="19.25" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1">
+    <row r="1" ht="15">
       <c r="A1" s="1" t="s">
         <v>111</v>
       </c>
     </row>
-    <row r="2" spans="1:1">
+    <row r="2" ht="15">
       <c r="A2" s="1" t="s">
         <v>112</v>
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet58.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{006ED08C-28C3-460C-941C-159F30186152}">
-  <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+<worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="18.5703125" customWidth="1"/>
-    <col min="2" max="2" width="18.28515625" customWidth="1"/>
+    <col min="1" max="1" width="18.625" customWidth="1"/>
+    <col min="2" max="2" width="18.25" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2">
+    <row r="1" ht="15">
       <c r="A1" t="s">
         <v>84</v>
       </c>
@@ -3005,7 +2854,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="2" spans="1:2">
+    <row r="2" ht="15">
       <c r="A2" t="s">
         <v>114</v>
       </c>
@@ -3014,16 +2863,14 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet59.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DDA25AE5-6655-45CB-9149-A8A61B5E732F}">
-  <dimension ref="A1:F2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1" spans="1:6">
+<worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetFormatPr defaultRowHeight="14.25"/>
+  <sheetData>
+    <row r="1" ht="15">
       <c r="A1" t="s">
         <v>84</v>
       </c>
@@ -3043,7 +2890,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="2" spans="1:6">
+    <row r="2" ht="15">
       <c r="A2" t="s">
         <v>6</v>
       </c>
@@ -3064,22 +2911,20 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FE237852-F036-4561-9C07-3E234A38E9FA}">
-  <dimension ref="A1:E2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+<worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="12.28515625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.7109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9.85546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="12.25" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.75" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.875" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="10" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5">
+    <row r="1" ht="15">
       <c r="A1" t="s">
         <v>20</v>
       </c>
@@ -3096,7 +2941,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="2" spans="1:5">
+    <row r="2" ht="15">
       <c r="A2" t="s">
         <v>24</v>
       </c>
@@ -3114,16 +2959,14 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet60.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C2F0C090-2891-474A-9164-D1CFD32D2A23}">
-  <dimension ref="A1:F2"/>
-  <sheetFormatPr defaultColWidth="14.7109375" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1" spans="1:6">
+<worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetFormatPr defaultColWidth="14.75" defaultRowHeight="14.25"/>
+  <sheetData>
+    <row r="1" ht="15">
       <c r="A1" t="s">
         <v>84</v>
       </c>
@@ -3143,7 +2986,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="2" spans="1:6">
+    <row r="2" ht="15">
       <c r="A2" t="s">
         <v>6</v>
       </c>
@@ -3164,16 +3007,14 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet61.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{22B1F532-E3A9-4507-B737-44BD308773F5}">
-  <dimension ref="A1:F2"/>
-  <sheetFormatPr defaultColWidth="13.85546875" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1" spans="1:6">
+<worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetFormatPr defaultColWidth="13.875" defaultRowHeight="14.25"/>
+  <sheetData>
+    <row r="1">
       <c r="A1" t="s">
         <v>84</v>
       </c>
@@ -3193,7 +3034,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="2" spans="1:6">
+    <row r="2">
       <c r="A2" t="s">
         <v>6</v>
       </c>
@@ -3214,16 +3055,14 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet62.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{545270BF-46D2-413A-9419-76683720126A}">
-  <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1" spans="1:2">
+<worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetFormatPr defaultRowHeight="14.25"/>
+  <sheetData>
+    <row r="1" ht="15">
       <c r="A1" s="1" t="s">
         <v>116</v>
       </c>
@@ -3231,7 +3070,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="2" spans="1:2">
+    <row r="2" ht="15">
       <c r="A2" s="1" t="s">
         <v>118</v>
       </c>
@@ -3240,36 +3079,32 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet63.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7A8A7719-5FC7-406C-A809-EBB81C7D304F}">
-  <dimension ref="A1:A2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1" spans="1:1">
+<worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetFormatPr defaultRowHeight="14.25"/>
+  <sheetData>
+    <row r="1" ht="15">
       <c r="A1" s="1" t="s">
         <v>116</v>
       </c>
     </row>
-    <row r="2" spans="1:1">
+    <row r="2" ht="15">
       <c r="A2" s="1" t="s">
         <v>120</v>
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet64.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4F180104-CB7F-4225-88B2-B743F65A2E71}">
-  <dimension ref="A1:E2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1" spans="1:5">
+<worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetFormatPr defaultRowHeight="14.25"/>
+  <sheetData>
+    <row r="1" ht="15">
       <c r="A1" t="s">
         <v>20</v>
       </c>
@@ -3286,7 +3121,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="2" spans="1:5">
+    <row r="2" ht="15">
       <c r="A2" t="s">
         <v>24</v>
       </c>
@@ -3304,16 +3139,14 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet65.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F12CCDE5-920D-49D0-950B-159A5A491EE7}">
-  <dimension ref="A1:G2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1" spans="1:7">
+<worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetFormatPr defaultRowHeight="14.25"/>
+  <sheetData>
+    <row r="1" ht="15">
       <c r="A1" s="1" t="s">
         <v>100</v>
       </c>
@@ -3336,7 +3169,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="2" spans="1:7">
+    <row r="2" ht="15">
       <c r="A2" s="1" t="s">
         <v>104</v>
       </c>
@@ -3360,19 +3193,17 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet66.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{57C2C09D-3106-4A2C-A972-09AF8ED3E7CC}">
-  <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultColWidth="13.85546875" defaultRowHeight="15"/>
+<worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetFormatPr defaultColWidth="13.875" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="13.85546875" customWidth="1"/>
+    <col min="1" max="1" width="13.875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2">
+    <row r="1" ht="15">
       <c r="A1" t="s">
         <v>17</v>
       </c>
@@ -3380,7 +3211,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="2" spans="1:2">
+    <row r="2" ht="15">
       <c r="A2" t="s">
         <v>5</v>
       </c>
@@ -3389,16 +3220,14 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet67.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{28C5798F-1A42-4810-A643-274C39BB5B89}">
-  <dimension ref="A1:D2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1" spans="1:4">
+<worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetFormatPr defaultRowHeight="14.25"/>
+  <sheetData>
+    <row r="1" ht="15">
       <c r="A1" s="1" t="s">
         <v>1</v>
       </c>
@@ -3408,11 +3237,11 @@
       <c r="C1" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="D1" s="6" t="s">
+      <c r="D1" s="5" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:4">
+    <row r="2" ht="15">
       <c r="A2" s="1" t="s">
         <v>49</v>
       </c>
@@ -3422,25 +3251,23 @@
       <c r="C2" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="D2" s="6" t="s">
+      <c r="D2" s="5" t="s">
         <v>49</v>
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet68.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DD547580-CDD4-4CA1-99D1-F4DBEB4DC61C}">
-  <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+<worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="1" width="16" customWidth="1"/>
-    <col min="2" max="2" width="14.5703125" customWidth="1"/>
+    <col min="2" max="2" width="14.625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2">
+    <row r="1" ht="15">
       <c r="A1" s="1" t="s">
         <v>111</v>
       </c>
@@ -3448,7 +3275,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="2" spans="1:2">
+    <row r="2" ht="15">
       <c r="A2" s="1" t="s">
         <v>112</v>
       </c>
@@ -3457,16 +3284,14 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet69.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5C851C18-BB40-4C4C-9358-B9D27BF745A2}">
-  <dimension ref="A1:C2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1" spans="1:3">
+<worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetFormatPr defaultRowHeight="14.25"/>
+  <sheetData>
+    <row r="1">
       <c r="A1" s="1" t="s">
         <v>123</v>
       </c>
@@ -3477,7 +3302,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="2" spans="1:3">
+    <row r="2">
       <c r="A2" s="1" t="s">
         <v>122</v>
       </c>
@@ -3489,19 +3314,17 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{29DDC4E0-08CB-46D1-AE6D-9F161D97ECBA}">
-  <dimension ref="A1:E2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+<worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="39.5703125" customWidth="1"/>
+    <col min="1" max="1" width="39.625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5">
+    <row r="1" ht="15">
       <c r="A1" t="s">
         <v>20</v>
       </c>
@@ -3518,7 +3341,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="2" spans="1:5">
+    <row r="2" ht="15">
       <c r="A2" t="s">
         <v>24</v>
       </c>
@@ -3536,16 +3359,14 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet70.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{30CA7E00-9554-459F-BF47-6B8E0B27B5B9}">
-  <dimension ref="A1:C2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1" spans="1:3">
+<worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetFormatPr defaultRowHeight="14.25"/>
+  <sheetData>
+    <row r="1" ht="15">
       <c r="A1" s="1" t="s">
         <v>123</v>
       </c>
@@ -3556,7 +3377,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="2" spans="1:3">
+    <row r="2" ht="15">
       <c r="A2" s="1" t="s">
         <v>122</v>
       </c>
@@ -3568,16 +3389,14 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet71.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{93B51C47-FA71-48A7-A2FD-49CB882674F9}">
-  <dimension ref="A1:C2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1" spans="1:3">
+<worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetFormatPr defaultRowHeight="14.25"/>
+  <sheetData>
+    <row r="1" ht="15">
       <c r="A1" s="1" t="s">
         <v>123</v>
       </c>
@@ -3588,7 +3407,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="2" spans="1:3">
+    <row r="2" ht="15">
       <c r="A2" s="1" t="s">
         <v>122</v>
       </c>
@@ -3600,16 +3419,14 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet72.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{485C4B2E-FC36-4946-BA8B-78C7FADE4211}">
-  <dimension ref="A1:G2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1" spans="1:7">
+<worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetFormatPr defaultRowHeight="14.25"/>
+  <sheetData>
+    <row r="1" ht="15">
       <c r="A1" s="1" t="s">
         <v>100</v>
       </c>
@@ -3632,7 +3449,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="2" spans="1:7">
+    <row r="2" ht="15">
       <c r="A2" s="1" t="s">
         <v>104</v>
       </c>
@@ -3656,16 +3473,14 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet73.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EBC66432-A9A4-4E48-A474-1F35C5F1C633}">
-  <dimension ref="A1:D2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1" spans="1:4">
+<worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetFormatPr defaultRowHeight="14.25"/>
+  <sheetData>
+    <row r="1" ht="15">
       <c r="A1" s="1" t="s">
         <v>1</v>
       </c>
@@ -3675,11 +3490,11 @@
       <c r="C1" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="D1" s="6" t="s">
+      <c r="D1" s="5" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:4">
+    <row r="2" ht="15">
       <c r="A2" s="1" t="s">
         <v>49</v>
       </c>
@@ -3689,21 +3504,19 @@
       <c r="C2" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="D2" s="6" t="s">
+      <c r="D2" s="5" t="s">
         <v>49</v>
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet74.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{849D9C7E-7FB2-4797-90F9-A5CEADA89D9C}">
-  <dimension ref="A1:F2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1" spans="1:6">
+<worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetFormatPr defaultRowHeight="14.25"/>
+  <sheetData>
+    <row r="1" ht="15">
       <c r="A1" t="s">
         <v>84</v>
       </c>
@@ -3723,7 +3536,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="2" spans="1:6">
+    <row r="2" ht="15">
       <c r="A2" t="s">
         <v>6</v>
       </c>
@@ -3744,16 +3557,14 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet75.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C4A8AAC5-4185-4C1C-93D4-1D0A64F4E1B7}">
-  <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1" spans="1:2">
+<worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetFormatPr defaultRowHeight="14.25"/>
+  <sheetData>
+    <row r="1">
       <c r="A1" s="1" t="s">
         <v>84</v>
       </c>
@@ -3761,7 +3572,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="2" spans="1:2">
+    <row r="2">
       <c r="A2" s="1" t="s">
         <v>104</v>
       </c>
@@ -3770,16 +3581,14 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet76.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9539B7F2-18EC-49F7-91A3-B0ABA5965519}">
-  <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1" spans="1:2">
+<worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetFormatPr defaultRowHeight="14.25"/>
+  <sheetData>
+    <row r="1">
       <c r="A1" s="1" t="s">
         <v>84</v>
       </c>
@@ -3787,7 +3596,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="2" spans="1:2">
+    <row r="2">
       <c r="A2" s="1" t="s">
         <v>104</v>
       </c>
@@ -3796,16 +3605,14 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet77.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{223C53EB-97BE-4EFF-B890-3A3BD91E9E72}">
-  <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1" spans="1:2">
+<worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetFormatPr defaultRowHeight="14.25"/>
+  <sheetData>
+    <row r="1">
       <c r="A1" s="1" t="s">
         <v>34</v>
       </c>
@@ -3813,7 +3620,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="2" spans="1:2">
+    <row r="2">
       <c r="A2" s="1" t="s">
         <v>5</v>
       </c>
@@ -3822,16 +3629,14 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet78.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7E2B8556-771D-4DAD-8C21-33E755A02656}">
-  <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1" spans="1:2">
+<worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetFormatPr defaultRowHeight="14.25"/>
+  <sheetData>
+    <row r="1">
       <c r="A1" s="1" t="s">
         <v>34</v>
       </c>
@@ -3839,7 +3644,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="2" spans="1:2">
+    <row r="2">
       <c r="A2" s="1" t="s">
         <v>5</v>
       </c>
@@ -3848,16 +3653,14 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet79.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A7FA2BA4-A228-45F5-B096-B0B6F3C5FCD9}">
-  <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1" spans="1:2">
+<worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetFormatPr defaultRowHeight="14.25"/>
+  <sheetData>
+    <row r="1">
       <c r="A1" s="1" t="s">
         <v>34</v>
       </c>
@@ -3865,7 +3668,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="2" spans="1:2">
+    <row r="2">
       <c r="A2" s="1" t="s">
         <v>5</v>
       </c>
@@ -3874,57 +3677,53 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8911F113-D9E9-4D95-B104-6502D772C745}">
-  <dimension ref="A1:D2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+<worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
-    <col min="2" max="2" width="22.28515625" customWidth="1"/>
+    <col min="2" max="2" width="22.25" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4">
-      <c r="A1" s="3" t="s">
+    <row r="1" ht="15">
+      <c r="A1" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="B1" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="C1" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="D1" s="4" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="2" spans="1:4">
-      <c r="A2" s="3" t="s">
+    <row r="2" ht="15">
+      <c r="A2" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="B2" s="3" t="s">
+      <c r="B2" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="C2" s="3" t="s">
+      <c r="C2" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="D2" s="3" t="s">
+      <c r="D2" s="4" t="s">
         <v>33</v>
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet80.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{763B8C95-495E-4740-BDD6-D904F75864FB}">
-  <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1" spans="1:2">
+<worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetFormatPr defaultRowHeight="14.25"/>
+  <sheetData>
+    <row r="1">
       <c r="A1" s="1" t="s">
         <v>34</v>
       </c>
@@ -3932,7 +3731,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="2" spans="1:2">
+    <row r="2">
       <c r="A2" s="1" t="s">
         <v>5</v>
       </c>
@@ -3941,24 +3740,57 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet81.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0D8151D4-D1A1-47AD-8B8F-43868BB4348D}">
-  <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1" spans="1:2">
+<worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetFormatPr defaultRowHeight="14.25"/>
+  <cols>
+    <col min="1" max="1" width="26.5" customWidth="1"/>
+    <col min="2" max="2" width="16.75" customWidth="1"/>
+    <col min="3" max="3" width="14.125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
       <c r="A1" s="1" t="s">
         <v>34</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>29</v>
       </c>
-    </row>
-    <row r="2" spans="1:2">
+      <c r="C1" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="C2" t="s">
+        <v>130</v>
+      </c>
+    </row>
+  </sheetData>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet82.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetFormatPr defaultRowHeight="14.25"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="2">
       <c r="A2" s="1" t="s">
         <v>5</v>
       </c>
@@ -3967,44 +3799,41 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{657AE5E9-3E74-406A-B22D-ED31893F34EB}">
-  <dimension ref="A1:D2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1" spans="1:4">
-      <c r="A1" s="3" t="s">
+<worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetFormatPr defaultRowHeight="14.25"/>
+  <sheetData>
+    <row r="1" ht="15">
+      <c r="A1" s="4" t="s">
         <v>34</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="B1" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="C1" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="D1" s="4" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="2" spans="1:4">
-      <c r="A2" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="B2" s="3" t="s">
+    <row r="2" ht="15">
+      <c r="A2" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="B2" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="C2" s="3" t="s">
+      <c r="C2" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="D2" s="3" t="s">
+      <c r="D2" s="4" t="s">
         <v>36</v>
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
updated requirement tab testcases and added 94,95,96 of testplan tab
</commit_message>
<xml_diff>
--- a/testData/requirementTabTestData/requirementTab_testData.xlsx
+++ b/testData/requirementTabTestData/requirementTab_testData.xlsx
@@ -1,11 +1,10 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29912"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:dbsheet="http://web.wps.cn/et/2021/dbsheet">
+  <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{72AAFBD2-10B3-4F05-B512-576B35A07306}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" firstSheet="78" activeTab="80" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView windowWidth="19200" windowHeight="6800" firstSheet="14" activeTab="19"/>
   </bookViews>
   <sheets>
     <sheet name="tc001" sheetId="1" r:id="rId1"/>
@@ -65,36 +64,37 @@
     <sheet name="tc066" sheetId="49" r:id="rId55"/>
     <sheet name="tc073" sheetId="50" r:id="rId56"/>
     <sheet name="tc074" sheetId="55" r:id="rId57"/>
-    <sheet name="tc077" sheetId="51" r:id="rId58"/>
-    <sheet name="tc086" sheetId="56" r:id="rId59"/>
-    <sheet name="tc087" sheetId="57" r:id="rId60"/>
-    <sheet name="tc088" sheetId="58" r:id="rId61"/>
-    <sheet name="tc093" sheetId="64" r:id="rId62"/>
-    <sheet name="tc094" sheetId="66" r:id="rId63"/>
-    <sheet name="tc096" sheetId="60" r:id="rId64"/>
-    <sheet name="tc097" sheetId="61" r:id="rId65"/>
-    <sheet name="tc098" sheetId="62" r:id="rId66"/>
-    <sheet name="tc099" sheetId="63" r:id="rId67"/>
-    <sheet name="tc100" sheetId="67" r:id="rId68"/>
-    <sheet name="tc102" sheetId="68" r:id="rId69"/>
-    <sheet name="tc103" sheetId="69" r:id="rId70"/>
-    <sheet name="tc104" sheetId="70" r:id="rId71"/>
-    <sheet name="tc105" sheetId="76" r:id="rId72"/>
-    <sheet name="tc106" sheetId="77" r:id="rId73"/>
-    <sheet name="tc107" sheetId="78" r:id="rId74"/>
-    <sheet name="tc110" sheetId="71" r:id="rId75"/>
-    <sheet name="tc111" sheetId="72" r:id="rId76"/>
-    <sheet name="tc129" sheetId="79" r:id="rId77"/>
-    <sheet name="tc130" sheetId="80" r:id="rId78"/>
-    <sheet name="tc131" sheetId="81" r:id="rId79"/>
-    <sheet name="tc132" sheetId="82" r:id="rId80"/>
-    <sheet name="tc133" sheetId="83" r:id="rId81"/>
+    <sheet name="tc086" sheetId="56" r:id="rId58"/>
+    <sheet name="tc087" sheetId="57" r:id="rId59"/>
+    <sheet name="tc088" sheetId="58" r:id="rId60"/>
+    <sheet name="tc093" sheetId="64" r:id="rId61"/>
+    <sheet name="tc094" sheetId="66" r:id="rId62"/>
+    <sheet name="tc096" sheetId="60" r:id="rId63"/>
+    <sheet name="tc097" sheetId="61" r:id="rId64"/>
+    <sheet name="tc098" sheetId="62" r:id="rId65"/>
+    <sheet name="tc099" sheetId="63" r:id="rId66"/>
+    <sheet name="tc100" sheetId="67" r:id="rId67"/>
+    <sheet name="tc102" sheetId="68" r:id="rId68"/>
+    <sheet name="tc103" sheetId="69" r:id="rId69"/>
+    <sheet name="tc104" sheetId="70" r:id="rId70"/>
+    <sheet name="tc105" sheetId="76" r:id="rId71"/>
+    <sheet name="tc106" sheetId="77" r:id="rId72"/>
+    <sheet name="tc107" sheetId="78" r:id="rId73"/>
+    <sheet name="tc110" sheetId="71" r:id="rId74"/>
+    <sheet name="tc111" sheetId="72" r:id="rId75"/>
+    <sheet name="tc117" sheetId="85" r:id="rId76"/>
+    <sheet name="tc118" sheetId="86" r:id="rId77"/>
+    <sheet name="tc119" sheetId="84" r:id="rId78"/>
+    <sheet name="tc129" sheetId="79" r:id="rId79"/>
+    <sheet name="tc130" sheetId="80" r:id="rId80"/>
+    <sheet name="tc131" sheetId="81" r:id="rId81"/>
+    <sheet name="tc132" sheetId="82" r:id="rId82"/>
+    <sheet name="tc133" sheetId="83" r:id="rId83"/>
+    <sheet name="tc077" sheetId="88" r:id="rId84"/>
+    <sheet name="Sheet4" sheetId="90" r:id="rId85"/>
   </sheets>
-  <calcPr calcId="191028"/>
+  <calcPr calcId="191029"/>
   <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
-      <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
         <xcalcf:feature name="microsoft.com:RD"/>
@@ -111,7 +111,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="613" uniqueCount="129">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="629" uniqueCount="131">
   <si>
     <t>Project Name</t>
   </si>
@@ -260,15 +260,15 @@
     <t>Module 22</t>
   </si>
   <si>
+    <t>Hi, changing description</t>
+  </si>
+  <si>
+    <t>Epic 13</t>
+  </si>
+  <si>
     <t>Epic - update the module</t>
   </si>
   <si>
-    <t>Hi, changing description</t>
-  </si>
-  <si>
-    <t>Epic 13</t>
-  </si>
-  <si>
     <t>MainProjectName</t>
   </si>
   <si>
@@ -452,6 +452,51 @@
     <t>module for 74</t>
   </si>
   <si>
+    <t xml:space="preserve">module name </t>
+  </si>
+  <si>
+    <t>rq title</t>
+  </si>
+  <si>
+    <t>Epic requirement</t>
+  </si>
+  <si>
+    <t>RQ testing</t>
+  </si>
+  <si>
+    <t>Module testing</t>
+  </si>
+  <si>
+    <t>SelectEpic</t>
+  </si>
+  <si>
+    <t>SET- DRIV</t>
+  </si>
+  <si>
+    <t>mdName</t>
+  </si>
+  <si>
+    <t>SetMdName</t>
+  </si>
+  <si>
+    <t>Module20</t>
+  </si>
+  <si>
+    <t>RqNAme</t>
+  </si>
+  <si>
+    <t>Requirement_testing</t>
+  </si>
+  <si>
+    <t>req</t>
+  </si>
+  <si>
+    <t>jTesting</t>
+  </si>
+  <si>
+    <t>RQ-2167</t>
+  </si>
+  <si>
     <t>setModuleName</t>
   </si>
   <si>
@@ -460,56 +505,23 @@
   <si>
     <t>Module for testing</t>
   </si>
-  <si>
-    <t xml:space="preserve">module name </t>
-  </si>
-  <si>
-    <t>rq title</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Epic requirement </t>
-  </si>
-  <si>
-    <t>RQ testing</t>
-  </si>
-  <si>
-    <t>Module testing</t>
-  </si>
-  <si>
-    <t>SelectEpic</t>
-  </si>
-  <si>
-    <t>SET- DRIV</t>
-  </si>
-  <si>
-    <t>mdName</t>
-  </si>
-  <si>
-    <t>SetMdName</t>
-  </si>
-  <si>
-    <t>Module20</t>
-  </si>
-  <si>
-    <t>RqNAme</t>
-  </si>
-  <si>
-    <t>Requirement_testing</t>
-  </si>
-  <si>
-    <t>jTesting</t>
-  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="8">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="xr9">
+  <numFmts count="4">
+    <numFmt numFmtId="176" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
+    <numFmt numFmtId="177" formatCode="_ &quot;₹&quot;* #,##0.00_ ;_ &quot;₹&quot;* \-#,##0.00_ ;_ &quot;₹&quot;* &quot;-&quot;??_ ;_ @_ "/>
+    <numFmt numFmtId="178" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
+    <numFmt numFmtId="179" formatCode="_ &quot;₹&quot;* #,##0_ ;_ &quot;₹&quot;* \-#,##0_ ;_ &quot;₹&quot;* &quot;-&quot;_ ;_ @_ "/>
+  </numFmts>
+  <fonts count="25">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
-      <family val="2"/>
+      <charset val="134"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -517,28 +529,6 @@
       <color rgb="FF000000"/>
       <name val="Aptos Narrow"/>
       <charset val="134"/>
-    </font>
-    <font>
-      <sz val="8.1999999999999993"/>
-      <color rgb="FF101828"/>
-      <name val="Arial"/>
-      <charset val="134"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF000000"/>
-      <name val="Aptos Narrow"/>
-      <charset val="1"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF000000"/>
-      <name val="Aptos Narrow"/>
-    </font>
-    <font>
-      <sz val="6.8"/>
-      <color rgb="FF6AAB73"/>
-      <name val="JetBrains Mono"/>
     </font>
     <font>
       <sz val="11"/>
@@ -549,18 +539,361 @@
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
-      <name val="Calibri"/>
+      <name val="Aptos Narrow"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="6.8"/>
+      <color rgb="FF6AAB73"/>
+      <name val="JetBrains Mono"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <sz val="8.2"/>
+      <color rgb="FF101828"/>
+      <name val="Arial"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color rgb="FF0000FF"/>
+      <name val="Aptos Narrow"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color rgb="FF800080"/>
+      <name val="Aptos Narrow"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Aptos Narrow"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="18"/>
+      <color theme="3"/>
+      <name val="Aptos Narrow"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="11"/>
+      <color rgb="FF7F7F7F"/>
+      <name val="Aptos Narrow"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="15"/>
+      <color theme="3"/>
+      <name val="Aptos Narrow"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="13"/>
+      <color theme="3"/>
+      <name val="Aptos Narrow"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="3"/>
+      <name val="Aptos Narrow"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF3F3F76"/>
+      <name val="Aptos Narrow"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF3F3F3F"/>
+      <name val="Aptos Narrow"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFA7D00"/>
+      <name val="Aptos Narrow"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Aptos Narrow"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFA7D00"/>
+      <name val="Aptos Narrow"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF006100"/>
+      <name val="Aptos Narrow"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF9C0006"/>
+      <name val="Aptos Narrow"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF9C6500"/>
+      <name val="Aptos Narrow"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="0"/>
+      <name val="Aptos Narrow"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="33">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFCC"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFCC99"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF2F2F2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFA5A5A5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC6EFCE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC7CE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFEB9C"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="9">
     <border>
       <left/>
       <right/>
@@ -568,31 +901,315 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFB2B2B2"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFB2B2B2"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFB2B2B2"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFB2B2B2"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color theme="4"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color theme="4" tint="0.499984740745262"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF7F7F7F"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF7F7F7F"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF7F7F7F"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF7F7F7F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF3F3F3F"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF3F3F3F"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF3F3F3F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="double">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right style="double">
+        <color rgb="FF3F3F3F"/>
+      </right>
+      <top style="double">
+        <color rgb="FF3F3F3F"/>
+      </top>
+      <bottom style="double">
+        <color rgb="FF3F3F3F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="double">
+        <color rgb="FFFF8001"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color theme="4"/>
+      </top>
+      <bottom style="double">
+        <color theme="4"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="176" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="177" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="178" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="3" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="4" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="4" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="5" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="49">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Comma" xfId="1" builtinId="3"/>
+    <cellStyle name="Currency" xfId="2" builtinId="4"/>
+    <cellStyle name="Percent" xfId="3" builtinId="5"/>
+    <cellStyle name="Comma [0]" xfId="4" builtinId="6"/>
+    <cellStyle name="Currency [0]" xfId="5" builtinId="7"/>
+    <cellStyle name="Link" xfId="6" builtinId="8"/>
+    <cellStyle name="Followed Hyperlink" xfId="7" builtinId="9"/>
+    <cellStyle name="Note" xfId="8" builtinId="10"/>
+    <cellStyle name="Warning Text" xfId="9" builtinId="11"/>
+    <cellStyle name="Title" xfId="10" builtinId="15"/>
+    <cellStyle name="CExplanatory Text" xfId="11" builtinId="53"/>
+    <cellStyle name="Heading 1" xfId="12" builtinId="16"/>
+    <cellStyle name="Heading 2" xfId="13" builtinId="17"/>
+    <cellStyle name="Heading 3" xfId="14" builtinId="18"/>
+    <cellStyle name="Heading 4" xfId="15" builtinId="19"/>
+    <cellStyle name="Input" xfId="16" builtinId="20"/>
+    <cellStyle name="Output" xfId="17" builtinId="21"/>
+    <cellStyle name="Calculation" xfId="18" builtinId="22"/>
+    <cellStyle name="Check Cell" xfId="19" builtinId="23"/>
+    <cellStyle name="Linked Cell" xfId="20" builtinId="24"/>
+    <cellStyle name="Total" xfId="21" builtinId="25"/>
+    <cellStyle name="Good" xfId="22" builtinId="26"/>
+    <cellStyle name="Bad" xfId="23" builtinId="27"/>
+    <cellStyle name="Neutral" xfId="24" builtinId="28"/>
+    <cellStyle name="Accent1" xfId="25" builtinId="29"/>
+    <cellStyle name="20% - Accent1" xfId="26" builtinId="30"/>
+    <cellStyle name="40% - Accent1" xfId="27" builtinId="31"/>
+    <cellStyle name="60% - Accent1" xfId="28" builtinId="32"/>
+    <cellStyle name="Accent2" xfId="29" builtinId="33"/>
+    <cellStyle name="20% - Accent2" xfId="30" builtinId="34"/>
+    <cellStyle name="40% - Accent2" xfId="31" builtinId="35"/>
+    <cellStyle name="60% - Accent2" xfId="32" builtinId="36"/>
+    <cellStyle name="Accent3" xfId="33" builtinId="37"/>
+    <cellStyle name="20% - Accent3" xfId="34" builtinId="38"/>
+    <cellStyle name="40% - Accent3" xfId="35" builtinId="39"/>
+    <cellStyle name="60% - Accent3" xfId="36" builtinId="40"/>
+    <cellStyle name="Accent4" xfId="37" builtinId="41"/>
+    <cellStyle name="20% - Accent4" xfId="38" builtinId="42"/>
+    <cellStyle name="40% - Accent4" xfId="39" builtinId="43"/>
+    <cellStyle name="60% - Accent4" xfId="40" builtinId="44"/>
+    <cellStyle name="Accent5" xfId="41" builtinId="45"/>
+    <cellStyle name="20% - Accent5" xfId="42" builtinId="46"/>
+    <cellStyle name="40% - Accent5" xfId="43" builtinId="47"/>
+    <cellStyle name="60% - Accent5" xfId="44" builtinId="48"/>
+    <cellStyle name="Accent6" xfId="45" builtinId="49"/>
+    <cellStyle name="20% - Accent6" xfId="46" builtinId="50"/>
+    <cellStyle name="40% - Accent6" xfId="47" builtinId="51"/>
+    <cellStyle name="60% - Accent6" xfId="48" builtinId="52"/>
   </cellStyles>
-  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleMedium9"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
     </ext>
   </extLst>
 </styleSheet>
@@ -641,7 +1258,7 @@
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Aptos Display" panose="020F0302020204030204"/>
+        <a:latin typeface="Aptos Display"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="游ゴシック Light"/>
@@ -674,26 +1291,9 @@
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Aptos Narrow" panose="02110004020202020204"/>
+        <a:latin typeface="Aptos Narrow"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="游ゴシック"/>
@@ -726,23 +1326,6 @@
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Office">
@@ -904,25 +1487,20 @@
       </a:style>
     </a:lnDef>
   </a:objectDefaults>
-  <a:extraClrSchemeLst/>
-  <a:extLst>
-    <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
-    </a:ext>
-  </a:extLst>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
   <dimension ref="A1:E3"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14" outlineLevelRow="2" outlineLevelCol="4"/>
   <cols>
-    <col min="1" max="1" width="30.7109375" customWidth="1"/>
-    <col min="2" max="2" width="14.140625" customWidth="1"/>
-    <col min="3" max="3" width="18.28515625" customWidth="1"/>
+    <col min="1" max="1" width="30.7083333333333" customWidth="1"/>
+    <col min="2" max="2" width="14.1333333333333" customWidth="1"/>
+    <col min="3" max="3" width="18.2833333333333" customWidth="1"/>
     <col min="4" max="4" width="16" customWidth="1"/>
-    <col min="5" max="5" width="12.28515625" customWidth="1"/>
+    <col min="5" max="5" width="12.2833333333333" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5">
@@ -955,7 +1533,7 @@
       <c r="D2" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="E2" s="2" t="s">
+      <c r="E2" s="5" t="s">
         <v>8</v>
       </c>
     </row>
@@ -972,25 +1550,27 @@
       <c r="D3" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="E3" s="2" t="s">
+      <c r="E3" s="5" t="s">
         <v>10</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5B3E68E9-6114-4137-93A6-9E3D35854EF2}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
   <dimension ref="A1:E2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14" outlineLevelRow="1" outlineLevelCol="4"/>
   <cols>
-    <col min="1" max="1" width="37.85546875" customWidth="1"/>
-    <col min="2" max="2" width="18.85546875" customWidth="1"/>
-    <col min="3" max="3" width="16.7109375" customWidth="1"/>
-    <col min="4" max="4" width="23.140625" customWidth="1"/>
-    <col min="5" max="5" width="23.7109375" customWidth="1"/>
+    <col min="1" max="1" width="37.8583333333333" customWidth="1"/>
+    <col min="2" max="2" width="18.8583333333333" customWidth="1"/>
+    <col min="3" max="3" width="16.7083333333333" customWidth="1"/>
+    <col min="4" max="4" width="23.1333333333333" customWidth="1"/>
+    <col min="5" max="5" width="23.7083333333333" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5">
@@ -1029,17 +1609,19 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{29BEAA1A-A534-4468-B9EC-E9F8BB732A2D}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
   <dimension ref="A1:C2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14" outlineLevelRow="1" outlineLevelCol="2"/>
   <cols>
-    <col min="1" max="1" width="39.5703125" customWidth="1"/>
+    <col min="1" max="1" width="39.575" customWidth="1"/>
     <col min="2" max="2" width="23" customWidth="1"/>
-    <col min="3" max="3" width="16.7109375" customWidth="1"/>
+    <col min="3" max="3" width="16.7083333333333" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
@@ -1066,16 +1648,18 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6FE5E322-70B6-4F63-AE80-0840E4095282}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
   <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14" outlineLevelRow="1" outlineLevelCol="1"/>
   <cols>
-    <col min="1" max="1" width="28.42578125" customWidth="1"/>
-    <col min="2" max="2" width="18.5703125" customWidth="1"/>
+    <col min="1" max="1" width="28.425" customWidth="1"/>
+    <col min="2" max="2" width="18.575" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2">
@@ -1096,13 +1680,15 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7C4F00CF-C1AA-4EBC-984F-C64E09298E67}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
   <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14" outlineLevelRow="1" outlineLevelCol="1"/>
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" s="3" t="s">
@@ -1122,13 +1708,15 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0C944F0C-FA76-4DBA-99AE-F54BD5BF8527}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
   <dimension ref="A1:E2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14" outlineLevelRow="1" outlineLevelCol="4"/>
   <sheetData>
     <row r="1" spans="1:5">
       <c r="A1" s="3" t="s">
@@ -1166,15 +1754,17 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0A546074-F4ED-46C4-9BFA-1A91CD65CFD3}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
   <dimension ref="A1:D2"/>
-  <sheetFormatPr defaultColWidth="15.5703125" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1" spans="1:4">
+  <sheetFormatPr defaultColWidth="15.575" defaultRowHeight="14" outlineLevelRow="1" outlineLevelCol="3"/>
+  <sheetData>
+    <row r="1" ht="14.5" spans="1:4">
       <c r="A1" s="1" t="s">
         <v>1</v>
       </c>
@@ -1184,35 +1774,37 @@
       <c r="C1" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="D1" s="6" t="s">
+      <c r="D1" s="2" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:4">
+    <row r="2" ht="14.5" spans="1:4">
       <c r="A2" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="B2" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="C2" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="C2" s="1" t="s">
+      <c r="D2" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="D2" s="6" t="s">
-        <v>49</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{710D6ACC-846B-479B-9D45-4664C5AACF8A}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
   <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14" outlineLevelRow="1" outlineLevelCol="1"/>
   <cols>
-    <col min="1" max="1" width="44.140625" customWidth="1"/>
+    <col min="1" max="1" width="44.1333333333333" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2">
@@ -1233,15 +1825,17 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E3C081D6-A9C0-44C4-B61F-ECF5E1994215}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
   <dimension ref="A1:E2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14" outlineLevelRow="1" outlineLevelCol="4"/>
   <cols>
-    <col min="1" max="1" width="26.7109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="26.7083333333333" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5">
@@ -1280,17 +1874,19 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D1339B4C-E482-471A-B298-7F44E9BDAA0D}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
   <dimension ref="A1:C2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14" outlineLevelRow="1" outlineLevelCol="2"/>
   <cols>
-    <col min="1" max="1" width="37.85546875" customWidth="1"/>
-    <col min="2" max="2" width="12.7109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="21.28515625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="37.8583333333333" customWidth="1"/>
+    <col min="2" max="2" width="12.7083333333333" customWidth="1"/>
+    <col min="3" max="3" width="21.2833333333333" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
@@ -1317,15 +1913,17 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B902D842-DC6C-4B26-A4EA-6A91C104A4CF}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
   <dimension ref="A1:G2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14" outlineLevelRow="1" outlineLevelCol="6"/>
   <cols>
-    <col min="4" max="4" width="10.7109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10.7083333333333" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7">
@@ -1376,18 +1974,20 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8608B23C-4D98-43D6-A740-8ABC6DE5C5DD}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
   <dimension ref="A1:D18"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14" outlineLevelCol="3"/>
   <cols>
-    <col min="1" max="1" width="35.140625" customWidth="1"/>
+    <col min="1" max="1" width="35.1333333333333" customWidth="1"/>
     <col min="2" max="2" width="28" customWidth="1"/>
-    <col min="3" max="3" width="32.5703125" customWidth="1"/>
-    <col min="4" max="4" width="32.85546875" customWidth="1"/>
+    <col min="3" max="3" width="32.575" customWidth="1"/>
+    <col min="4" max="4" width="32.8583333333333" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4">
@@ -1424,24 +2024,26 @@
       <c r="C3" s="1"/>
       <c r="D3" s="1"/>
     </row>
-    <row r="16" spans="1:4">
-      <c r="C16" s="5"/>
+    <row r="16" spans="3:3">
+      <c r="C16" s="4"/>
     </row>
     <row r="18" spans="3:3">
       <c r="C18" s="3"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{28779ED8-A79D-4E0B-852B-088D1DC08811}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
   <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14" outlineLevelRow="1" outlineLevelCol="1"/>
   <cols>
-    <col min="1" max="1" width="30.85546875" customWidth="1"/>
-    <col min="2" max="2" width="13.140625" customWidth="1"/>
+    <col min="1" max="1" width="30.8583333333333" customWidth="1"/>
+    <col min="2" max="2" width="13.1333333333333" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2">
@@ -1462,13 +2064,15 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C4AF5BF0-3AF2-4AD0-B35F-8942D3128B73}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
   <dimension ref="A1:C2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14" outlineLevelRow="1" outlineLevelCol="2"/>
   <sheetData>
     <row r="1" spans="1:3">
       <c r="A1" s="3" t="s">
@@ -1494,13 +2098,15 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{816A20FB-0778-47B6-A652-A1B2BA52FD0E}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
   <dimension ref="A1:F2"/>
-  <sheetFormatPr defaultColWidth="14" defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="14" defaultRowHeight="14" outlineLevelRow="1" outlineLevelCol="5"/>
   <sheetData>
     <row r="1" spans="1:6">
       <c r="A1" t="s">
@@ -1544,13 +2150,15 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DAEF2594-B7B7-40EF-9BFC-A865F0ACD5B2}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
   <dimension ref="A1:F2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14" outlineLevelRow="1" outlineLevelCol="5"/>
   <cols>
     <col min="1" max="1" width="39" customWidth="1"/>
   </cols>
@@ -1597,56 +2205,60 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F98E6EE4-5435-41BC-8AD6-B776B53E8FC7}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
   <dimension ref="A1:D2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14" outlineLevelRow="1" outlineLevelCol="3"/>
   <cols>
     <col min="1" max="1" width="21" customWidth="1"/>
-    <col min="2" max="2" width="17.28515625" customWidth="1"/>
-    <col min="3" max="3" width="29.42578125" customWidth="1"/>
+    <col min="2" max="2" width="17.2833333333333" customWidth="1"/>
+    <col min="3" max="3" width="29.425" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4">
-      <c r="A1" s="4" t="s">
+      <c r="A1" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="B1" s="4" t="s">
+      <c r="B1" s="1" t="s">
         <v>38</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="D1" s="4" t="s">
+      <c r="D1" s="1" t="s">
         <v>65</v>
       </c>
     </row>
     <row r="2" spans="1:4">
-      <c r="A2" s="4" t="s">
+      <c r="A2" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="B2" s="4" t="s">
+      <c r="B2" s="1" t="s">
         <v>6</v>
       </c>
       <c r="C2" s="1" t="s">
         <v>66</v>
       </c>
-      <c r="D2" s="4" t="s">
+      <c r="D2" s="1" t="s">
         <v>55</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C29E5669-D6FB-40EE-905B-49DC274A1C27}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
   <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14" outlineLevelRow="1" outlineLevelCol="1"/>
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" s="3" t="s">
@@ -1666,13 +2278,15 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet26.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{62439209-6131-4BE4-BE2D-E6BCB6386DC8}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
   <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14" outlineLevelRow="1" outlineLevelCol="1"/>
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" t="s">
@@ -1692,16 +2306,18 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet27.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E3AFD247-EFEB-43D1-A5E4-94260D9F042E}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
   <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14" outlineLevelRow="1" outlineLevelCol="1"/>
   <cols>
-    <col min="1" max="1" width="37.140625" customWidth="1"/>
-    <col min="2" max="2" width="22.85546875" customWidth="1"/>
+    <col min="1" max="1" width="37.1333333333333" customWidth="1"/>
+    <col min="2" max="2" width="22.8583333333333" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2">
@@ -1722,16 +2338,18 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet28.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{49C7D945-A188-4743-BACF-F57BC8D8AB86}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
   <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14" outlineLevelRow="1" outlineLevelCol="1"/>
   <cols>
-    <col min="1" max="1" width="30.28515625" customWidth="1"/>
-    <col min="2" max="2" width="18.42578125" customWidth="1"/>
+    <col min="1" max="1" width="30.2833333333333" customWidth="1"/>
+    <col min="2" max="2" width="18.425" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2">
@@ -1752,15 +2370,17 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet29.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0E83F4D4-5FFA-485C-BDFA-643C5CC60A7E}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
   <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14" outlineLevelRow="1" outlineLevelCol="1"/>
   <cols>
-    <col min="1" max="1" width="20.140625" customWidth="1"/>
+    <col min="1" max="1" width="20.1333333333333" customWidth="1"/>
     <col min="2" max="2" width="17" customWidth="1"/>
   </cols>
   <sheetData>
@@ -1782,13 +2402,15 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6191B1E8-3F90-4D43-967E-7EE476AB5B81}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
   <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14" outlineLevelRow="1" outlineLevelCol="1"/>
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" t="s">
@@ -1808,15 +2430,17 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet30.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8B4C698C-6A33-4329-A05F-252C36050919}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
   <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14" outlineLevelRow="1" outlineLevelCol="1"/>
   <cols>
-    <col min="1" max="1" width="28.140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="28.1333333333333" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2">
@@ -1837,15 +2461,17 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet31.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B5FC98DF-CF4C-4978-974B-D4FADFCADB14}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
   <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultColWidth="16.85546875" defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="16.8583333333333" defaultRowHeight="14" outlineLevelRow="1" outlineLevelCol="1"/>
   <cols>
-    <col min="1" max="1" width="28.140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="28.1333333333333" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2">
@@ -1866,13 +2492,15 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet32.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A839ABB3-9810-4866-9009-03B8EC041C5D}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
   <dimension ref="A1:C2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14" outlineLevelRow="1" outlineLevelCol="2"/>
   <sheetData>
     <row r="1" spans="1:3">
       <c r="A1" t="s">
@@ -1898,13 +2526,15 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet33.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E3263998-2B97-4B1C-A029-FD6DD8C1EF37}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
   <dimension ref="A1:C2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14" outlineLevelRow="1" outlineLevelCol="2"/>
   <sheetData>
     <row r="1" spans="1:3">
       <c r="A1" t="s">
@@ -1930,13 +2560,15 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet34.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E29F0755-87F3-476B-9C2A-E1FFC8CED030}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
   <dimension ref="A1:C2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14" outlineLevelRow="1" outlineLevelCol="2"/>
   <sheetData>
     <row r="1" spans="1:3">
       <c r="A1" t="s">
@@ -1962,13 +2594,15 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet35.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{329E8FAE-2129-4C94-87E6-C180C21CB613}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
   <dimension ref="A1:D2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14" outlineLevelRow="1" outlineLevelCol="3"/>
   <sheetData>
     <row r="1" spans="1:4">
       <c r="A1" t="s">
@@ -2000,13 +2634,15 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet36.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A5CE032F-302C-42A6-BC66-0FA2D092FC8A}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
   <dimension ref="A1:D2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14" outlineLevelRow="1" outlineLevelCol="3"/>
   <sheetData>
     <row r="1" spans="1:4">
       <c r="A1" t="s">
@@ -2038,13 +2674,15 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet37.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{74185B4F-4AE7-4DA3-9215-6ECBA7280E7B}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
   <dimension ref="A1:C2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14" outlineLevelRow="1" outlineLevelCol="2"/>
   <sheetData>
     <row r="1" spans="1:3">
       <c r="A1" t="s">
@@ -2070,13 +2708,15 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet38.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7D8774BA-3EC4-46E1-BB9D-1078ACED313F}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
   <dimension ref="A1:I2"/>
-  <sheetFormatPr defaultColWidth="14" defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="14" defaultRowHeight="14" outlineLevelRow="1"/>
   <sheetData>
     <row r="1" spans="1:9">
       <c r="A1" t="s">
@@ -2138,13 +2778,15 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet39.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A5C4203B-5A01-4381-A3CE-38EA6C51F801}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
   <dimension ref="A1:D2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14" outlineLevelRow="1" outlineLevelCol="3"/>
   <sheetData>
     <row r="1" spans="1:4">
       <c r="A1" t="s">
@@ -2176,15 +2818,17 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{326BFDAD-078A-4AAF-9BA5-44F9F397DA35}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
   <dimension ref="A1:A2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14" outlineLevelRow="1"/>
   <cols>
-    <col min="1" max="1" width="33.85546875" customWidth="1"/>
+    <col min="1" max="1" width="33.8583333333333" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:1">
@@ -2199,13 +2843,15 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet40.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{35D5D97A-4287-4435-9AB2-0BB45EA4FBC3}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
   <dimension ref="A1:C2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14" outlineLevelRow="1" outlineLevelCol="2"/>
   <sheetData>
     <row r="1" spans="1:3">
       <c r="A1" t="s">
@@ -2231,13 +2877,15 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet41.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{294C6248-6B39-4869-9A5F-1A9888AB4466}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
   <dimension ref="A1:D2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14" outlineLevelRow="1" outlineLevelCol="3"/>
   <sheetData>
     <row r="1" spans="1:4">
       <c r="A1" t="s">
@@ -2269,13 +2917,15 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet42.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{56AA5574-913A-4A1D-9D18-82898727775C}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
   <dimension ref="A1:C2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14" outlineLevelRow="1" outlineLevelCol="2"/>
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
   </cols>
@@ -2304,13 +2954,15 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet43.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D1996804-B5A0-41DE-8EAB-89A8717FC7C7}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
   <dimension ref="A1:C2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14" outlineLevelRow="1" outlineLevelCol="2"/>
   <sheetData>
     <row r="1" spans="1:3">
       <c r="A1" t="s">
@@ -2336,13 +2988,15 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet44.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CEEC45CA-B3F0-4D96-A6FC-9B253BF98967}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
   <dimension ref="A1:D2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14" outlineLevelRow="1" outlineLevelCol="3"/>
   <sheetData>
     <row r="1" spans="1:4">
       <c r="A1" t="s">
@@ -2374,13 +3028,15 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet45.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9CEA2948-6B4B-43CF-AB32-61387B2A8875}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
   <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14" outlineLevelRow="1" outlineLevelCol="1"/>
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" t="s">
@@ -2400,13 +3056,15 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet46.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{14C972A6-008E-41DF-A05C-AF5318F8FD4B}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
   <dimension ref="A1:I2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14" outlineLevelRow="1"/>
   <sheetData>
     <row r="1" spans="1:9">
       <c r="A1" t="s">
@@ -2468,13 +3126,15 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet47.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8DC0861F-7791-458B-B1CF-76DF8B36CFCB}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
   <dimension ref="A1:H2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14" outlineLevelRow="1" outlineLevelCol="7"/>
   <sheetData>
     <row r="1" spans="1:8">
       <c r="A1" t="s">
@@ -2530,13 +3190,15 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet48.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{702F240E-6DDC-40E1-A471-6D34CE8EC8A9}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
   <dimension ref="A1:C2"/>
-  <sheetFormatPr defaultColWidth="14.5703125" defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="14.575" defaultRowHeight="14" outlineLevelRow="1" outlineLevelCol="2"/>
   <sheetData>
     <row r="1" spans="1:3">
       <c r="A1" t="s">
@@ -2562,13 +3224,15 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet49.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1B6F8DC7-5D71-4D0F-BD39-85D8C4667F97}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
   <dimension ref="A1:D2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14" outlineLevelRow="1" outlineLevelCol="3"/>
   <sheetData>
     <row r="1" spans="1:4">
       <c r="A1" t="s">
@@ -2600,16 +3264,18 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3EE3B721-E210-46E8-9FE1-A1A0FFD663F0}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
   <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14" outlineLevelRow="1" outlineLevelCol="1"/>
   <cols>
-    <col min="1" max="1" width="32.85546875" customWidth="1"/>
-    <col min="2" max="2" width="20.7109375" customWidth="1"/>
+    <col min="1" max="1" width="32.8583333333333" customWidth="1"/>
+    <col min="2" max="2" width="20.7083333333333" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2">
@@ -2630,13 +3296,15 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet50.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B54BFBCC-7C3F-461E-8867-D0FC9227F8D2}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
   <dimension ref="A1:E2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14" outlineLevelRow="1" outlineLevelCol="4"/>
   <sheetData>
     <row r="1" spans="1:5">
       <c r="A1" t="s">
@@ -2674,13 +3342,15 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet51.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1B6C8D86-E59C-4B0D-9190-1A812D82FFD2}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
   <dimension ref="A1:E2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14" outlineLevelRow="1" outlineLevelCol="4"/>
   <sheetData>
     <row r="1" spans="1:5">
       <c r="A1" t="s">
@@ -2718,16 +3388,18 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet52.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7696B79F-033D-404F-9E1D-E22617A3BDAC}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
   <dimension ref="A1:F2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1" spans="1:6">
-      <c r="A1" s="7" t="s">
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14" outlineLevelRow="1" outlineLevelCol="5"/>
+  <sheetData>
+    <row r="1" ht="14.5" spans="1:6">
+      <c r="A1" s="2" t="s">
         <v>91</v>
       </c>
       <c r="B1" t="s">
@@ -2746,8 +3418,8 @@
         <v>23</v>
       </c>
     </row>
-    <row r="2" spans="1:6">
-      <c r="A2" s="7" t="s">
+    <row r="2" ht="14.5" spans="1:6">
+      <c r="A2" s="2" t="s">
         <v>94</v>
       </c>
       <c r="B2" t="s">
@@ -2768,16 +3440,18 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet53.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4A192C83-0F47-4844-AB01-D5A2E984F7DB}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
   <dimension ref="A1:G2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1" spans="1:7">
-      <c r="A1" s="6" t="s">
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14" outlineLevelRow="1" outlineLevelCol="6"/>
+  <sheetData>
+    <row r="1" ht="14.5" spans="1:7">
+      <c r="A1" s="2" t="s">
         <v>91</v>
       </c>
       <c r="B1" s="1" t="s">
@@ -2799,8 +3473,8 @@
         <v>97</v>
       </c>
     </row>
-    <row r="2" spans="1:7">
-      <c r="A2" s="6" t="s">
+    <row r="2" ht="14.5" spans="1:7">
+      <c r="A2" s="2" t="s">
         <v>94</v>
       </c>
       <c r="B2" s="1" t="s">
@@ -2824,13 +3498,15 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet54.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3011021D-4819-4690-B3D7-76A026828EC9}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
   <dimension ref="A1:G2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14" outlineLevelRow="1" outlineLevelCol="6"/>
   <sheetData>
     <row r="1" spans="1:7">
       <c r="A1" s="1" t="s">
@@ -2880,13 +3556,15 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet55.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{02E7FD6A-85B6-48DD-983C-2558ACC9E840}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
   <dimension ref="A1:C2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14" outlineLevelRow="1" outlineLevelCol="2"/>
   <sheetData>
     <row r="1" spans="1:3">
       <c r="A1" s="1" t="s">
@@ -2912,13 +3590,15 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet56.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{47958D0E-DE08-4FC8-AE6D-9F22489AEEFF}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
   <dimension ref="A1:F2"/>
-  <sheetFormatPr defaultColWidth="18.85546875" defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="18.8583333333333" defaultRowHeight="14" outlineLevelRow="1" outlineLevelCol="5"/>
   <sheetData>
     <row r="1" spans="1:6">
       <c r="A1" t="s">
@@ -2962,15 +3642,17 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet57.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{42B9D63B-BC76-46EA-ADB4-8766AF6817A7}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
   <dimension ref="A1:A2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14" outlineLevelRow="1"/>
   <cols>
-    <col min="1" max="1" width="19.28515625" customWidth="1"/>
+    <col min="1" max="1" width="19.2833333333333" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:1">
@@ -2985,996 +3667,1155 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet58.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{006ED08C-28C3-460C-941C-159F30186152}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
+  <dimension ref="A1:F2"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14" outlineLevelRow="1" outlineLevelCol="5"/>
+  <sheetData>
+    <row r="1" spans="1:6">
+      <c r="A1" t="s">
+        <v>84</v>
+      </c>
+      <c r="B1" t="s">
+        <v>108</v>
+      </c>
+      <c r="C1" t="s">
+        <v>15</v>
+      </c>
+      <c r="D1" t="s">
+        <v>21</v>
+      </c>
+      <c r="E1" t="s">
+        <v>22</v>
+      </c>
+      <c r="F1" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6">
+      <c r="A2" t="s">
+        <v>6</v>
+      </c>
+      <c r="B2" t="s">
+        <v>109</v>
+      </c>
+      <c r="C2" t="s">
+        <v>110</v>
+      </c>
+      <c r="D2" t="s">
+        <v>26</v>
+      </c>
+      <c r="E2" t="s">
+        <v>27</v>
+      </c>
+      <c r="F2" t="s">
+        <v>28</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <headerFooter/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet59.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
+  <dimension ref="A1:F2"/>
+  <sheetFormatPr defaultColWidth="14.7083333333333" defaultRowHeight="14" outlineLevelRow="1" outlineLevelCol="5"/>
+  <sheetData>
+    <row r="1" spans="1:6">
+      <c r="A1" t="s">
+        <v>84</v>
+      </c>
+      <c r="B1" t="s">
+        <v>108</v>
+      </c>
+      <c r="C1" t="s">
+        <v>15</v>
+      </c>
+      <c r="D1" t="s">
+        <v>21</v>
+      </c>
+      <c r="E1" t="s">
+        <v>22</v>
+      </c>
+      <c r="F1" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6">
+      <c r="A2" t="s">
+        <v>6</v>
+      </c>
+      <c r="B2" t="s">
+        <v>109</v>
+      </c>
+      <c r="C2" t="s">
+        <v>110</v>
+      </c>
+      <c r="D2" t="s">
+        <v>26</v>
+      </c>
+      <c r="E2" t="s">
+        <v>27</v>
+      </c>
+      <c r="F2" t="s">
+        <v>28</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <headerFooter/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
+  <dimension ref="A1:E2"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14" outlineLevelRow="1" outlineLevelCol="4"/>
+  <cols>
+    <col min="1" max="1" width="12.2833333333333" customWidth="1"/>
+    <col min="2" max="2" width="10.7083333333333" customWidth="1"/>
+    <col min="3" max="3" width="9.85833333333333" customWidth="1"/>
+    <col min="5" max="5" width="10" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5">
+      <c r="A1" t="s">
+        <v>20</v>
+      </c>
+      <c r="B1" t="s">
+        <v>15</v>
+      </c>
+      <c r="C1" t="s">
+        <v>21</v>
+      </c>
+      <c r="D1" t="s">
+        <v>22</v>
+      </c>
+      <c r="E1" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5">
+      <c r="A2" t="s">
+        <v>24</v>
+      </c>
+      <c r="B2" t="s">
+        <v>25</v>
+      </c>
+      <c r="C2" t="s">
+        <v>26</v>
+      </c>
+      <c r="D2" t="s">
+        <v>27</v>
+      </c>
+      <c r="E2" t="s">
+        <v>28</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <headerFooter/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet60.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
+  <dimension ref="A1:F2"/>
+  <sheetFormatPr defaultColWidth="13.8583333333333" defaultRowHeight="14" outlineLevelRow="1" outlineLevelCol="5"/>
+  <sheetData>
+    <row r="1" spans="1:6">
+      <c r="A1" t="s">
+        <v>84</v>
+      </c>
+      <c r="B1" t="s">
+        <v>108</v>
+      </c>
+      <c r="C1" t="s">
+        <v>15</v>
+      </c>
+      <c r="D1" t="s">
+        <v>21</v>
+      </c>
+      <c r="E1" t="s">
+        <v>22</v>
+      </c>
+      <c r="F1" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6">
+      <c r="A2" t="s">
+        <v>6</v>
+      </c>
+      <c r="B2" t="s">
+        <v>109</v>
+      </c>
+      <c r="C2" t="s">
+        <v>110</v>
+      </c>
+      <c r="D2" t="s">
+        <v>26</v>
+      </c>
+      <c r="E2" t="s">
+        <v>27</v>
+      </c>
+      <c r="F2" t="s">
+        <v>28</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <headerFooter/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet61.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
   <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14" outlineLevelRow="1" outlineLevelCol="1"/>
+  <sheetData>
+    <row r="1" spans="1:2">
+      <c r="A1" s="1" t="s">
+        <v>113</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2">
+      <c r="A2" s="1" t="s">
+        <v>115</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>116</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <headerFooter/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet62.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
+  <dimension ref="A1:A2"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14" outlineLevelRow="1"/>
+  <sheetData>
+    <row r="1" spans="1:1">
+      <c r="A1" s="1" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1">
+      <c r="A2" s="1" t="s">
+        <v>117</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <headerFooter/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet63.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
+  <dimension ref="A1:E2"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14" outlineLevelRow="1" outlineLevelCol="4"/>
+  <sheetData>
+    <row r="1" spans="1:5">
+      <c r="A1" t="s">
+        <v>20</v>
+      </c>
+      <c r="B1" t="s">
+        <v>15</v>
+      </c>
+      <c r="C1" t="s">
+        <v>21</v>
+      </c>
+      <c r="D1" t="s">
+        <v>22</v>
+      </c>
+      <c r="E1" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5">
+      <c r="A2" t="s">
+        <v>24</v>
+      </c>
+      <c r="B2" t="s">
+        <v>25</v>
+      </c>
+      <c r="C2" t="s">
+        <v>26</v>
+      </c>
+      <c r="D2" t="s">
+        <v>27</v>
+      </c>
+      <c r="E2" t="s">
+        <v>28</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <headerFooter/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet64.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
+  <dimension ref="A1:G2"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14" outlineLevelRow="1" outlineLevelCol="6"/>
+  <sheetData>
+    <row r="1" spans="1:7">
+      <c r="A1" s="1" t="s">
+        <v>100</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>101</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>102</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>103</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7">
+      <c r="A2" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>105</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="F2" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="G2" s="1" t="s">
+        <v>107</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <headerFooter/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet65.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
+  <dimension ref="A1:B2"/>
+  <sheetFormatPr defaultColWidth="13.8583333333333" defaultRowHeight="14" outlineLevelRow="1" outlineLevelCol="1"/>
   <cols>
-    <col min="1" max="1" width="18.5703125" customWidth="1"/>
-    <col min="2" max="2" width="18.28515625" customWidth="1"/>
+    <col min="1" max="1" width="13.8583333333333" customWidth="1"/>
   </cols>
+  <sheetData>
+    <row r="1" spans="1:2">
+      <c r="A1" t="s">
+        <v>17</v>
+      </c>
+      <c r="B1" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2">
+      <c r="A2" t="s">
+        <v>5</v>
+      </c>
+      <c r="B2" t="s">
+        <v>19</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <headerFooter/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet66.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
+  <dimension ref="A1:D2"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14" outlineLevelRow="1" outlineLevelCol="3"/>
+  <sheetData>
+    <row r="1" ht="14.5" spans="1:4">
+      <c r="A1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" ht="14.5" spans="1:4">
+      <c r="A2" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>51</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <headerFooter/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet67.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
+  <dimension ref="A1:B2"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14" outlineLevelRow="1" outlineLevelCol="1"/>
+  <cols>
+    <col min="1" max="1" width="16" customWidth="1"/>
+    <col min="2" max="2" width="14.575" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2">
+      <c r="A1" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="B1" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2">
+      <c r="A2" s="1" t="s">
+        <v>112</v>
+      </c>
+      <c r="B2" t="s">
+        <v>119</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <headerFooter/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet68.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
+  <dimension ref="A1:C2"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14" outlineLevelRow="1" outlineLevelCol="2"/>
+  <sheetData>
+    <row r="1" spans="1:3">
+      <c r="A1" s="1" t="s">
+        <v>120</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>121</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3">
+      <c r="A2" s="1" t="s">
+        <v>119</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>122</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>101</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <headerFooter/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet69.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
+  <dimension ref="A1:C2"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14" outlineLevelRow="1" outlineLevelCol="2"/>
+  <sheetData>
+    <row r="1" spans="1:3">
+      <c r="A1" s="1" t="s">
+        <v>120</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>121</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3">
+      <c r="A2" s="1" t="s">
+        <v>119</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>122</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>101</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <headerFooter/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
+  <dimension ref="A1:E2"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14" outlineLevelRow="1" outlineLevelCol="4"/>
+  <cols>
+    <col min="1" max="1" width="39.575" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5">
+      <c r="A1" t="s">
+        <v>20</v>
+      </c>
+      <c r="B1" t="s">
+        <v>15</v>
+      </c>
+      <c r="C1" t="s">
+        <v>21</v>
+      </c>
+      <c r="D1" t="s">
+        <v>22</v>
+      </c>
+      <c r="E1" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5">
+      <c r="A2" t="s">
+        <v>24</v>
+      </c>
+      <c r="B2" t="s">
+        <v>25</v>
+      </c>
+      <c r="C2" t="s">
+        <v>26</v>
+      </c>
+      <c r="D2" t="s">
+        <v>27</v>
+      </c>
+      <c r="E2" t="s">
+        <v>28</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <headerFooter/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet70.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
+  <dimension ref="A1:C2"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14" outlineLevelRow="1" outlineLevelCol="2"/>
+  <sheetData>
+    <row r="1" spans="1:3">
+      <c r="A1" s="1" t="s">
+        <v>120</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>121</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3">
+      <c r="A2" s="1" t="s">
+        <v>119</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>122</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>101</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <headerFooter/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet71.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
+  <dimension ref="A1:G2"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14" outlineLevelRow="1" outlineLevelCol="6"/>
+  <sheetData>
+    <row r="1" spans="1:7">
+      <c r="A1" s="1" t="s">
+        <v>100</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>101</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>102</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>103</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7">
+      <c r="A2" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>105</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="F2" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="G2" s="1" t="s">
+        <v>107</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <headerFooter/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet72.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
+  <dimension ref="A1:D2"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14" outlineLevelRow="1" outlineLevelCol="3"/>
+  <sheetData>
+    <row r="1" ht="14.5" spans="1:4">
+      <c r="A1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" ht="14.5" spans="1:4">
+      <c r="A2" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>51</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <headerFooter/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet73.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
+  <dimension ref="A1:F2"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14" outlineLevelRow="1" outlineLevelCol="5"/>
+  <sheetData>
+    <row r="1" spans="1:6">
+      <c r="A1" t="s">
+        <v>84</v>
+      </c>
+      <c r="B1" t="s">
+        <v>108</v>
+      </c>
+      <c r="C1" t="s">
+        <v>15</v>
+      </c>
+      <c r="D1" t="s">
+        <v>21</v>
+      </c>
+      <c r="E1" t="s">
+        <v>22</v>
+      </c>
+      <c r="F1" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6">
+      <c r="A2" t="s">
+        <v>6</v>
+      </c>
+      <c r="B2" t="s">
+        <v>109</v>
+      </c>
+      <c r="C2" t="s">
+        <v>110</v>
+      </c>
+      <c r="D2" t="s">
+        <v>26</v>
+      </c>
+      <c r="E2" t="s">
+        <v>27</v>
+      </c>
+      <c r="F2" t="s">
+        <v>28</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <headerFooter/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet74.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
+  <dimension ref="A1:B2"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14" outlineLevelRow="1" outlineLevelCol="1"/>
+  <sheetData>
+    <row r="1" spans="1:2">
+      <c r="A1" s="1" t="s">
+        <v>84</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2">
+      <c r="A2" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>124</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <headerFooter/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet75.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
+  <dimension ref="A1:B2"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14" outlineLevelRow="1" outlineLevelCol="1"/>
+  <sheetData>
+    <row r="1" spans="1:2">
+      <c r="A1" s="1" t="s">
+        <v>84</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2">
+      <c r="A2" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>124</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <headerFooter/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet76.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
+  <dimension ref="A1:C2"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14" outlineLevelRow="1" outlineLevelCol="2"/>
+  <sheetData>
+    <row r="1" spans="1:3">
+      <c r="A1" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3">
+      <c r="A2" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>126</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>127</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <headerFooter/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet77.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
+  <dimension ref="A1:C2"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14" outlineLevelRow="1" outlineLevelCol="2"/>
+  <sheetData>
+    <row r="1" spans="1:3">
+      <c r="A1" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3">
+      <c r="A2" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>126</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>127</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <headerFooter/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet78.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
+  <dimension ref="A1:B2"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14" outlineLevelRow="1" outlineLevelCol="1"/>
+  <sheetData>
+    <row r="1" spans="1:2">
+      <c r="A1" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2">
+      <c r="A2" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>126</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <headerFooter/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet79.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
+  <dimension ref="A1:B2"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14" outlineLevelRow="1" outlineLevelCol="1"/>
+  <sheetData>
+    <row r="1" spans="1:2">
+      <c r="A1" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2">
+      <c r="A2" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>126</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <headerFooter/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
+  <dimension ref="A1:D2"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14" outlineLevelRow="1" outlineLevelCol="3"/>
+  <cols>
+    <col min="2" max="2" width="22.2833333333333" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4">
+      <c r="A1" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4">
+      <c r="A2" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="D2" s="3" t="s">
+        <v>33</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <headerFooter/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet80.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
+  <dimension ref="A1:B2"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14" outlineLevelRow="1" outlineLevelCol="1"/>
+  <sheetData>
+    <row r="1" spans="1:2">
+      <c r="A1" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2">
+      <c r="A2" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>126</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <headerFooter/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet81.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
+  <dimension ref="A1:B2"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14" outlineLevelRow="1" outlineLevelCol="1"/>
+  <sheetData>
+    <row r="1" spans="1:2">
+      <c r="A1" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2">
+      <c r="A2" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>126</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <headerFooter/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet82.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
+  <dimension ref="A1:B2"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14" outlineLevelRow="1" outlineLevelCol="1"/>
+  <sheetData>
+    <row r="1" spans="1:2">
+      <c r="A1" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2">
+      <c r="A2" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>126</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <headerFooter/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet83.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
+  <dimension ref="A1:B2"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14" outlineLevelRow="1" outlineLevelCol="1"/>
+  <sheetData>
+    <row r="1" spans="1:2">
+      <c r="A1" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2">
+      <c r="A2" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>126</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <headerFooter/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet84.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
+  <dimension ref="A1:B2"/>
+  <sheetFormatPr defaultColWidth="8.725" defaultRowHeight="14" outlineLevelRow="1" outlineLevelCol="1"/>
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" t="s">
         <v>84</v>
       </c>
       <c r="B1" t="s">
-        <v>113</v>
+        <v>128</v>
       </c>
     </row>
     <row r="2" spans="1:2">
       <c r="A2" t="s">
-        <v>114</v>
+        <v>129</v>
       </c>
       <c r="B2" t="s">
-        <v>115</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet59.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DDA25AE5-6655-45CB-9149-A8A61B5E732F}">
-  <dimension ref="A1:F2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1" spans="1:6">
-      <c r="A1" t="s">
-        <v>84</v>
-      </c>
-      <c r="B1" t="s">
-        <v>108</v>
-      </c>
-      <c r="C1" t="s">
-        <v>15</v>
-      </c>
-      <c r="D1" t="s">
-        <v>21</v>
-      </c>
-      <c r="E1" t="s">
-        <v>22</v>
-      </c>
-      <c r="F1" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="2" spans="1:6">
-      <c r="A2" t="s">
-        <v>6</v>
-      </c>
-      <c r="B2" t="s">
-        <v>109</v>
-      </c>
-      <c r="C2" t="s">
-        <v>110</v>
-      </c>
-      <c r="D2" t="s">
-        <v>26</v>
-      </c>
-      <c r="E2" t="s">
-        <v>27</v>
-      </c>
-      <c r="F2" t="s">
-        <v>28</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FE237852-F036-4561-9C07-3E234A38E9FA}">
-  <dimension ref="A1:E2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <cols>
-    <col min="1" max="1" width="12.28515625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.7109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9.85546875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="10" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:5">
-      <c r="A1" t="s">
-        <v>20</v>
-      </c>
-      <c r="B1" t="s">
-        <v>15</v>
-      </c>
-      <c r="C1" t="s">
-        <v>21</v>
-      </c>
-      <c r="D1" t="s">
-        <v>22</v>
-      </c>
-      <c r="E1" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5">
-      <c r="A2" t="s">
-        <v>24</v>
-      </c>
-      <c r="B2" t="s">
-        <v>25</v>
-      </c>
-      <c r="C2" t="s">
-        <v>26</v>
-      </c>
-      <c r="D2" t="s">
-        <v>27</v>
-      </c>
-      <c r="E2" t="s">
-        <v>28</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet60.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C2F0C090-2891-474A-9164-D1CFD32D2A23}">
-  <dimension ref="A1:F2"/>
-  <sheetFormatPr defaultColWidth="14.7109375" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1" spans="1:6">
-      <c r="A1" t="s">
-        <v>84</v>
-      </c>
-      <c r="B1" t="s">
-        <v>108</v>
-      </c>
-      <c r="C1" t="s">
-        <v>15</v>
-      </c>
-      <c r="D1" t="s">
-        <v>21</v>
-      </c>
-      <c r="E1" t="s">
-        <v>22</v>
-      </c>
-      <c r="F1" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="2" spans="1:6">
-      <c r="A2" t="s">
-        <v>6</v>
-      </c>
-      <c r="B2" t="s">
-        <v>109</v>
-      </c>
-      <c r="C2" t="s">
-        <v>110</v>
-      </c>
-      <c r="D2" t="s">
-        <v>26</v>
-      </c>
-      <c r="E2" t="s">
-        <v>27</v>
-      </c>
-      <c r="F2" t="s">
-        <v>28</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet61.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{22B1F532-E3A9-4507-B737-44BD308773F5}">
-  <dimension ref="A1:F2"/>
-  <sheetFormatPr defaultColWidth="13.85546875" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1" spans="1:6">
-      <c r="A1" t="s">
-        <v>84</v>
-      </c>
-      <c r="B1" t="s">
-        <v>108</v>
-      </c>
-      <c r="C1" t="s">
-        <v>15</v>
-      </c>
-      <c r="D1" t="s">
-        <v>21</v>
-      </c>
-      <c r="E1" t="s">
-        <v>22</v>
-      </c>
-      <c r="F1" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="2" spans="1:6">
-      <c r="A2" t="s">
-        <v>6</v>
-      </c>
-      <c r="B2" t="s">
-        <v>109</v>
-      </c>
-      <c r="C2" t="s">
-        <v>110</v>
-      </c>
-      <c r="D2" t="s">
-        <v>26</v>
-      </c>
-      <c r="E2" t="s">
-        <v>27</v>
-      </c>
-      <c r="F2" t="s">
-        <v>28</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet62.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{545270BF-46D2-413A-9419-76683720126A}">
-  <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1" spans="1:2">
-      <c r="A1" s="1" t="s">
-        <v>116</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="2" spans="1:2">
-      <c r="A2" s="1" t="s">
-        <v>118</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>119</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet63.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7A8A7719-5FC7-406C-A809-EBB81C7D304F}">
-  <dimension ref="A1:A2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1" spans="1:1">
-      <c r="A1" s="1" t="s">
-        <v>116</v>
-      </c>
-    </row>
-    <row r="2" spans="1:1">
-      <c r="A2" s="1" t="s">
-        <v>120</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet64.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4F180104-CB7F-4225-88B2-B743F65A2E71}">
-  <dimension ref="A1:E2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1" spans="1:5">
-      <c r="A1" t="s">
-        <v>20</v>
-      </c>
-      <c r="B1" t="s">
-        <v>15</v>
-      </c>
-      <c r="C1" t="s">
-        <v>21</v>
-      </c>
-      <c r="D1" t="s">
-        <v>22</v>
-      </c>
-      <c r="E1" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5">
-      <c r="A2" t="s">
-        <v>24</v>
-      </c>
-      <c r="B2" t="s">
-        <v>25</v>
-      </c>
-      <c r="C2" t="s">
-        <v>26</v>
-      </c>
-      <c r="D2" t="s">
-        <v>27</v>
-      </c>
-      <c r="E2" t="s">
-        <v>28</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet65.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F12CCDE5-920D-49D0-950B-159A5A491EE7}">
-  <dimension ref="A1:G2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1" spans="1:7">
-      <c r="A1" s="1" t="s">
-        <v>100</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>92</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>101</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>102</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>103</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="2" spans="1:7">
-      <c r="A2" s="1" t="s">
-        <v>104</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>105</v>
-      </c>
-      <c r="C2" s="1" t="s">
-        <v>106</v>
-      </c>
-      <c r="D2" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="E2" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="F2" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="G2" s="1" t="s">
-        <v>107</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet66.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{57C2C09D-3106-4A2C-A972-09AF8ED3E7CC}">
-  <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultColWidth="13.85546875" defaultRowHeight="15"/>
-  <cols>
-    <col min="1" max="1" width="13.85546875" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:2">
-      <c r="A1" t="s">
-        <v>17</v>
-      </c>
-      <c r="B1" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="2" spans="1:2">
-      <c r="A2" t="s">
-        <v>5</v>
-      </c>
-      <c r="B2" t="s">
-        <v>19</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet67.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{28C5798F-1A42-4810-A643-274C39BB5B89}">
+        <v>130</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <headerFooter/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet85.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultColWidth="8.725" defaultRowHeight="14"/>
+  <sheetData/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <headerFooter/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
   <dimension ref="A1:D2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1" spans="1:4">
-      <c r="A1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>46</v>
-      </c>
-      <c r="D1" s="6" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4">
-      <c r="A2" s="1" t="s">
-        <v>49</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="C2" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="D2" s="6" t="s">
-        <v>49</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet68.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DD547580-CDD4-4CA1-99D1-F4DBEB4DC61C}">
-  <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <cols>
-    <col min="1" max="1" width="16" customWidth="1"/>
-    <col min="2" max="2" width="14.5703125" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:2">
-      <c r="A1" s="1" t="s">
-        <v>111</v>
-      </c>
-      <c r="B1" t="s">
-        <v>121</v>
-      </c>
-    </row>
-    <row r="2" spans="1:2">
-      <c r="A2" s="1" t="s">
-        <v>112</v>
-      </c>
-      <c r="B2" t="s">
-        <v>122</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet69.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5C851C18-BB40-4C4C-9358-B9D27BF745A2}">
-  <dimension ref="A1:C2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1" spans="1:3">
-      <c r="A1" s="1" t="s">
-        <v>123</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>124</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3">
-      <c r="A2" s="1" t="s">
-        <v>122</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>125</v>
-      </c>
-      <c r="C2" s="1" t="s">
-        <v>101</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{29DDC4E0-08CB-46D1-AE6D-9F161D97ECBA}">
-  <dimension ref="A1:E2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <cols>
-    <col min="1" max="1" width="39.5703125" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:5">
-      <c r="A1" t="s">
-        <v>20</v>
-      </c>
-      <c r="B1" t="s">
-        <v>15</v>
-      </c>
-      <c r="C1" t="s">
-        <v>21</v>
-      </c>
-      <c r="D1" t="s">
-        <v>22</v>
-      </c>
-      <c r="E1" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5">
-      <c r="A2" t="s">
-        <v>24</v>
-      </c>
-      <c r="B2" t="s">
-        <v>25</v>
-      </c>
-      <c r="C2" t="s">
-        <v>26</v>
-      </c>
-      <c r="D2" t="s">
-        <v>27</v>
-      </c>
-      <c r="E2" t="s">
-        <v>28</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet70.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{30CA7E00-9554-459F-BF47-6B8E0B27B5B9}">
-  <dimension ref="A1:C2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1" spans="1:3">
-      <c r="A1" s="1" t="s">
-        <v>123</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>124</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3">
-      <c r="A2" s="1" t="s">
-        <v>122</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>125</v>
-      </c>
-      <c r="C2" s="1" t="s">
-        <v>101</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet71.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{93B51C47-FA71-48A7-A2FD-49CB882674F9}">
-  <dimension ref="A1:C2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1" spans="1:3">
-      <c r="A1" s="1" t="s">
-        <v>123</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>124</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3">
-      <c r="A2" s="1" t="s">
-        <v>122</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>125</v>
-      </c>
-      <c r="C2" s="1" t="s">
-        <v>101</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet72.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{485C4B2E-FC36-4946-BA8B-78C7FADE4211}">
-  <dimension ref="A1:G2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1" spans="1:7">
-      <c r="A1" s="1" t="s">
-        <v>100</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>92</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>101</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>102</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>103</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="2" spans="1:7">
-      <c r="A2" s="1" t="s">
-        <v>104</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>105</v>
-      </c>
-      <c r="C2" s="1" t="s">
-        <v>106</v>
-      </c>
-      <c r="D2" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="E2" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="F2" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="G2" s="1" t="s">
-        <v>107</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet73.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EBC66432-A9A4-4E48-A474-1F35C5F1C633}">
-  <dimension ref="A1:D2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1" spans="1:4">
-      <c r="A1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>46</v>
-      </c>
-      <c r="D1" s="6" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4">
-      <c r="A2" s="1" t="s">
-        <v>49</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="C2" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="D2" s="6" t="s">
-        <v>49</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet74.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{849D9C7E-7FB2-4797-90F9-A5CEADA89D9C}">
-  <dimension ref="A1:F2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1" spans="1:6">
-      <c r="A1" t="s">
-        <v>84</v>
-      </c>
-      <c r="B1" t="s">
-        <v>108</v>
-      </c>
-      <c r="C1" t="s">
-        <v>15</v>
-      </c>
-      <c r="D1" t="s">
-        <v>21</v>
-      </c>
-      <c r="E1" t="s">
-        <v>22</v>
-      </c>
-      <c r="F1" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="2" spans="1:6">
-      <c r="A2" t="s">
-        <v>6</v>
-      </c>
-      <c r="B2" t="s">
-        <v>109</v>
-      </c>
-      <c r="C2" t="s">
-        <v>110</v>
-      </c>
-      <c r="D2" t="s">
-        <v>26</v>
-      </c>
-      <c r="E2" t="s">
-        <v>27</v>
-      </c>
-      <c r="F2" t="s">
-        <v>28</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet75.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C4A8AAC5-4185-4C1C-93D4-1D0A64F4E1B7}">
-  <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1" spans="1:2">
-      <c r="A1" s="1" t="s">
-        <v>84</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>126</v>
-      </c>
-    </row>
-    <row r="2" spans="1:2">
-      <c r="A2" s="1" t="s">
-        <v>104</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>127</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet76.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9539B7F2-18EC-49F7-91A3-B0ABA5965519}">
-  <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1" spans="1:2">
-      <c r="A1" s="1" t="s">
-        <v>84</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>126</v>
-      </c>
-    </row>
-    <row r="2" spans="1:2">
-      <c r="A2" s="1" t="s">
-        <v>104</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>127</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet77.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{223C53EB-97BE-4EFF-B890-3A3BD91E9E72}">
-  <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1" spans="1:2">
-      <c r="A1" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="2" spans="1:2">
-      <c r="A2" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>128</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet78.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7E2B8556-771D-4DAD-8C21-33E755A02656}">
-  <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1" spans="1:2">
-      <c r="A1" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="2" spans="1:2">
-      <c r="A2" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>128</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet79.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A7FA2BA4-A228-45F5-B096-B0B6F3C5FCD9}">
-  <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1" spans="1:2">
-      <c r="A1" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="2" spans="1:2">
-      <c r="A2" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>128</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8911F113-D9E9-4D95-B104-6502D772C745}">
-  <dimension ref="A1:D2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <cols>
-    <col min="2" max="2" width="22.28515625" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:4">
-      <c r="A1" s="3" t="s">
-        <v>29</v>
-      </c>
-      <c r="B1" s="3" t="s">
-        <v>30</v>
-      </c>
-      <c r="C1" s="3" t="s">
-        <v>31</v>
-      </c>
-      <c r="D1" s="3" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4">
-      <c r="A2" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="B2" s="3" t="s">
-        <v>32</v>
-      </c>
-      <c r="C2" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="D2" s="3" t="s">
-        <v>33</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet80.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{763B8C95-495E-4740-BDD6-D904F75864FB}">
-  <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1" spans="1:2">
-      <c r="A1" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="2" spans="1:2">
-      <c r="A2" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>128</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet81.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0D8151D4-D1A1-47AD-8B8F-43868BB4348D}">
-  <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1" spans="1:2">
-      <c r="A1" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="2" spans="1:2">
-      <c r="A2" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>128</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{657AE5E9-3E74-406A-B22D-ED31893F34EB}">
-  <dimension ref="A1:D2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14" outlineLevelRow="1" outlineLevelCol="3"/>
   <sheetData>
     <row r="1" spans="1:4">
       <c r="A1" s="3" t="s">
@@ -4006,5 +4847,6 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <headerFooter/>
 </worksheet>
 </file>
</xml_diff>